<commit_message>
Adiciona capacidade NIRE 2 adultos + 2 criancas (reforma)
- Nova aba "BUDGET NIRE 2+2" no template (clonada da CHAITEN 2+2,
  mesma estrutura de formulas, so troca a referencia de cabana)
- Nova coluna Y na BUDGET RESUMO com todas as formulas de agregacao
  (subtotal, taxa agencia, taxa CC, valor por pessoa)
- RESULTADO atualizado para somar a coluna Y nas 8 categorias
- CABIN_MAP: NIRE (2,2) -> coluna Y
- _hide_inactive_budget_cols e flags de ativacao ampliados para incluir Y
- Label do app atualizado: "NIRE (ate 2 adultos + 2 criancas)"
- Testado: geracao isolada de NIRE 2+2 bate com a formula de calibracao
  (fator 0.95) usada nas outras cabanas; regressao com as 4 cabanas
  simultaneas confirma que nada quebrou
</commit_message>
<xml_diff>
--- a/assets/templates/planilha_orcamentos_python.xlsx
+++ b/assets/templates/planilha_orcamentos_python.xlsx
@@ -23,6 +23,7 @@
     <sheet name="BUDGET NIRE 1" sheetId="8" r:id="rId8"/>
     <sheet name="BUDGET NIRE 2" sheetId="9" r:id="rId9"/>
     <sheet name="BUDGET NIRE 2+1" sheetId="10" r:id="rId10"/>
+    <sheet name="BUDGET NIRE 2+2" sheetId="27" r:id="rId31"/>
     <sheet name="BUDGET CHAITEN 1" sheetId="11" r:id="rId11"/>
     <sheet name="BUDGET CHAITEN 2" sheetId="12" r:id="rId12"/>
     <sheet name="BUDGET CHAITEN 2+1" sheetId="13" r:id="rId13"/>
@@ -51277,10 +51278,2620 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+  <sheetPr codeName="Sheet11"/>
+  <dimension ref="A1:P101"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="48.796875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="23.796875" style="52" customWidth="1"/>
+    <col min="3" max="3" width="24" style="7" customWidth="1"/>
+    <col min="4" max="4" width="22.796875" style="12" customWidth="1"/>
+    <col min="5" max="5" width="22.19921875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="31.19921875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="27.796875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="32.3984375" style="7" customWidth="1"/>
+    <col min="9" max="9" width="23.59765625" style="7" customWidth="1"/>
+    <col min="10" max="10" width="25.19921875" style="7" customWidth="1"/>
+    <col min="11" max="11" width="28.796875" style="7" customWidth="1"/>
+    <col min="12" max="12" width="36.19921875" style="7" customWidth="1"/>
+    <col min="13" max="28" width="11" style="7" customWidth="1"/>
+    <col min="29" max="16384" width="11" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="22" hidden="1" customHeight="1" thickBot="1"/>
+    <row r="2" spans="1:16" ht="7" customHeight="1">
+      <c r="D2" s="13"/>
+    </row>
+    <row r="3" spans="1:16" s="10" customFormat="1" ht="1" customHeight="1">
+      <c r="A3" s="14"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:16" s="10" customFormat="1" ht="19" customHeight="1">
+      <c r="A4" s="14"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5" spans="1:16" s="10" customFormat="1" ht="46" customHeight="1">
+      <c r="A5" s="54" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" s="674">
+        <v>2</v>
+      </c>
+      <c r="C5" s="675"/>
+      <c r="D5" s="277"/>
+      <c r="E5" s="277" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="278"/>
+      <c r="G5" s="9"/>
+    </row>
+    <row r="6" spans="1:16" s="8" customFormat="1" ht="37" customHeight="1">
+      <c r="A6" s="54" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="683">
+        <v>2</v>
+      </c>
+      <c r="C6" s="684"/>
+      <c r="D6" s="682" t="s">
+        <v>131</v>
+      </c>
+      <c r="E6" s="661"/>
+      <c r="F6" s="106">
+        <f>D21</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="9"/>
+      <c r="H6" s="10"/>
+    </row>
+    <row r="7" spans="1:16" s="8" customFormat="1" ht="33" customHeight="1">
+      <c r="A7" s="55" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" s="662">
+        <f>CALENDAR!C2</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="661"/>
+      <c r="D7" s="660" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="661"/>
+      <c r="F7" s="107">
+        <f>SUM(F12:F20)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="9"/>
+      <c r="H7" s="10"/>
+    </row>
+    <row r="8" spans="1:16" s="8" customFormat="1" ht="31" customHeight="1">
+      <c r="A8" s="54" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="680">
+        <f>CALENDAR!C3</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="661"/>
+      <c r="D8" s="681" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" s="661"/>
+      <c r="F8" s="108">
+        <f>F6-F7</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="9"/>
+      <c r="H8" s="10"/>
+    </row>
+    <row r="9" spans="1:16" s="8" customFormat="1" ht="32" customHeight="1">
+      <c r="A9" s="55" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="678">
+        <f>CALENDAR!J2</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="661"/>
+      <c r="D9" s="679" t="s">
+        <v>137</v>
+      </c>
+      <c r="E9" s="661"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="10"/>
+    </row>
+    <row r="10" spans="1:16" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A10" s="16"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+    </row>
+    <row r="11" spans="1:16" s="6" customFormat="1" ht="44" customHeight="1" thickBot="1">
+      <c r="A11" s="671" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="677" t="s">
+        <v>139</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>140</v>
+      </c>
+      <c r="D11" s="677" t="s">
+        <v>141</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="738" t="str">
+        <f>E5</f>
+        <v>CHAITEN</v>
+      </c>
+      <c r="G11" s="664"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="658" t="s">
+        <v>142</v>
+      </c>
+      <c r="J11" s="659"/>
+      <c r="K11" s="659"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+    </row>
+    <row r="12" spans="1:16" s="6" customFormat="1" ht="32" customHeight="1">
+      <c r="A12" s="659"/>
+      <c r="B12" s="659"/>
+      <c r="C12" s="58">
+        <v>0.05</v>
+      </c>
+      <c r="D12" s="659"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="665"/>
+      <c r="G12" s="666"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="J12" s="60" t="s">
+        <v>143</v>
+      </c>
+      <c r="K12" s="60" t="s">
+        <v>144</v>
+      </c>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+    </row>
+    <row r="13" spans="1:16" ht="22" customHeight="1" thickBot="1">
+      <c r="A13" s="61" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="109">
+        <f>G28</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="109">
+        <f t="shared" ref="C13:C20" si="0">B13*$C$12</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="109">
+        <f t="shared" ref="D13:D20" si="1">B13+(B13*$C$12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="667"/>
+      <c r="G13" s="668"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="5"/>
+    </row>
+    <row r="14" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A14" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="110">
+        <f>J49</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="110">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D14" s="110">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="271" t="str">
+        <f t="shared" ref="F14:F19" si="2">A14</f>
+        <v>2.FOOD</v>
+      </c>
+      <c r="G14" s="261">
+        <f>G49</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="7"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+    </row>
+    <row r="15" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A15" s="63" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="111">
+        <f>E59</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="111">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D15" s="111">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="7"/>
+      <c r="F15" s="272" t="str">
+        <f t="shared" si="2"/>
+        <v>3.DRINKS</v>
+      </c>
+      <c r="G15" s="262">
+        <f>G59</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="7"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+    </row>
+    <row r="16" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A16" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="112">
+        <f>$E$72</f>
+        <v>0</v>
+      </c>
+      <c r="C16" s="112">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D16" s="112">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E16" s="7"/>
+      <c r="F16" s="273" t="str">
+        <f t="shared" si="2"/>
+        <v>4. ACTIVITIES</v>
+      </c>
+      <c r="G16" s="263">
+        <f>G72</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="7"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+    </row>
+    <row r="17" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A17" s="63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="111">
+        <f>$E$80</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="111">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D17" s="111">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="7"/>
+      <c r="F17" s="274" t="str">
+        <f t="shared" si="2"/>
+        <v>5.TRANSPORT</v>
+      </c>
+      <c r="G17" s="174">
+        <f>G80</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="7"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+    </row>
+    <row r="18" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A18" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="113">
+        <f>$E$86</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="113">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D18" s="113">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="F18" s="275" t="str">
+        <f t="shared" si="2"/>
+        <v>6.EXPERIENCES</v>
+      </c>
+      <c r="G18" s="264">
+        <f>G86</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="7"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+    </row>
+    <row r="19" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A19" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="114">
+        <f>$E$95</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="114">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D19" s="114">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E19" s="7"/>
+      <c r="F19" s="276" t="str">
+        <f t="shared" si="2"/>
+        <v>7.EXTRAS</v>
+      </c>
+      <c r="G19" s="151">
+        <f>G95</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="7"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+    </row>
+    <row r="20" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1" thickBot="1">
+      <c r="A20" s="66" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="115">
+        <f>$E$99</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="115">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D20" s="115">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="7"/>
+      <c r="F20" s="676" t="s">
+        <v>145</v>
+      </c>
+      <c r="G20" s="669">
+        <f>G14+G15+G16+G17+G18+G19</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="7"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+    </row>
+    <row r="21" spans="1:16" ht="35" customHeight="1" thickBot="1">
+      <c r="A21" s="67" t="s">
+        <v>146</v>
+      </c>
+      <c r="B21" s="116">
+        <f>SUM(B13:B20)</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="116"/>
+      <c r="D21" s="116">
+        <f>SUM(D13:D20)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="51"/>
+      <c r="F21" s="670"/>
+      <c r="G21" s="670"/>
+    </row>
+    <row r="22" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A22" s="16"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+    </row>
+    <row r="23" spans="1:16" ht="44" customHeight="1" thickBot="1">
+      <c r="A23" s="68" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="69" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="69" t="s">
+        <v>147</v>
+      </c>
+      <c r="D23" s="69" t="s">
+        <v>148</v>
+      </c>
+      <c r="E23" s="70" t="s">
+        <v>149</v>
+      </c>
+      <c r="F23" s="70" t="s">
+        <v>150</v>
+      </c>
+      <c r="G23" s="70" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="20" customHeight="1">
+      <c r="A24" s="71" t="s">
+        <v>166</v>
+      </c>
+      <c r="B24" s="93">
+        <v>0</v>
+      </c>
+      <c r="C24" s="117">
+        <f>288190.9</f>
+        <v>288190.90000000002</v>
+      </c>
+      <c r="D24" s="118"/>
+      <c r="E24" s="119">
+        <f>(C24+D24)*$B$9*B24</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="119">
+        <f>E24-(E24*F24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="20" customHeight="1">
+      <c r="A25" s="71" t="s">
+        <v>167</v>
+      </c>
+      <c r="B25" s="93">
+        <v>1</v>
+      </c>
+      <c r="C25" s="117">
+        <f>288190.9</f>
+        <v>288190.90000000002</v>
+      </c>
+      <c r="D25" s="118">
+        <f>$B$6*50000</f>
+        <v>100000</v>
+      </c>
+      <c r="E25" s="119">
+        <f>(C25+D25)*$B$9*B25</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0</v>
+      </c>
+      <c r="G25" s="119">
+        <f>E25-(E25*F25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="20" customHeight="1">
+      <c r="A26" s="71" t="s">
+        <v>168</v>
+      </c>
+      <c r="B26" s="93">
+        <v>0</v>
+      </c>
+      <c r="C26" s="117">
+        <f>259371.81</f>
+        <v>259371.81</v>
+      </c>
+      <c r="D26" s="118"/>
+      <c r="E26" s="119">
+        <f>(C26+D26)*$B$9*B26</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="119">
+        <f>E26-(E26*F26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A27" s="71" t="s">
+        <v>169</v>
+      </c>
+      <c r="B27" s="93">
+        <v>0</v>
+      </c>
+      <c r="C27" s="117">
+        <f>259371.81</f>
+        <v>259371.81</v>
+      </c>
+      <c r="D27" s="118">
+        <v>50000</v>
+      </c>
+      <c r="E27" s="119">
+        <f>(C27+D27)*$B$9*B27</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0</v>
+      </c>
+      <c r="G27" s="119">
+        <f>E27-(E27*F27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="29" customHeight="1" thickBot="1">
+      <c r="A28" s="672" t="s">
+        <v>156</v>
+      </c>
+      <c r="B28" s="673"/>
+      <c r="C28" s="673"/>
+      <c r="D28" s="673"/>
+      <c r="E28" s="72"/>
+      <c r="F28" s="73"/>
+      <c r="G28" s="120">
+        <f>SUM(G24:G27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A29" s="16"/>
+      <c r="B29" s="56"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="7"/>
+      <c r="P29" s="7"/>
+    </row>
+    <row r="30" spans="1:16" s="10" customFormat="1" ht="40" customHeight="1" thickBot="1">
+      <c r="A30" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="159" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="160" t="s">
+        <v>53</v>
+      </c>
+      <c r="D30" s="153" t="s">
+        <v>54</v>
+      </c>
+      <c r="E30" s="149" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" s="103" t="s">
+        <v>158</v>
+      </c>
+      <c r="G30" s="147" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A31" s="154" t="str">
+        <f>'BASE PAX'!A6</f>
+        <v>BREAKFAST</v>
+      </c>
+      <c r="B31" s="284">
+        <f>(B5*B9*'BASE PAX'!G6)+('BASE PAX'!H6*B6*B9)</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="121"/>
+      <c r="D31" s="144"/>
+      <c r="E31" s="283"/>
+      <c r="F31" s="122">
+        <f t="shared" ref="F31:F46" si="3">B31*C31</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="325">
+        <f>0.2*B31</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="351" t="str">
+        <f>'BASE PAX'!A6</f>
+        <v>BREAKFAST</v>
+      </c>
+      <c r="I31" s="357">
+        <f>B31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="20" customHeight="1">
+      <c r="A32" s="155" t="str">
+        <f>'BASE PAX'!A7</f>
+        <v>LUNCH 1</v>
+      </c>
+      <c r="B32" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B7</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="123">
+        <f>'BASE PAX'!C7</f>
+        <v>40000</v>
+      </c>
+      <c r="D32" s="125">
+        <f>'BASE PAX'!D7</f>
+        <v>48000</v>
+      </c>
+      <c r="E32" s="151">
+        <f t="shared" ref="E32:E46" si="4">D32*B32</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G32" s="146">
+        <f t="shared" ref="G32:G46" si="5">E32-F32</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="292"/>
+      <c r="I32" s="295"/>
+    </row>
+    <row r="33" spans="1:11" ht="20" customHeight="1">
+      <c r="A33" s="155" t="str">
+        <f>'BASE PAX'!A8</f>
+        <v>LUNCH 2</v>
+      </c>
+      <c r="B33" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B8</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="123">
+        <f>'BASE PAX'!C8</f>
+        <v>40000</v>
+      </c>
+      <c r="D33" s="125">
+        <f>'BASE PAX'!D8</f>
+        <v>48000</v>
+      </c>
+      <c r="E33" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F33" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G33" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H33" s="292"/>
+      <c r="I33" s="295"/>
+    </row>
+    <row r="34" spans="1:11" ht="20" customHeight="1">
+      <c r="A34" s="155" t="str">
+        <f>'BASE PAX'!A9</f>
+        <v>LUNCH 3</v>
+      </c>
+      <c r="B34" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B9</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="123">
+        <f>'BASE PAX'!C9</f>
+        <v>40000</v>
+      </c>
+      <c r="D34" s="125">
+        <f>'BASE PAX'!D9</f>
+        <v>48000</v>
+      </c>
+      <c r="E34" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F34" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G34" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H34" s="292"/>
+      <c r="I34" s="295"/>
+    </row>
+    <row r="35" spans="1:11" ht="20" customHeight="1">
+      <c r="A35" s="155" t="str">
+        <f>'BASE PAX'!A10</f>
+        <v>LUNCH 4</v>
+      </c>
+      <c r="B35" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B10</f>
+        <v>0</v>
+      </c>
+      <c r="C35" s="123">
+        <f>'BASE PAX'!C10</f>
+        <v>45000</v>
+      </c>
+      <c r="D35" s="125">
+        <f>'BASE PAX'!D10</f>
+        <v>54000</v>
+      </c>
+      <c r="E35" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F35" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G35" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H35" s="292"/>
+      <c r="I35" s="295"/>
+    </row>
+    <row r="36" spans="1:11" ht="20" customHeight="1">
+      <c r="A36" s="155" t="str">
+        <f>'BASE PAX'!A11</f>
+        <v>LUNCH 5</v>
+      </c>
+      <c r="B36" s="91">
+        <f>($B$5+($B$6*0.6))*'BASE PAX'!B11</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="123">
+        <f>'BASE PAX'!C11</f>
+        <v>50000</v>
+      </c>
+      <c r="D36" s="125">
+        <f>'BASE PAX'!D11</f>
+        <v>60000</v>
+      </c>
+      <c r="E36" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F36" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G36" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H36" s="292"/>
+      <c r="I36" s="295"/>
+    </row>
+    <row r="37" spans="1:11" ht="20" customHeight="1">
+      <c r="A37" s="155" t="str">
+        <f>'BASE PAX'!A12</f>
+        <v>LUNCH 6</v>
+      </c>
+      <c r="B37" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B12</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="123">
+        <f>'BASE PAX'!C12</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="125">
+        <f>'BASE PAX'!D12</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F37" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G37" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H37" s="292"/>
+      <c r="I37" s="295"/>
+    </row>
+    <row r="38" spans="1:11" ht="20" customHeight="1">
+      <c r="A38" s="155" t="str">
+        <f>'BASE PAX'!A13</f>
+        <v>LUNCH 7</v>
+      </c>
+      <c r="B38" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B13</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="123">
+        <f>'BASE PAX'!C13</f>
+        <v>5000</v>
+      </c>
+      <c r="D38" s="125">
+        <f>'BASE PAX'!D13</f>
+        <v>6000</v>
+      </c>
+      <c r="E38" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H38" s="292"/>
+      <c r="I38" s="295"/>
+    </row>
+    <row r="39" spans="1:11" ht="20" customHeight="1">
+      <c r="A39" s="156" t="str">
+        <f>'BASE PAX'!A14</f>
+        <v>SNACKS</v>
+      </c>
+      <c r="B39" s="92">
+        <f>($B$5+$B$6)*'BASE PAX'!B14</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="125">
+        <f>'BASE PAX'!C14</f>
+        <v>8000</v>
+      </c>
+      <c r="D39" s="145">
+        <f>'BASE PAX'!D14</f>
+        <v>9600</v>
+      </c>
+      <c r="E39" s="150">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F39" s="122">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G39" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H39" s="292"/>
+      <c r="I39" s="295"/>
+    </row>
+    <row r="40" spans="1:11" ht="20" customHeight="1">
+      <c r="A40" s="155" t="str">
+        <f>'BASE PAX'!A15</f>
+        <v>DINNER 1</v>
+      </c>
+      <c r="B40" s="91">
+        <f>($B$5+($B$6*0.6))*'BASE PAX'!B15</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="123">
+        <f>'BASE PAX'!C15</f>
+        <v>70000</v>
+      </c>
+      <c r="D40" s="125">
+        <f>'BASE PAX'!D15</f>
+        <v>84000</v>
+      </c>
+      <c r="E40" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F40" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G40" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H40" s="292"/>
+      <c r="I40" s="295"/>
+    </row>
+    <row r="41" spans="1:11" ht="20" customHeight="1">
+      <c r="A41" s="155" t="str">
+        <f>'BASE PAX'!A16</f>
+        <v>DINNER 2</v>
+      </c>
+      <c r="B41" s="91">
+        <f>($B$5+($B$6*0.6))*'BASE PAX'!B16</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="123">
+        <f>'BASE PAX'!C16</f>
+        <v>25000</v>
+      </c>
+      <c r="D41" s="125">
+        <f>'BASE PAX'!D16</f>
+        <v>30000</v>
+      </c>
+      <c r="E41" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F41" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G41" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H41" s="292"/>
+      <c r="I41" s="295"/>
+    </row>
+    <row r="42" spans="1:11" ht="20" customHeight="1">
+      <c r="A42" s="155" t="str">
+        <f>'BASE PAX'!A17</f>
+        <v>DINNER 3</v>
+      </c>
+      <c r="B42" s="91">
+        <f>($B$5+($B$6*0.6))*'BASE PAX'!B17</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="123">
+        <f>'BASE PAX'!C17</f>
+        <v>50000</v>
+      </c>
+      <c r="D42" s="125">
+        <f>'BASE PAX'!D17</f>
+        <v>60000</v>
+      </c>
+      <c r="E42" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F42" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G42" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H42" s="292"/>
+      <c r="I42" s="295"/>
+    </row>
+    <row r="43" spans="1:11" ht="20" customHeight="1">
+      <c r="A43" s="155" t="str">
+        <f>'BASE PAX'!A18</f>
+        <v>DINNER 4</v>
+      </c>
+      <c r="B43" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B18</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="123">
+        <f>'BASE PAX'!C18</f>
+        <v>65000</v>
+      </c>
+      <c r="D43" s="125">
+        <f>'BASE PAX'!D18</f>
+        <v>78000</v>
+      </c>
+      <c r="E43" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F43" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G43" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H43" s="292"/>
+      <c r="I43" s="295"/>
+    </row>
+    <row r="44" spans="1:11" ht="20" customHeight="1">
+      <c r="A44" s="155" t="str">
+        <f>'BASE PAX'!A19</f>
+        <v>DINNER 5</v>
+      </c>
+      <c r="B44" s="91">
+        <f>($B$5+($B$6*0.6))*'BASE PAX'!B19</f>
+        <v>0</v>
+      </c>
+      <c r="C44" s="123">
+        <f>'BASE PAX'!C19</f>
+        <v>75000</v>
+      </c>
+      <c r="D44" s="125">
+        <f>'BASE PAX'!D19</f>
+        <v>90000</v>
+      </c>
+      <c r="E44" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F44" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G44" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H44" s="292"/>
+      <c r="I44" s="295"/>
+    </row>
+    <row r="45" spans="1:11" ht="20" customHeight="1">
+      <c r="A45" s="155" t="str">
+        <f>'BASE PAX'!A20</f>
+        <v>DINNER 6</v>
+      </c>
+      <c r="B45" s="91">
+        <f>($B$5+($B$6*0.5))*'BASE PAX'!B20</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="123">
+        <f>'BASE PAX'!C20</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="125">
+        <f>'BASE PAX'!D20</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F45" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G45" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H45" s="292"/>
+      <c r="I45" s="295"/>
+    </row>
+    <row r="46" spans="1:11" ht="20" customHeight="1" thickBot="1">
+      <c r="A46" s="155" t="str">
+        <f>'BASE PAX'!A21</f>
+        <v>DINNER 7</v>
+      </c>
+      <c r="B46" s="91">
+        <f>($B$5+($B$6*0.6))*'BASE PAX'!B21</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="123">
+        <f>'BASE PAX'!C21</f>
+        <v>75000</v>
+      </c>
+      <c r="D46" s="125">
+        <f>'BASE PAX'!D21</f>
+        <v>90000</v>
+      </c>
+      <c r="E46" s="151">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="124">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G46" s="146">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="292"/>
+      <c r="I46" s="295"/>
+    </row>
+    <row r="47" spans="1:11" ht="20" customHeight="1">
+      <c r="A47" s="155" t="str">
+        <f>'BASE PAX'!A22</f>
+        <v>QUANT. TOTAL | PADRAO ALMOÇO</v>
+      </c>
+      <c r="B47" s="91">
+        <f>'BASE PAX'!B22</f>
+        <v>0</v>
+      </c>
+      <c r="C47" s="123"/>
+      <c r="D47" s="125"/>
+      <c r="E47" s="151"/>
+      <c r="F47" s="124"/>
+      <c r="G47" s="325">
+        <f>0.2*I47</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="337" t="str">
+        <f>'BASE PAX'!A22</f>
+        <v>QUANT. TOTAL | PADRAO ALMOÇO</v>
+      </c>
+      <c r="I47" s="350">
+        <f>(B5*B47*'BASE PAX'!G22)+(B6*B47*'BASE PAX'!H22)</f>
+        <v>0</v>
+      </c>
+      <c r="J47" s="328"/>
+      <c r="K47" s="329"/>
+    </row>
+    <row r="48" spans="1:11" ht="20" customHeight="1" thickBot="1">
+      <c r="A48" s="163" t="str">
+        <f>'BASE PAX'!A23</f>
+        <v>QUANT. TOTAL | PADRAO JANTAR</v>
+      </c>
+      <c r="B48" s="171">
+        <f>'BASE PAX'!B23</f>
+        <v>0</v>
+      </c>
+      <c r="C48" s="165"/>
+      <c r="D48" s="166"/>
+      <c r="E48" s="167"/>
+      <c r="F48" s="168"/>
+      <c r="G48" s="326">
+        <f>0.2*I48</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="346" t="str">
+        <f>'BASE PAX'!A23</f>
+        <v>QUANT. TOTAL | PADRAO JANTAR</v>
+      </c>
+      <c r="I48" s="336">
+        <f>(B5*B48*'BASE PAX'!G23)+(B6*B48*'BASE PAX'!H23)</f>
+        <v>0</v>
+      </c>
+      <c r="J48" s="330"/>
+      <c r="K48" s="331"/>
+    </row>
+    <row r="49" spans="1:16" ht="29" customHeight="1" thickBot="1">
+      <c r="A49" s="161" t="s">
+        <v>72</v>
+      </c>
+      <c r="B49" s="157"/>
+      <c r="C49" s="158"/>
+      <c r="D49" s="152"/>
+      <c r="E49" s="300">
+        <f>SUM(E31:E48)</f>
+        <v>0</v>
+      </c>
+      <c r="F49" s="104">
+        <f>SUM(F31:F48)</f>
+        <v>0</v>
+      </c>
+      <c r="G49" s="327">
+        <f>SUM(G31:G48)</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="339" t="s">
+        <v>55</v>
+      </c>
+      <c r="I49" s="343">
+        <f>I31+I47+I48</f>
+        <v>0</v>
+      </c>
+      <c r="J49" s="361">
+        <f>I49+E49</f>
+        <v>0</v>
+      </c>
+      <c r="K49" s="345" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A50" s="16"/>
+      <c r="B50" s="56"/>
+      <c r="C50" s="105"/>
+      <c r="D50" s="102"/>
+      <c r="E50" s="102"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="17"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="295"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
+    </row>
+    <row r="51" spans="1:16" ht="34" customHeight="1" thickBot="1">
+      <c r="A51" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="B51" s="207" t="s">
+        <v>52</v>
+      </c>
+      <c r="C51" s="208" t="s">
+        <v>53</v>
+      </c>
+      <c r="D51" s="209" t="s">
+        <v>54</v>
+      </c>
+      <c r="E51" s="172" t="s">
+        <v>55</v>
+      </c>
+      <c r="F51" s="142" t="s">
+        <v>158</v>
+      </c>
+      <c r="G51" s="182" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" ht="20" customHeight="1">
+      <c r="A52" s="76" t="str">
+        <f>'BASE PAX'!A27</f>
+        <v>SUCOS</v>
+      </c>
+      <c r="B52" s="205">
+        <f>'BASE PAX'!B27</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="193">
+        <f>'BASE PAX'!C27</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="206">
+        <f t="shared" ref="D52:D58" si="6">(C52*0.2)+C52</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="174">
+        <f t="shared" ref="E52:E58" si="7">D52*B52</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="173">
+        <f t="shared" ref="F52:F58" si="8">B52*C52</f>
+        <v>0</v>
+      </c>
+      <c r="G52" s="183">
+        <f t="shared" ref="G52:G59" si="9">E52-F52</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" ht="20" customHeight="1">
+      <c r="A53" s="76" t="str">
+        <f>'BASE PAX'!A28</f>
+        <v>SUCOS</v>
+      </c>
+      <c r="B53" s="205">
+        <f>'BASE PAX'!B28</f>
+        <v>0</v>
+      </c>
+      <c r="C53" s="175">
+        <f>'BASE PAX'!C28</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="176">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E53" s="174">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F53" s="173">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G53" s="183">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="20" customHeight="1">
+      <c r="A54" s="87" t="str">
+        <f>'BASE PAX'!A29</f>
+        <v>CERVEJAS</v>
+      </c>
+      <c r="B54" s="205">
+        <f>'BASE PAX'!B29</f>
+        <v>0</v>
+      </c>
+      <c r="C54" s="175">
+        <f>'BASE PAX'!C29</f>
+        <v>2000</v>
+      </c>
+      <c r="D54" s="176">
+        <f t="shared" si="6"/>
+        <v>2400</v>
+      </c>
+      <c r="E54" s="174">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F54" s="173">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G54" s="183">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" ht="20" customHeight="1">
+      <c r="A55" s="87" t="str">
+        <f>'BASE PAX'!A30</f>
+        <v>VINHOS</v>
+      </c>
+      <c r="B55" s="205">
+        <f>'BASE PAX'!B30</f>
+        <v>0</v>
+      </c>
+      <c r="C55" s="175">
+        <f>'BASE PAX'!C30</f>
+        <v>8000</v>
+      </c>
+      <c r="D55" s="176">
+        <f t="shared" si="6"/>
+        <v>9600</v>
+      </c>
+      <c r="E55" s="174">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F55" s="173">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G55" s="183">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="20" customHeight="1">
+      <c r="A56" s="87" t="str">
+        <f>'BASE PAX'!A31</f>
+        <v>DRINKS</v>
+      </c>
+      <c r="B56" s="205">
+        <f>'BASE PAX'!B31</f>
+        <v>0</v>
+      </c>
+      <c r="C56" s="175">
+        <f>'BASE PAX'!C31</f>
+        <v>15000</v>
+      </c>
+      <c r="D56" s="176">
+        <f t="shared" si="6"/>
+        <v>18000</v>
+      </c>
+      <c r="E56" s="174">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F56" s="173">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G56" s="183">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="20" customHeight="1">
+      <c r="A57" s="87" t="str">
+        <f>'BASE PAX'!A32</f>
+        <v>COOLER</v>
+      </c>
+      <c r="B57" s="205">
+        <f>'BASE PAX'!B32</f>
+        <v>0</v>
+      </c>
+      <c r="C57" s="175">
+        <f>'BASE PAX'!C32</f>
+        <v>5000</v>
+      </c>
+      <c r="D57" s="176">
+        <f t="shared" si="6"/>
+        <v>6000</v>
+      </c>
+      <c r="E57" s="174">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F57" s="173">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G57" s="183">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A58" s="180">
+        <f>'BASE PAX'!A33</f>
+        <v>0</v>
+      </c>
+      <c r="B58" s="205">
+        <f>'BASE PAX'!B33</f>
+        <v>0</v>
+      </c>
+      <c r="C58" s="178">
+        <f>'BASE PAX'!C33</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="179">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E58" s="184">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F58" s="185">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G58" s="186">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" ht="48" customHeight="1" thickBot="1">
+      <c r="A59" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B59" s="77"/>
+      <c r="C59" s="126"/>
+      <c r="D59" s="181"/>
+      <c r="E59" s="127">
+        <f>SUM(E52:E58)</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="188">
+        <f>SUM(F52:F58)</f>
+        <v>0</v>
+      </c>
+      <c r="G59" s="189">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A60" s="16"/>
+      <c r="B60" s="56"/>
+      <c r="C60" s="105"/>
+      <c r="D60" s="102"/>
+      <c r="E60" s="102"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="17"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+      <c r="J60" s="7"/>
+      <c r="K60" s="7"/>
+      <c r="L60" s="7"/>
+      <c r="M60" s="7"/>
+      <c r="N60" s="7"/>
+      <c r="O60" s="7"/>
+      <c r="P60" s="7"/>
+    </row>
+    <row r="61" spans="1:16" s="10" customFormat="1" ht="42" customHeight="1" thickBot="1">
+      <c r="A61" s="226" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61" s="227" t="s">
+        <v>52</v>
+      </c>
+      <c r="C61" s="228" t="s">
+        <v>53</v>
+      </c>
+      <c r="D61" s="229" t="s">
+        <v>54</v>
+      </c>
+      <c r="E61" s="229" t="s">
+        <v>55</v>
+      </c>
+      <c r="F61" s="228" t="s">
+        <v>158</v>
+      </c>
+      <c r="G61" s="230" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" ht="20" customHeight="1">
+      <c r="A62" s="223" t="str">
+        <f>'BASE PAX'!A37</f>
+        <v>HOTTUBE</v>
+      </c>
+      <c r="B62" s="224">
+        <f>'BASE PAX'!B37</f>
+        <v>0</v>
+      </c>
+      <c r="C62" s="195">
+        <f>'BASE PAX'!C37</f>
+        <v>12000</v>
+      </c>
+      <c r="D62" s="225">
+        <f t="shared" ref="D62:D71" si="10">C62*0.2+C62</f>
+        <v>14400</v>
+      </c>
+      <c r="E62" s="225">
+        <f t="shared" ref="E62:E71" si="11">D62*B62</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="195">
+        <f t="shared" ref="F62:F72" si="12">B62*C62</f>
+        <v>0</v>
+      </c>
+      <c r="G62" s="194">
+        <f t="shared" ref="G62:G72" si="13">E62-F62</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" ht="20" customHeight="1">
+      <c r="A63" s="219" t="str">
+        <f>'BASE PAX'!A38</f>
+        <v>TREKKING 1/2 DAY</v>
+      </c>
+      <c r="B63" s="224">
+        <f>'BASE PAX'!B38</f>
+        <v>0</v>
+      </c>
+      <c r="C63" s="196">
+        <f>'BASE PAX'!C38</f>
+        <v>60000</v>
+      </c>
+      <c r="D63" s="220">
+        <f t="shared" si="10"/>
+        <v>72000</v>
+      </c>
+      <c r="E63" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F63" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G63" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" ht="20" customHeight="1">
+      <c r="A64" s="219" t="str">
+        <f>'BASE PAX'!A39</f>
+        <v>TREKKING FUK DAY</v>
+      </c>
+      <c r="B64" s="224">
+        <f>'BASE PAX'!B39</f>
+        <v>0</v>
+      </c>
+      <c r="C64" s="196">
+        <f>'BASE PAX'!C39</f>
+        <v>90000</v>
+      </c>
+      <c r="D64" s="220">
+        <f t="shared" si="10"/>
+        <v>108000</v>
+      </c>
+      <c r="E64" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F64" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G64" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" ht="20" customHeight="1">
+      <c r="A65" s="219" t="str">
+        <f>'BASE PAX'!A40</f>
+        <v>FLOTADA FAMILIAR</v>
+      </c>
+      <c r="B65" s="224">
+        <f>'BASE PAX'!B40</f>
+        <v>0</v>
+      </c>
+      <c r="C65" s="196">
+        <f>'BASE PAX'!C40</f>
+        <v>60000</v>
+      </c>
+      <c r="D65" s="220">
+        <f t="shared" si="10"/>
+        <v>72000</v>
+      </c>
+      <c r="E65" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F65" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G65" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" ht="20" customHeight="1">
+      <c r="A66" s="219" t="str">
+        <f>'BASE PAX'!A41</f>
+        <v>RAFTING 1/2 DAY</v>
+      </c>
+      <c r="B66" s="224">
+        <f>'BASE PAX'!B41</f>
+        <v>0</v>
+      </c>
+      <c r="C66" s="196">
+        <f>'BASE PAX'!C41</f>
+        <v>75000</v>
+      </c>
+      <c r="D66" s="220">
+        <f t="shared" si="10"/>
+        <v>90000</v>
+      </c>
+      <c r="E66" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F66" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G66" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" ht="20" customHeight="1">
+      <c r="A67" s="219" t="str">
+        <f>'BASE PAX'!A42</f>
+        <v>RAFTING FULL DAY</v>
+      </c>
+      <c r="B67" s="224">
+        <f>'BASE PAX'!B42</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="196">
+        <f>'BASE PAX'!C42</f>
+        <v>110000</v>
+      </c>
+      <c r="D67" s="220">
+        <f t="shared" si="10"/>
+        <v>132000</v>
+      </c>
+      <c r="E67" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F67" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G67" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" ht="20" customHeight="1">
+      <c r="A68" s="219" t="str">
+        <f>'BASE PAX'!A43</f>
+        <v>CABALGADA 1/2 DAy</v>
+      </c>
+      <c r="B68" s="224">
+        <f>'BASE PAX'!B43</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="196">
+        <f>'BASE PAX'!C43</f>
+        <v>90000</v>
+      </c>
+      <c r="D68" s="220">
+        <f t="shared" si="10"/>
+        <v>108000</v>
+      </c>
+      <c r="E68" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F68" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G68" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" ht="20" customHeight="1">
+      <c r="A69" s="219" t="str">
+        <f>'BASE PAX'!A44</f>
+        <v>CABALGADA FULL DAY</v>
+      </c>
+      <c r="B69" s="224">
+        <f>'BASE PAX'!B44</f>
+        <v>0</v>
+      </c>
+      <c r="C69" s="196">
+        <f>'BASE PAX'!C44</f>
+        <v>140000</v>
+      </c>
+      <c r="D69" s="220">
+        <f t="shared" si="10"/>
+        <v>168000</v>
+      </c>
+      <c r="E69" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F69" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G69" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" ht="20" customHeight="1">
+      <c r="A70" s="219" t="str">
+        <f>'BASE PAX'!A45</f>
+        <v>LANCHA YELCHO</v>
+      </c>
+      <c r="B70" s="224">
+        <f>'BASE PAX'!B45</f>
+        <v>0</v>
+      </c>
+      <c r="C70" s="196">
+        <f>'BASE PAX'!C45</f>
+        <v>120000</v>
+      </c>
+      <c r="D70" s="220">
+        <f t="shared" si="10"/>
+        <v>144000</v>
+      </c>
+      <c r="E70" s="220">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F70" s="196">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G70" s="190">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A71" s="221" t="str">
+        <f>'BASE PAX'!A46</f>
+        <v>RECREACAO INFANTIL 3HS</v>
+      </c>
+      <c r="B71" s="224">
+        <f>'BASE PAX'!B46</f>
+        <v>0</v>
+      </c>
+      <c r="C71" s="197">
+        <f>'BASE PAX'!C46</f>
+        <v>30000</v>
+      </c>
+      <c r="D71" s="220">
+        <f t="shared" si="10"/>
+        <v>36000</v>
+      </c>
+      <c r="E71" s="222">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F71" s="197">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G71" s="192">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" ht="48" customHeight="1" thickBot="1">
+      <c r="A72" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="B72" s="79"/>
+      <c r="C72" s="128"/>
+      <c r="D72" s="128"/>
+      <c r="E72" s="198">
+        <f>SUM(E62:E71)</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="204">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G72" s="203">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" ht="37" customHeight="1" thickBot="1"/>
+    <row r="74" spans="1:16" s="8" customFormat="1" ht="36" customHeight="1" thickBot="1">
+      <c r="A74" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B74" s="214" t="s">
+        <v>52</v>
+      </c>
+      <c r="C74" s="215" t="s">
+        <v>53</v>
+      </c>
+      <c r="D74" s="153" t="s">
+        <v>54</v>
+      </c>
+      <c r="E74" s="153" t="s">
+        <v>55</v>
+      </c>
+      <c r="F74" s="143" t="s">
+        <v>162</v>
+      </c>
+      <c r="G74" s="147" t="s">
+        <v>159</v>
+      </c>
+      <c r="H74" s="7"/>
+      <c r="I74" s="7"/>
+      <c r="J74" s="7"/>
+      <c r="K74" s="7"/>
+      <c r="L74" s="7"/>
+      <c r="M74" s="7"/>
+      <c r="N74" s="7"/>
+      <c r="O74" s="7"/>
+      <c r="P74" s="7"/>
+    </row>
+    <row r="75" spans="1:16" ht="20" customHeight="1">
+      <c r="A75" s="88" t="str">
+        <f>'BASE PAX'!A50</f>
+        <v>TRANSFER AEROPORTO CHEGADA</v>
+      </c>
+      <c r="B75" s="211">
+        <f>'BASE PAX'!B50</f>
+        <v>0</v>
+      </c>
+      <c r="C75" s="213">
+        <v>50000</v>
+      </c>
+      <c r="D75" s="231">
+        <f>C75*0.2+C75</f>
+        <v>60000</v>
+      </c>
+      <c r="E75" s="231">
+        <f>D75*B75</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="210">
+        <f>B75*C75</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="199">
+        <f t="shared" ref="G75:G80" si="14">E75-F75</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" ht="20" customHeight="1">
+      <c r="A76" s="88" t="str">
+        <f>'BASE PAX'!A51</f>
+        <v>TRANSFER AEROPORTO PARTIDA</v>
+      </c>
+      <c r="B76" s="211">
+        <f>'BASE PAX'!B51</f>
+        <v>0</v>
+      </c>
+      <c r="C76" s="212">
+        <f>'BASE PAX'!C51</f>
+        <v>80000</v>
+      </c>
+      <c r="D76" s="232">
+        <f>C76*0.2+C76</f>
+        <v>96000</v>
+      </c>
+      <c r="E76" s="232">
+        <f>D76*B76</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="210">
+        <f>B76*C76</f>
+        <v>0</v>
+      </c>
+      <c r="G76" s="200">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" ht="20" customHeight="1">
+      <c r="A77" s="88" t="str">
+        <f>'BASE PAX'!A52</f>
+        <v>TRANSFERS INTERNO</v>
+      </c>
+      <c r="B77" s="211">
+        <f>'BASE PAX'!B52</f>
+        <v>0</v>
+      </c>
+      <c r="C77" s="212">
+        <f>'BASE PAX'!C52</f>
+        <v>18000</v>
+      </c>
+      <c r="D77" s="232">
+        <f>C77*0.2+C77</f>
+        <v>21600</v>
+      </c>
+      <c r="E77" s="232">
+        <f>D77*B77</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="210">
+        <f>B77*C77</f>
+        <v>0</v>
+      </c>
+      <c r="G77" s="200">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" ht="20" customHeight="1">
+      <c r="A78" s="88" t="str">
+        <f>'BASE PAX'!A53</f>
+        <v>EXTRAS 1</v>
+      </c>
+      <c r="B78" s="211">
+        <f>'BASE PAX'!B53</f>
+        <v>0</v>
+      </c>
+      <c r="C78" s="212">
+        <f>'BASE PAX'!C53</f>
+        <v>150000</v>
+      </c>
+      <c r="D78" s="232">
+        <f>C78*0.2+C78</f>
+        <v>180000</v>
+      </c>
+      <c r="E78" s="232">
+        <f>D78*B78</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="210">
+        <f>B78*C78</f>
+        <v>0</v>
+      </c>
+      <c r="G78" s="200">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A79" s="218" t="str">
+        <f>'BASE PAX'!A54</f>
+        <v>EXTRAS 2</v>
+      </c>
+      <c r="B79" s="211">
+        <f>'BASE PAX'!B54</f>
+        <v>0</v>
+      </c>
+      <c r="C79" s="216">
+        <f>'BASE PAX'!C54</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="233">
+        <f>C79*0.2+C79</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="233">
+        <f>D79*B79</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="217">
+        <f>B79*C79</f>
+        <v>0</v>
+      </c>
+      <c r="G79" s="201">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" ht="44" customHeight="1" thickBot="1">
+      <c r="A80" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B80" s="80"/>
+      <c r="C80" s="130"/>
+      <c r="D80" s="130"/>
+      <c r="E80" s="131">
+        <f>SUM(E75:E79)</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="131">
+        <f>SUM(F75:F79)</f>
+        <v>0</v>
+      </c>
+      <c r="G80" s="203">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A81" s="16"/>
+      <c r="B81" s="56"/>
+      <c r="C81" s="105"/>
+      <c r="D81" s="102"/>
+      <c r="E81" s="102"/>
+      <c r="F81" s="7"/>
+      <c r="G81" s="17"/>
+      <c r="H81" s="7"/>
+      <c r="I81" s="7"/>
+      <c r="J81" s="7"/>
+      <c r="K81" s="7"/>
+      <c r="L81" s="7"/>
+      <c r="M81" s="7"/>
+      <c r="N81" s="7"/>
+      <c r="O81" s="7"/>
+      <c r="P81" s="7"/>
+    </row>
+    <row r="82" spans="1:16" s="9" customFormat="1" ht="42" customHeight="1" thickBot="1">
+      <c r="A82" s="246" t="s">
+        <v>117</v>
+      </c>
+      <c r="B82" s="247" t="s">
+        <v>52</v>
+      </c>
+      <c r="C82" s="248" t="s">
+        <v>53</v>
+      </c>
+      <c r="D82" s="249" t="s">
+        <v>54</v>
+      </c>
+      <c r="E82" s="249" t="s">
+        <v>55</v>
+      </c>
+      <c r="F82" s="248" t="s">
+        <v>162</v>
+      </c>
+      <c r="G82" s="147" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" ht="20" customHeight="1">
+      <c r="A83" s="81" t="str">
+        <f>'BASE PAX'!A58</f>
+        <v>WS INSTRUCTOR</v>
+      </c>
+      <c r="B83" s="238">
+        <f>'BASE PAX'!B58</f>
+        <v>0</v>
+      </c>
+      <c r="C83" s="239">
+        <f>'BASE PAX'!C58</f>
+        <v>3415000</v>
+      </c>
+      <c r="D83" s="240">
+        <f>(C83*0.15)+C83</f>
+        <v>3927250</v>
+      </c>
+      <c r="E83" s="240">
+        <f>D83*B83</f>
+        <v>0</v>
+      </c>
+      <c r="F83" s="234">
+        <f>B83*C83</f>
+        <v>0</v>
+      </c>
+      <c r="G83" s="199">
+        <f>E83-F83</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" ht="20" customHeight="1">
+      <c r="A84" s="81" t="str">
+        <f>'BASE PAX'!A59</f>
+        <v>PRODUCER FEE</v>
+      </c>
+      <c r="B84" s="235">
+        <f>'BASE PAX'!B59</f>
+        <v>0</v>
+      </c>
+      <c r="C84" s="236">
+        <f>'BASE PAX'!C59</f>
+        <v>180000</v>
+      </c>
+      <c r="D84" s="237">
+        <f>(C84*0.15)+C84</f>
+        <v>207000</v>
+      </c>
+      <c r="E84" s="237">
+        <f>D84*B84</f>
+        <v>0</v>
+      </c>
+      <c r="F84" s="234">
+        <f>B84*C84</f>
+        <v>0</v>
+      </c>
+      <c r="G84" s="200">
+        <f>E84-F84</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A85" s="241">
+        <f>'BASE PAX'!A60</f>
+        <v>0</v>
+      </c>
+      <c r="B85" s="242">
+        <f>'BASE PAX'!B60</f>
+        <v>0</v>
+      </c>
+      <c r="C85" s="243">
+        <f>'BASE PAX'!C60</f>
+        <v>20000</v>
+      </c>
+      <c r="D85" s="244">
+        <f>(C85*0.15)+C85</f>
+        <v>23000</v>
+      </c>
+      <c r="E85" s="244">
+        <f>D85*B85</f>
+        <v>0</v>
+      </c>
+      <c r="F85" s="245">
+        <f>B85*C85</f>
+        <v>0</v>
+      </c>
+      <c r="G85" s="201">
+        <f>E85-F85</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" ht="41" customHeight="1" thickBot="1">
+      <c r="A86" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="B86" s="82"/>
+      <c r="C86" s="132"/>
+      <c r="D86" s="132"/>
+      <c r="E86" s="133">
+        <f>SUM(E83:E85)</f>
+        <v>0</v>
+      </c>
+      <c r="F86" s="133">
+        <f>SUM(F81:F85)</f>
+        <v>0</v>
+      </c>
+      <c r="G86" s="203">
+        <f>E86-F86</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A87" s="16"/>
+      <c r="B87" s="56"/>
+      <c r="C87" s="105"/>
+      <c r="D87" s="102"/>
+      <c r="E87" s="102"/>
+      <c r="F87" s="7"/>
+      <c r="G87" s="17"/>
+      <c r="H87" s="7"/>
+      <c r="I87" s="7"/>
+      <c r="J87" s="7"/>
+      <c r="K87" s="7"/>
+      <c r="L87" s="7"/>
+      <c r="M87" s="7"/>
+      <c r="N87" s="7"/>
+      <c r="O87" s="7"/>
+      <c r="P87" s="7"/>
+    </row>
+    <row r="88" spans="1:16" ht="38" customHeight="1" thickBot="1">
+      <c r="A88" s="258" t="s">
+        <v>164</v>
+      </c>
+      <c r="B88" s="259" t="s">
+        <v>92</v>
+      </c>
+      <c r="C88" s="250" t="s">
+        <v>53</v>
+      </c>
+      <c r="D88" s="260" t="s">
+        <v>54</v>
+      </c>
+      <c r="E88" s="260" t="s">
+        <v>55</v>
+      </c>
+      <c r="F88" s="250"/>
+      <c r="G88" s="147" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" ht="20" customHeight="1">
+      <c r="A89" s="255" t="str">
+        <f>'BASE PAX'!A64</f>
+        <v>COORDENAÇÃO PRODUÇÃO</v>
+      </c>
+      <c r="B89" s="256">
+        <f>'BASE PAX'!B64</f>
+        <v>0</v>
+      </c>
+      <c r="C89" s="257">
+        <f>'BASE PAX'!C64</f>
+        <v>50000</v>
+      </c>
+      <c r="D89" s="257">
+        <f>'BASE PAX'!D64</f>
+        <v>0</v>
+      </c>
+      <c r="E89" s="121">
+        <f>D89*B89</f>
+        <v>0</v>
+      </c>
+      <c r="F89" s="257"/>
+      <c r="G89" s="199">
+        <f t="shared" ref="G89:G94" si="15">E89*0.2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" ht="20" customHeight="1">
+      <c r="A90" s="251" t="str">
+        <f>'BASE PAX'!A65</f>
+        <v>EXTRA MÃO DE OBRA</v>
+      </c>
+      <c r="B90" s="256">
+        <f>'BASE PAX'!B65</f>
+        <v>0</v>
+      </c>
+      <c r="C90" s="253">
+        <f>'BASE PAX'!C65</f>
+        <v>50000</v>
+      </c>
+      <c r="D90" s="253">
+        <f>'BASE PAX'!D65</f>
+        <v>0</v>
+      </c>
+      <c r="E90" s="121">
+        <f t="shared" ref="E90:E94" si="16">D90*B90</f>
+        <v>0</v>
+      </c>
+      <c r="F90" s="253"/>
+      <c r="G90" s="199">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" ht="20" customHeight="1">
+      <c r="A91" s="251" t="str">
+        <f>'BASE PAX'!A66</f>
+        <v>TAXA LIMPEZA CHECK IN / CHECKOUT</v>
+      </c>
+      <c r="B91" s="252">
+        <f>'BASE PAX'!B66</f>
+        <v>0</v>
+      </c>
+      <c r="C91" s="253">
+        <f>'BASE PAX'!C66</f>
+        <v>40000</v>
+      </c>
+      <c r="D91" s="253">
+        <f>'BASE PAX'!D66</f>
+        <v>0</v>
+      </c>
+      <c r="E91" s="121">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F91" s="253"/>
+      <c r="G91" s="199">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" ht="20" customHeight="1">
+      <c r="A92" s="251" t="str">
+        <f>'BASE PAX'!A67</f>
+        <v>TAXA LIMPEZA DIARIA</v>
+      </c>
+      <c r="B92" s="254">
+        <f>'BASE PAX'!B67</f>
+        <v>0</v>
+      </c>
+      <c r="C92" s="253">
+        <f>'BASE PAX'!C67</f>
+        <v>30000</v>
+      </c>
+      <c r="D92" s="253">
+        <f>'BASE PAX'!D67</f>
+        <v>0</v>
+      </c>
+      <c r="E92" s="121">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F92" s="253"/>
+      <c r="G92" s="199">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" ht="20" customHeight="1">
+      <c r="A93" s="251" t="str">
+        <f>'BASE PAX'!A68</f>
+        <v>SOUVENIR</v>
+      </c>
+      <c r="B93" s="254">
+        <f>'BASE PAX'!B68</f>
+        <v>0</v>
+      </c>
+      <c r="C93" s="253">
+        <f>'BASE PAX'!C68</f>
+        <v>15000</v>
+      </c>
+      <c r="D93" s="253">
+        <f>'BASE PAX'!D68</f>
+        <v>0</v>
+      </c>
+      <c r="E93" s="121">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F93" s="253"/>
+      <c r="G93" s="199">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:16" ht="20" customHeight="1" thickBot="1">
+      <c r="A94" s="251" t="str">
+        <f>'BASE PAX'!A69</f>
+        <v>ASSISTENTE COORDENAÇÃO</v>
+      </c>
+      <c r="B94" s="256">
+        <f>'BASE PAX'!B69</f>
+        <v>0</v>
+      </c>
+      <c r="C94" s="253">
+        <f>'BASE PAX'!C69</f>
+        <v>30000</v>
+      </c>
+      <c r="D94" s="253">
+        <f>'BASE PAX'!D69</f>
+        <v>0</v>
+      </c>
+      <c r="E94" s="121">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F94" s="253"/>
+      <c r="G94" s="199">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" ht="41" customHeight="1" thickBot="1">
+      <c r="A95" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="B95" s="83"/>
+      <c r="C95" s="134"/>
+      <c r="D95" s="134"/>
+      <c r="E95" s="135">
+        <f>SUM(E89:E94)</f>
+        <v>0</v>
+      </c>
+      <c r="F95" s="135"/>
+      <c r="G95" s="203">
+        <f>SUM(G89:G94)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" s="8" customFormat="1" ht="11" customHeight="1" thickBot="1">
+      <c r="A96" s="16"/>
+      <c r="B96" s="56"/>
+      <c r="C96" s="105"/>
+      <c r="D96" s="102"/>
+      <c r="E96" s="102"/>
+      <c r="F96" s="7"/>
+      <c r="G96" s="17"/>
+      <c r="H96" s="7"/>
+      <c r="I96" s="7"/>
+      <c r="J96" s="7"/>
+      <c r="K96" s="7"/>
+      <c r="L96" s="7"/>
+      <c r="M96" s="7"/>
+      <c r="N96" s="7"/>
+      <c r="O96" s="7"/>
+      <c r="P96" s="7"/>
+    </row>
+    <row r="97" spans="1:16" ht="38" customHeight="1" thickBot="1">
+      <c r="A97" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="B97" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="C97" s="136" t="s">
+        <v>53</v>
+      </c>
+      <c r="D97" s="136" t="s">
+        <v>54</v>
+      </c>
+      <c r="E97" s="137" t="s">
+        <v>55</v>
+      </c>
+      <c r="F97" s="20"/>
+      <c r="G97" s="20"/>
+    </row>
+    <row r="98" spans="1:16" ht="23" customHeight="1" thickBot="1">
+      <c r="A98" s="84" t="str">
+        <f>'BASE PAX'!A73</f>
+        <v xml:space="preserve">QUINCHO DAY USE / CABIN </v>
+      </c>
+      <c r="B98" s="279">
+        <f>'BASE PAX'!B73</f>
+        <v>0</v>
+      </c>
+      <c r="C98" s="138">
+        <f>'BASE PAX'!C73</f>
+        <v>15000</v>
+      </c>
+      <c r="D98" s="138">
+        <f>C98+(C98*0.2)</f>
+        <v>18000</v>
+      </c>
+      <c r="E98" s="139">
+        <f>D98*B98</f>
+        <v>0</v>
+      </c>
+      <c r="F98" s="19"/>
+      <c r="G98" s="17"/>
+    </row>
+    <row r="99" spans="1:16" ht="42" customHeight="1" thickBot="1">
+      <c r="A99" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="B99" s="86"/>
+      <c r="C99" s="140"/>
+      <c r="D99" s="140"/>
+      <c r="E99" s="141">
+        <f>E98</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" s="6" customFormat="1" ht="20" customHeight="1">
+      <c r="A100" s="28"/>
+      <c r="B100" s="52"/>
+      <c r="C100" s="11"/>
+      <c r="D100" s="11"/>
+      <c r="E100" s="11"/>
+      <c r="F100" s="7"/>
+      <c r="H100" s="7"/>
+      <c r="I100" s="7"/>
+      <c r="J100" s="7"/>
+      <c r="K100" s="7"/>
+      <c r="L100" s="7"/>
+      <c r="M100" s="7"/>
+      <c r="N100" s="7"/>
+      <c r="O100" s="7"/>
+      <c r="P100" s="7"/>
+    </row>
+    <row r="101" spans="1:16" ht="9" customHeight="1"/>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="17">
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F11:G13"/>
+    <mergeCell ref="G20:G21"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="B1:X96"/>
+  <dimension ref="B1:Y96"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="1.3984375" style="7" customWidth="1"/>
@@ -51307,7 +53918,8 @@
     <col min="22" max="22" width="24.19921875" style="474" customWidth="1"/>
     <col min="23" max="23" width="24.19921875" style="7" customWidth="1"/>
     <col min="24" max="24" width="21.59765625" style="7" customWidth="1"/>
-    <col min="25" max="27" width="25.796875" style="7" customWidth="1"/>
+    <col min="25" max="25" width="25.796875" style="7" customWidth="1"/>
+    <col min="26" max="27" width="25.796875" style="7" customWidth="1"/>
     <col min="28" max="34" width="11" style="7" customWidth="1"/>
     <col min="35" max="16384" width="11" style="7"/>
   </cols>
@@ -51435,6 +54047,9 @@
       <c r="X4" s="486" t="s">
         <v>1</v>
       </c>
+      <c r="Y4" s="486" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="2:24" s="489" customFormat="1" ht="40" customHeight="1" thickBot="1">
       <c r="B5" s="715"/>
@@ -51504,6 +54119,9 @@
       <c r="X5" s="488">
         <v>5</v>
       </c>
+      <c r="Y5" s="488" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="2:24" s="489" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1">
       <c r="B6" s="716"/>
@@ -51572,6 +54190,9 @@
       </c>
       <c r="X6" s="492">
         <v>5</v>
+      </c>
+      <c r="Y6" s="488">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="2:24" s="8" customFormat="1" ht="32" customHeight="1" thickBot="1">
@@ -51600,6 +54221,7 @@
       <c r="V7" s="673"/>
       <c r="W7" s="673"/>
       <c r="X7" s="673"/>
+      <c r="Y7" s="673"/>
     </row>
     <row r="8" spans="2:24" s="8" customFormat="1" ht="24" customHeight="1" thickBot="1">
       <c r="B8" s="670"/>
@@ -51669,6 +54291,9 @@
       <c r="X8" s="555">
         <v>0</v>
       </c>
+      <c r="Y8" s="555">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="2:24" s="496" customFormat="1" ht="40" customHeight="1" thickBot="1">
       <c r="B9" s="493" t="s">
@@ -51740,6 +54365,9 @@
       <c r="X9" s="495" t="s">
         <v>14</v>
       </c>
+      <c r="Y9" s="495" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="10" spans="2:24" ht="40" customHeight="1">
       <c r="B10" s="497" t="s">
@@ -51833,6 +54461,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$13*X8</f>
         <v>0</v>
       </c>
+      <c r="Y10" s="499">
+        <f>'BUDGET NIRE 2+2'!$D$13*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="2:24" s="8" customFormat="1" ht="40" customHeight="1">
       <c r="B11" s="500" t="s">
@@ -51926,6 +54558,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$14*X8</f>
         <v>0</v>
       </c>
+      <c r="Y11" s="502">
+        <f>'BUDGET NIRE 2+2'!$D$14*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="2:24" ht="40" customHeight="1">
       <c r="B12" s="503" t="s">
@@ -52019,6 +54655,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$15*X8</f>
         <v>0</v>
       </c>
+      <c r="Y12" s="505">
+        <f>'BUDGET NIRE 2+2'!$D$15*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="2:24" ht="40" customHeight="1">
       <c r="B13" s="506" t="s">
@@ -52112,6 +54752,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$16*X8</f>
         <v>0</v>
       </c>
+      <c r="Y13" s="508">
+        <f>'BUDGET NIRE 2+2'!$D$16*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="2:24" ht="40" customHeight="1">
       <c r="B14" s="509" t="s">
@@ -52205,6 +54849,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$17*X8</f>
         <v>0</v>
       </c>
+      <c r="Y14" s="511">
+        <f>'BUDGET NIRE 2+2'!$D$17*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="2:24" ht="40" customHeight="1">
       <c r="B15" s="512" t="s">
@@ -52298,6 +54946,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$18*X8</f>
         <v>0</v>
       </c>
+      <c r="Y15" s="514">
+        <f>'BUDGET NIRE 2+2'!$D$18*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="2:24" ht="40" customHeight="1">
       <c r="B16" s="515" t="s">
@@ -52391,6 +55043,10 @@
         <f>'BUDGET CORCOVADO 5'!$D$19*X8</f>
         <v>0</v>
       </c>
+      <c r="Y16" s="517">
+        <f>'BUDGET NIRE 2+2'!$D$19*Y8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:24" ht="40" customHeight="1" thickBot="1">
       <c r="B17" s="518" t="s">
@@ -52482,6 +55138,10 @@
       </c>
       <c r="X17" s="520">
         <f>'BUDGET CORCOVADO 5'!$D$20*X8</f>
+        <v>0</v>
+      </c>
+      <c r="Y17" s="520">
+        <f>'BUDGET NIRE 2+2'!$D$20*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -52509,6 +55169,7 @@
       <c r="V18" s="522"/>
       <c r="W18" s="523"/>
       <c r="X18" s="523"/>
+      <c r="Y18" s="523"/>
     </row>
     <row r="19" spans="2:24" s="526" customFormat="1" ht="40" customHeight="1" thickBot="1">
       <c r="B19" s="524" t="s">
@@ -52602,6 +55263,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="Y19" s="525">
+        <f>SUM(Y10:Y17)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="2:24" s="526" customFormat="1" ht="29" customHeight="1" thickBot="1">
       <c r="B20" s="527" t="s">
@@ -52695,6 +55360,10 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="Y20" s="529">
+        <f>Y19*0.05</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="2:24" s="526" customFormat="1" ht="40" customHeight="1" thickBot="1">
       <c r="B21" s="530" t="s">
@@ -52786,6 +55455,10 @@
       </c>
       <c r="X21" s="532">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y21" s="532">
+        <f>Y19-Y20</f>
         <v>0</v>
       </c>
     </row>
@@ -52813,6 +55486,7 @@
       <c r="V22" s="534"/>
       <c r="W22" s="535"/>
       <c r="X22" s="535"/>
+      <c r="Y22" s="535"/>
     </row>
     <row r="23" spans="2:24" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="B23" s="536" t="s">
@@ -52843,6 +55517,7 @@
       <c r="V23" s="362"/>
       <c r="W23" s="362"/>
       <c r="X23" s="362"/>
+      <c r="Y23" s="538"/>
     </row>
     <row r="24" spans="2:24" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="B24" s="539" t="s">
@@ -52873,6 +55548,7 @@
       <c r="V24" s="362"/>
       <c r="W24" s="362"/>
       <c r="X24" s="362"/>
+      <c r="Y24" s="538"/>
     </row>
     <row r="25" spans="2:24" s="489" customFormat="1" ht="48" customHeight="1">
       <c r="B25" s="540" t="s">
@@ -52966,6 +55642,10 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+      <c r="Y25" s="542">
+        <f>Y21+(Y21*$C$23)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="2:24" s="489" customFormat="1" ht="49" customHeight="1" thickBot="1">
       <c r="B26" s="543" t="s">
@@ -53059,6 +55739,10 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="Y26" s="544">
+        <f>Y25+(Y25*$C$24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="2:24" ht="40" customHeight="1" thickBot="1">
       <c r="B27" s="545" t="s">
@@ -53150,6 +55834,10 @@
       </c>
       <c r="X27" s="547">
         <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Y27" s="547">
+        <f>Y26-Y19</f>
         <v>0</v>
       </c>
     </row>
@@ -53246,6 +55934,10 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="Y29" s="525">
+        <f>Y19/Y6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="2:24" s="489" customFormat="1" ht="49" customHeight="1" thickBot="1">
       <c r="B30" s="543" t="s">
@@ -53339,6 +56031,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="Y30" s="544">
+        <f>Y29+(Y29*Y28)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="2:24" ht="54" customHeight="1" thickBot="1">
       <c r="B31" s="545" t="s">
@@ -53430,6 +56126,10 @@
       </c>
       <c r="X31" s="547">
         <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="Y31" s="547">
+        <f>Y30-Y24</f>
         <v>0</v>
       </c>
     </row>
@@ -54470,7 +57170,7 @@
       <c r="C11" s="586"/>
       <c r="D11" s="586"/>
       <c r="E11" s="587">
-        <f>('BUDGET RESUMO'!C10*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D10*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F10*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G10*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I10*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J10*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L10*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N10*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O10*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P10*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q10*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R10*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S10*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T10*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U10*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V10*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E10*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H10*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M10*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X10*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W10*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K10*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C10*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D10*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F10*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G10*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I10*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J10*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L10*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N10*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O10*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P10*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q10*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R10*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S10*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T10*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U10*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V10*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E10*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H10*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M10*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X10*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W10*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K10*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y10*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="H11" s="581"/>
@@ -54489,7 +57189,7 @@
       <c r="C13" s="590"/>
       <c r="D13" s="590"/>
       <c r="E13" s="591">
-        <f>('BUDGET RESUMO'!C11*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D11*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F11*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G11*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I11*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J11*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L11*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N11*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O11*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P11*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q11*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R11*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S11*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T11*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U11*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V11*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E11*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H11*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M11*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X11*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W11*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K11*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C11*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D11*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F11*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G11*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I11*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J11*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L11*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N11*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O11*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P11*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q11*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R11*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S11*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T11*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U11*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V11*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E11*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H11*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M11*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X11*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W11*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K11*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y11*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="G13" s="592">
@@ -54516,7 +57216,7 @@
       <c r="C15" s="599"/>
       <c r="D15" s="599"/>
       <c r="E15" s="600">
-        <f>('BUDGET RESUMO'!C12*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D12*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F12*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G12*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I12*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J12*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L12*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N12*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O12*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P12*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q12*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R12*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S12*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T12*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U12*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V12*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E12*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H12*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M12*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X12*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W12*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K12*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C12*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D12*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F12*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G12*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I12*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J12*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L12*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N12*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O12*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P12*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q12*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R12*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S12*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T12*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U12*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V12*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E12*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H12*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M12*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X12*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W12*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K12*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y12*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="H15" s="593">
@@ -54538,7 +57238,7 @@
       <c r="C17" s="606"/>
       <c r="D17" s="606"/>
       <c r="E17" s="607">
-        <f>('BUDGET RESUMO'!C13*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D13*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F13*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G13*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I13*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J13*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L13*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N13*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O13*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P13*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q13*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R13*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S13*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T13*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U13*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V13*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E13*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H13*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M13*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X13*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W13*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K13*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C13*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D13*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F13*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G13*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I13*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J13*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L13*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N13*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O13*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P13*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q13*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R13*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S13*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T13*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U13*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V13*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E13*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H13*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M13*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X13*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W13*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K13*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y13*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="H17" s="593">
@@ -54560,7 +57260,7 @@
       <c r="C19" s="609"/>
       <c r="D19" s="609"/>
       <c r="E19" s="613">
-        <f>('BUDGET RESUMO'!C14*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D14*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F14*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G14*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I14*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J14*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L14*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N14*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O14*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P14*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q14*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R14*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S14*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T14*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U14*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V14*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E14*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H14*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M14*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X14*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W14*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K14*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C14*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D14*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F14*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G14*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I14*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J14*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L14*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N14*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O14*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P14*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q14*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R14*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S14*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T14*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U14*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V14*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E14*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H14*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M14*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X14*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W14*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K14*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y14*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="H19" s="593">
@@ -54582,7 +57282,7 @@
       <c r="C21" s="618"/>
       <c r="D21" s="618"/>
       <c r="E21" s="619">
-        <f>('BUDGET RESUMO'!C15*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D15*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F15*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G15*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I15*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J15*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L15*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N15*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O15*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P15*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q15*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R15*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S15*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T15*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U15*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V15*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E15*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H15*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M15*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X15*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W15*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K15*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C15*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D15*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F15*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G15*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I15*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J15*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L15*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N15*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O15*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P15*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q15*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R15*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S15*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T15*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U15*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V15*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E15*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H15*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M15*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X15*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W15*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K15*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y15*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="H21" s="593">
@@ -54604,7 +57304,7 @@
       <c r="C23" s="624"/>
       <c r="D23" s="624"/>
       <c r="E23" s="625">
-        <f>('BUDGET RESUMO'!C16*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D16*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F16*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G16*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I16*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J16*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L16*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N16*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O16*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P16*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q16*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R16*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S16*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T16*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U16*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V16*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E16*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H16*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M16*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X16*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W16*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K16*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C16*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D16*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F16*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G16*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I16*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J16*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L16*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N16*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O16*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P16*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q16*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R16*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S16*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T16*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U16*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V16*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E16*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H16*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M16*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X16*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W16*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K16*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y16*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
       <c r="H23" s="593">
@@ -54628,7 +57328,7 @@
       <c r="C25" s="631"/>
       <c r="D25" s="631"/>
       <c r="E25" s="632">
-        <f>('BUDGET RESUMO'!C17*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D17*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F17*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G17*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I17*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J17*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L17*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N17*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O17*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P17*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q17*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R17*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S17*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T17*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U17*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V17*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E17*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H17*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M17*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X17*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W17*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K17*'BUDGET RESUMO'!$K$8)</f>
+        <f>('BUDGET RESUMO'!C17*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D17*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F17*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G17*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I17*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J17*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L17*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N17*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O17*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P17*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q17*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R17*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S17*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T17*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U17*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V17*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E17*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H17*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M17*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X17*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W17*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K17*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y17*'BUDGET RESUMO'!$Y$8)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorganiza coluna NIRE 2+2 para ficar junto das outras colunas NIRE
- NIRE 2+2 estava anexada no final da BUDGET RESUMO (coluna Y) -
  movida para logo apos NIRE 2+1 (coluna I), com CHAITEN/CORCOVADO
  deslocados uma coluna a mais (J-Y) para nao colidir
- CABIN_MAP atualizado com as novas letras de CHAITEN e CORCOVADO
- Testado: geracao isolada NIRE 2+2 e regressao com as 4 cabanas
  simultaneas batem exatamente com os valores de antes do deslocamento
</commit_message>
<xml_diff>
--- a/assets/templates/planilha_orcamentos_python.xlsx
+++ b/assets/templates/planilha_orcamentos_python.xlsx
@@ -53929,7 +53929,7 @@
       <c r="B2" s="9"/>
       <c r="E2" s="9"/>
       <c r="H2" s="9"/>
-      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
     </row>
     <row r="3" spans="2:24" s="10" customFormat="1" ht="69" customHeight="1" thickBot="1">
       <c r="B3" s="475"/>
@@ -53950,24 +53950,23 @@
         <v>1</v>
       </c>
       <c r="H3" s="479"/>
-      <c r="I3" s="480"/>
-      <c r="J3" s="481" t="str">
+      <c r="J3" s="480"/>
+      <c r="K3" s="481" t="str">
         <f>CALENDAR!I2</f>
         <v>NIGHTS</v>
       </c>
-      <c r="K3" s="482">
+      <c r="L3" s="482">
         <f>CALENDAR!J2</f>
         <v>0</v>
       </c>
-      <c r="L3" s="483">
+      <c r="M3" s="483">
         <f>CALENDAR!J2</f>
         <v>0</v>
       </c>
-      <c r="M3" s="718" t="str">
+      <c r="N3" s="718" t="str">
         <f>CALENDAR!K2</f>
         <v>NOME CLIENTE | PROGRAMA</v>
       </c>
-      <c r="N3" s="673"/>
       <c r="O3" s="673"/>
       <c r="P3" s="673"/>
       <c r="Q3" s="673"/>
@@ -53978,6 +53977,7 @@
       <c r="V3" s="673"/>
       <c r="W3" s="673"/>
       <c r="X3" s="673"/>
+      <c r="Y3" s="673"/>
     </row>
     <row r="4" spans="2:24" s="8" customFormat="1" ht="32" customHeight="1" thickBot="1">
       <c r="B4" s="484"/>
@@ -53999,22 +53999,22 @@
       <c r="H4" s="486" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="485" t="s">
+      <c r="I4" s="486" t="s">
         <v>1</v>
       </c>
       <c r="J4" s="485" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="486" t="s">
+      <c r="K4" s="485" t="s">
         <v>1</v>
       </c>
-      <c r="L4" s="485" t="s">
+      <c r="L4" s="486" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="486" t="s">
+      <c r="M4" s="485" t="s">
         <v>1</v>
       </c>
-      <c r="N4" s="485" t="s">
+      <c r="N4" s="486" t="s">
         <v>1</v>
       </c>
       <c r="O4" s="485" t="s">
@@ -54041,7 +54041,7 @@
       <c r="V4" s="485" t="s">
         <v>1</v>
       </c>
-      <c r="W4" s="486" t="s">
+      <c r="W4" s="485" t="s">
         <v>1</v>
       </c>
       <c r="X4" s="486" t="s">
@@ -54071,56 +54071,56 @@
       <c r="H5" s="488" t="s">
         <v>2</v>
       </c>
-      <c r="I5" s="487">
+      <c r="I5" s="488" t="s">
+        <v>4</v>
+      </c>
+      <c r="J5" s="487">
         <v>1</v>
       </c>
-      <c r="J5" s="487">
+      <c r="K5" s="487">
         <v>2</v>
       </c>
-      <c r="K5" s="488" t="s">
+      <c r="L5" s="488" t="s">
         <v>3</v>
       </c>
-      <c r="L5" s="487" t="s">
+      <c r="M5" s="487" t="s">
         <v>2</v>
       </c>
-      <c r="M5" s="488" t="s">
+      <c r="N5" s="488" t="s">
         <v>4</v>
       </c>
-      <c r="N5" s="487">
+      <c r="O5" s="487">
         <v>1</v>
       </c>
-      <c r="O5" s="487">
+      <c r="P5" s="487">
         <v>2</v>
       </c>
-      <c r="P5" s="487" t="s">
+      <c r="Q5" s="487" t="s">
         <v>2</v>
       </c>
-      <c r="Q5" s="487" t="s">
+      <c r="R5" s="487" t="s">
         <v>4</v>
       </c>
-      <c r="R5" s="487" t="s">
+      <c r="S5" s="487" t="s">
         <v>5</v>
       </c>
-      <c r="S5" s="487">
+      <c r="T5" s="487">
         <v>3</v>
       </c>
-      <c r="T5" s="487" t="s">
+      <c r="U5" s="487" t="s">
         <v>6</v>
       </c>
-      <c r="U5" s="487" t="s">
+      <c r="V5" s="487" t="s">
         <v>7</v>
       </c>
-      <c r="V5" s="487">
+      <c r="W5" s="487">
         <v>4</v>
       </c>
-      <c r="W5" s="488" t="s">
+      <c r="X5" s="488" t="s">
         <v>8</v>
       </c>
-      <c r="X5" s="488">
+      <c r="Y5" s="488">
         <v>5</v>
-      </c>
-      <c r="Y5" s="488" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:24" s="489" customFormat="1" ht="40" hidden="1" customHeight="1" thickBot="1">
@@ -54143,56 +54143,56 @@
       <c r="H6" s="492">
         <v>3</v>
       </c>
-      <c r="I6" s="491">
+      <c r="I6" s="488">
+        <v>4</v>
+      </c>
+      <c r="J6" s="491">
         <v>1</v>
       </c>
-      <c r="J6" s="491">
+      <c r="K6" s="491">
         <v>2</v>
       </c>
-      <c r="K6" s="488">
+      <c r="L6" s="488">
         <v>3</v>
       </c>
-      <c r="L6" s="487">
+      <c r="M6" s="487">
         <v>3</v>
       </c>
-      <c r="M6" s="488">
+      <c r="N6" s="488">
         <v>4</v>
       </c>
-      <c r="N6" s="491">
+      <c r="O6" s="491">
         <v>1</v>
       </c>
-      <c r="O6" s="491">
+      <c r="P6" s="491">
         <v>2</v>
       </c>
-      <c r="P6" s="487">
+      <c r="Q6" s="487">
         <v>3</v>
       </c>
-      <c r="Q6" s="491">
+      <c r="R6" s="491">
         <v>4</v>
       </c>
-      <c r="R6" s="491">
+      <c r="S6" s="491">
         <v>5</v>
       </c>
-      <c r="S6" s="491">
+      <c r="T6" s="491">
         <v>3</v>
       </c>
-      <c r="T6" s="491">
+      <c r="U6" s="491">
         <v>4</v>
       </c>
-      <c r="U6" s="491">
+      <c r="V6" s="491">
         <v>5</v>
       </c>
-      <c r="V6" s="491">
+      <c r="W6" s="491">
         <v>4</v>
-      </c>
-      <c r="W6" s="492">
-        <v>5</v>
       </c>
       <c r="X6" s="492">
         <v>5</v>
       </c>
-      <c r="Y6" s="488">
-        <v>4</v>
+      <c r="Y6" s="492">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:24" s="8" customFormat="1" ht="32" customHeight="1" thickBot="1">
@@ -54243,22 +54243,22 @@
       <c r="H8" s="555">
         <v>0</v>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="555">
         <v>0</v>
       </c>
       <c r="J8" s="31">
         <v>0</v>
       </c>
-      <c r="K8" s="555">
-        <v>0</v>
-      </c>
-      <c r="L8" s="31">
-        <v>0</v>
-      </c>
-      <c r="M8" s="555">
-        <v>0</v>
-      </c>
-      <c r="N8" s="31">
+      <c r="K8" s="31">
+        <v>0</v>
+      </c>
+      <c r="L8" s="555">
+        <v>0</v>
+      </c>
+      <c r="M8" s="31">
+        <v>0</v>
+      </c>
+      <c r="N8" s="555">
         <v>0</v>
       </c>
       <c r="O8" s="31">
@@ -54285,7 +54285,7 @@
       <c r="V8" s="31">
         <v>0</v>
       </c>
-      <c r="W8" s="555">
+      <c r="W8" s="31">
         <v>0</v>
       </c>
       <c r="X8" s="555">
@@ -54317,23 +54317,23 @@
       <c r="H9" s="495" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="494" t="s">
-        <v>13</v>
+      <c r="I9" s="495" t="s">
+        <v>12</v>
       </c>
       <c r="J9" s="494" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="495" t="s">
+      <c r="K9" s="494" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="494" t="s">
+      <c r="L9" s="495" t="s">
         <v>13</v>
       </c>
-      <c r="M9" s="495" t="s">
+      <c r="M9" s="494" t="s">
         <v>13</v>
       </c>
-      <c r="N9" s="494" t="s">
-        <v>14</v>
+      <c r="N9" s="495" t="s">
+        <v>13</v>
       </c>
       <c r="O9" s="494" t="s">
         <v>14</v>
@@ -54359,14 +54359,14 @@
       <c r="V9" s="494" t="s">
         <v>14</v>
       </c>
-      <c r="W9" s="495" t="s">
+      <c r="W9" s="494" t="s">
         <v>14</v>
       </c>
       <c r="X9" s="495" t="s">
         <v>14</v>
       </c>
       <c r="Y9" s="495" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:24" ht="40" customHeight="1">
@@ -54397,72 +54397,72 @@
         <f>'BUDGET NIRE 2+1'!$D$13*H8</f>
         <v>0</v>
       </c>
-      <c r="I10" s="498">
-        <f>'BUDGET CHAITEN 1'!$D$13*I8</f>
+      <c r="I10" s="499">
+        <f>'BUDGET NIRE 2+2'!$D$13*I8</f>
         <v>0</v>
       </c>
       <c r="J10" s="498">
-        <f>'BUDGET CHAITEN 2'!$D$13*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="499">
-        <f>'BUDGET CHAITEN 3'!$D$13*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L10" s="498">
-        <f>'BUDGET CHAITEN 2+1'!$D$13*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M10" s="499">
-        <f>'BUDGET CHAITEN 2+2'!$D$13*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N10" s="498">
-        <f>'BUDGET CORCOVADO 1'!$D$13*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$13*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="498">
+        <f>'BUDGET CHAITEN 2'!$D$13*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="499">
+        <f>'BUDGET CHAITEN 3'!$D$13*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="498">
+        <f>'BUDGET CHAITEN 2+1'!$D$13*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="499">
+        <f>'BUDGET CHAITEN 2+2'!$D$13*N8</f>
         <v>0</v>
       </c>
       <c r="O10" s="498">
-        <f>'BUDGET CORCOVADO 2'!$D$13*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$13*O8</f>
         <v>0</v>
       </c>
       <c r="P10" s="498">
-        <f>'BUDGET CORCOVADO 2+1'!$D$13*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$13*P8</f>
         <v>0</v>
       </c>
       <c r="Q10" s="498">
-        <f>'BUDGET CORCOVADO 2+2'!$D$13*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$13*Q8</f>
         <v>0</v>
       </c>
       <c r="R10" s="498">
-        <f>'BUDGET CORCOVADO 2+3'!$D$13*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$13*R8</f>
         <v>0</v>
       </c>
       <c r="S10" s="498">
-        <f>'BUDGET CORCOVADO 3'!$D$13*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$13*S8</f>
         <v>0</v>
       </c>
       <c r="T10" s="498">
-        <f>'BUDGET CORCOVADO 3+1'!$D$13*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$13*T8</f>
         <v>0</v>
       </c>
       <c r="U10" s="498">
-        <f>'BUDGET CORCOVADO 3+2'!$D$13*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$13*U8</f>
         <v>0</v>
       </c>
       <c r="V10" s="498">
-        <f>'BUDGET CORCOVADO 4'!$D$13*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W10" s="499">
-        <f>'BUDGET CORCOVADO 4+1'!$D$13*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$13*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W10" s="498">
+        <f>'BUDGET CORCOVADO 4'!$D$13*W8</f>
         <v>0</v>
       </c>
       <c r="X10" s="499">
-        <f>'BUDGET CORCOVADO 5'!$D$13*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$13*X8</f>
         <v>0</v>
       </c>
       <c r="Y10" s="499">
-        <f>'BUDGET NIRE 2+2'!$D$13*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$13*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -54494,72 +54494,72 @@
         <f>'BUDGET NIRE 2+1'!$D$14*H8</f>
         <v>0</v>
       </c>
-      <c r="I11" s="501">
-        <f>'BUDGET CHAITEN 1'!$D$14*I8</f>
+      <c r="I11" s="502">
+        <f>'BUDGET NIRE 2+2'!$D$14*I8</f>
         <v>0</v>
       </c>
       <c r="J11" s="501">
-        <f>'BUDGET CHAITEN 2'!$D$14*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="502">
-        <f>'BUDGET CHAITEN 3'!$D$14*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L11" s="501">
-        <f>'BUDGET CHAITEN 2+1'!$D$14*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="502">
-        <f>'BUDGET CHAITEN 2+2'!$D$14*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="501">
-        <f>'BUDGET CORCOVADO 1'!$D$14*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$14*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="501">
+        <f>'BUDGET CHAITEN 2'!$D$14*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="502">
+        <f>'BUDGET CHAITEN 3'!$D$14*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="501">
+        <f>'BUDGET CHAITEN 2+1'!$D$14*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="502">
+        <f>'BUDGET CHAITEN 2+2'!$D$14*N8</f>
         <v>0</v>
       </c>
       <c r="O11" s="501">
-        <f>'BUDGET CORCOVADO 2'!$D$14*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$14*O8</f>
         <v>0</v>
       </c>
       <c r="P11" s="501">
-        <f>'BUDGET CORCOVADO 2+1'!$D$14*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$14*P8</f>
         <v>0</v>
       </c>
       <c r="Q11" s="501">
-        <f>'BUDGET CORCOVADO 2+2'!$D$14*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$14*Q8</f>
         <v>0</v>
       </c>
       <c r="R11" s="501">
-        <f>'BUDGET CORCOVADO 2+3'!$D$14*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$14*R8</f>
         <v>0</v>
       </c>
       <c r="S11" s="501">
-        <f>'BUDGET CORCOVADO 3'!$D$14*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$14*S8</f>
         <v>0</v>
       </c>
       <c r="T11" s="501">
-        <f>'BUDGET CORCOVADO 3+1'!$D$14*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$14*T8</f>
         <v>0</v>
       </c>
       <c r="U11" s="501">
-        <f>'BUDGET CORCOVADO 3+2'!$D$14*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$14*U8</f>
         <v>0</v>
       </c>
       <c r="V11" s="501">
-        <f>'BUDGET CORCOVADO 4'!$D$14*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W11" s="502">
-        <f>'BUDGET CORCOVADO 4+1'!$D$14*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$14*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W11" s="501">
+        <f>'BUDGET CORCOVADO 4'!$D$14*W8</f>
         <v>0</v>
       </c>
       <c r="X11" s="502">
-        <f>'BUDGET CORCOVADO 5'!$D$14*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$14*X8</f>
         <v>0</v>
       </c>
       <c r="Y11" s="502">
-        <f>'BUDGET NIRE 2+2'!$D$14*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$14*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -54591,72 +54591,72 @@
         <f>'BUDGET NIRE 2+1'!$D$15*H8</f>
         <v>0</v>
       </c>
-      <c r="I12" s="504">
-        <f>'BUDGET CHAITEN 1'!$D$15*I8</f>
+      <c r="I12" s="505">
+        <f>'BUDGET NIRE 2+2'!$D$15*I8</f>
         <v>0</v>
       </c>
       <c r="J12" s="504">
-        <f>'BUDGET CHAITEN 2'!$D$15*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="505">
-        <f>'BUDGET CHAITEN 3'!$D$15*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="504">
-        <f>'BUDGET CHAITEN 2+1'!$D$15*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M12" s="505">
-        <f>'BUDGET CHAITEN 2+2'!$D$15*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N12" s="504">
-        <f>'BUDGET CORCOVADO 1'!$D$15*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$15*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="504">
+        <f>'BUDGET CHAITEN 2'!$D$15*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="505">
+        <f>'BUDGET CHAITEN 3'!$D$15*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="504">
+        <f>'BUDGET CHAITEN 2+1'!$D$15*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N12" s="505">
+        <f>'BUDGET CHAITEN 2+2'!$D$15*N8</f>
         <v>0</v>
       </c>
       <c r="O12" s="504">
-        <f>'BUDGET CORCOVADO 2'!$D$15*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$15*O8</f>
         <v>0</v>
       </c>
       <c r="P12" s="504">
-        <f>'BUDGET CORCOVADO 2+1'!$D$15*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$15*P8</f>
         <v>0</v>
       </c>
       <c r="Q12" s="504">
-        <f>'BUDGET CORCOVADO 2+2'!$D$15*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$15*Q8</f>
         <v>0</v>
       </c>
       <c r="R12" s="504">
-        <f>'BUDGET CORCOVADO 2+3'!$D$15*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$15*R8</f>
         <v>0</v>
       </c>
       <c r="S12" s="504">
-        <f>'BUDGET CORCOVADO 3'!$D$15*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$15*S8</f>
         <v>0</v>
       </c>
       <c r="T12" s="504">
-        <f>'BUDGET CORCOVADO 3+1'!$D$15*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$15*T8</f>
         <v>0</v>
       </c>
       <c r="U12" s="504">
-        <f>'BUDGET CORCOVADO 3+2'!$D$15*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$15*U8</f>
         <v>0</v>
       </c>
       <c r="V12" s="504">
-        <f>'BUDGET CORCOVADO 4'!$D$15*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W12" s="505">
-        <f>'BUDGET CORCOVADO 4+1'!$D$15*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$15*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W12" s="504">
+        <f>'BUDGET CORCOVADO 4'!$D$15*W8</f>
         <v>0</v>
       </c>
       <c r="X12" s="505">
-        <f>'BUDGET CORCOVADO 5'!$D$15*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$15*X8</f>
         <v>0</v>
       </c>
       <c r="Y12" s="505">
-        <f>'BUDGET NIRE 2+2'!$D$15*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$15*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -54688,72 +54688,72 @@
         <f>'BUDGET NIRE 2+1'!$D$16*H8</f>
         <v>0</v>
       </c>
-      <c r="I13" s="507">
-        <f>'BUDGET CHAITEN 1'!$D$16*I8</f>
+      <c r="I13" s="508">
+        <f>'BUDGET NIRE 2+2'!$D$16*I8</f>
         <v>0</v>
       </c>
       <c r="J13" s="507">
-        <f>'BUDGET CHAITEN 2'!$D$16*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K13" s="508">
-        <f>'BUDGET CHAITEN 3'!$D$16*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L13" s="507">
-        <f>'BUDGET CHAITEN 2+1'!$D$16*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="508">
-        <f>'BUDGET CHAITEN 2+2'!$D$16*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N13" s="507">
-        <f>'BUDGET CORCOVADO 1'!$D$16*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$16*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="507">
+        <f>'BUDGET CHAITEN 2'!$D$16*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="508">
+        <f>'BUDGET CHAITEN 3'!$D$16*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="507">
+        <f>'BUDGET CHAITEN 2+1'!$D$16*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N13" s="508">
+        <f>'BUDGET CHAITEN 2+2'!$D$16*N8</f>
         <v>0</v>
       </c>
       <c r="O13" s="507">
-        <f>'BUDGET CORCOVADO 2'!$D$16*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$16*O8</f>
         <v>0</v>
       </c>
       <c r="P13" s="507">
-        <f>'BUDGET CORCOVADO 2+1'!$D$16*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$16*P8</f>
         <v>0</v>
       </c>
       <c r="Q13" s="507">
-        <f>'BUDGET CORCOVADO 2+2'!$D$16*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$16*Q8</f>
         <v>0</v>
       </c>
       <c r="R13" s="507">
-        <f>'BUDGET CORCOVADO 2+3'!$D$16*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$16*R8</f>
         <v>0</v>
       </c>
       <c r="S13" s="507">
-        <f>'BUDGET CORCOVADO 3'!$D$16*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$16*S8</f>
         <v>0</v>
       </c>
       <c r="T13" s="507">
-        <f>'BUDGET CORCOVADO 3+1'!$D$16*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$16*T8</f>
         <v>0</v>
       </c>
       <c r="U13" s="507">
-        <f>'BUDGET CORCOVADO 3+2'!$D$16*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$16*U8</f>
         <v>0</v>
       </c>
       <c r="V13" s="507">
-        <f>'BUDGET CORCOVADO 4'!$D$16*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W13" s="508">
-        <f>'BUDGET CORCOVADO 4+1'!$D$16*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$16*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W13" s="507">
+        <f>'BUDGET CORCOVADO 4'!$D$16*W8</f>
         <v>0</v>
       </c>
       <c r="X13" s="508">
-        <f>'BUDGET CORCOVADO 5'!$D$16*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$16*X8</f>
         <v>0</v>
       </c>
       <c r="Y13" s="508">
-        <f>'BUDGET NIRE 2+2'!$D$16*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$16*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -54785,72 +54785,72 @@
         <f>'BUDGET NIRE 2+1'!$D$17*H8</f>
         <v>0</v>
       </c>
-      <c r="I14" s="510">
-        <f>'BUDGET CHAITEN 1'!$D$17*I8</f>
+      <c r="I14" s="511">
+        <f>'BUDGET NIRE 2+2'!$D$17*I8</f>
         <v>0</v>
       </c>
       <c r="J14" s="510">
-        <f>'BUDGET CHAITEN 2'!$D$17*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="511">
-        <f>'BUDGET CHAITEN 3'!$D$17*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="510">
-        <f>'BUDGET CHAITEN 2+1'!$D$17*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="511">
-        <f>'BUDGET CHAITEN 2+2'!$D$17*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N14" s="510">
-        <f>'BUDGET CORCOVADO 1'!$D$17*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$17*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="510">
+        <f>'BUDGET CHAITEN 2'!$D$17*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="511">
+        <f>'BUDGET CHAITEN 3'!$D$17*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="510">
+        <f>'BUDGET CHAITEN 2+1'!$D$17*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="511">
+        <f>'BUDGET CHAITEN 2+2'!$D$17*N8</f>
         <v>0</v>
       </c>
       <c r="O14" s="510">
-        <f>'BUDGET CORCOVADO 2'!$D$17*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$17*O8</f>
         <v>0</v>
       </c>
       <c r="P14" s="510">
-        <f>'BUDGET CORCOVADO 2+1'!$D$17*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$17*P8</f>
         <v>0</v>
       </c>
       <c r="Q14" s="510">
-        <f>'BUDGET CORCOVADO 2+2'!$D$17*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$17*Q8</f>
         <v>0</v>
       </c>
       <c r="R14" s="510">
-        <f>'BUDGET CORCOVADO 2+3'!$D$17*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$17*R8</f>
         <v>0</v>
       </c>
       <c r="S14" s="510">
-        <f>'BUDGET CORCOVADO 3'!$D$17*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$17*S8</f>
         <v>0</v>
       </c>
       <c r="T14" s="510">
-        <f>'BUDGET CORCOVADO 3+1'!$D$17*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$17*T8</f>
         <v>0</v>
       </c>
       <c r="U14" s="510">
-        <f>'BUDGET CORCOVADO 3+2'!$D$17*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$17*U8</f>
         <v>0</v>
       </c>
       <c r="V14" s="510">
-        <f>'BUDGET CORCOVADO 4'!$D$17*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W14" s="511">
-        <f>'BUDGET CORCOVADO 4+1'!$D$17*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$17*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W14" s="510">
+        <f>'BUDGET CORCOVADO 4'!$D$17*W8</f>
         <v>0</v>
       </c>
       <c r="X14" s="511">
-        <f>'BUDGET CORCOVADO 5'!$D$17*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$17*X8</f>
         <v>0</v>
       </c>
       <c r="Y14" s="511">
-        <f>'BUDGET NIRE 2+2'!$D$17*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$17*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -54882,72 +54882,72 @@
         <f>'BUDGET NIRE 2+1'!$D$18*H8</f>
         <v>0</v>
       </c>
-      <c r="I15" s="513">
-        <f>'BUDGET CHAITEN 1'!$D$18*I8</f>
+      <c r="I15" s="514">
+        <f>'BUDGET NIRE 2+2'!$D$18*I8</f>
         <v>0</v>
       </c>
       <c r="J15" s="513">
-        <f>'BUDGET CHAITEN 2'!$D$18*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="514">
-        <f>'BUDGET CHAITEN 3'!$D$18*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="513">
-        <f>'BUDGET CHAITEN 2+1'!$D$18*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="514">
-        <f>'BUDGET CHAITEN 2+2'!$D$18*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="513">
-        <f>'BUDGET CORCOVADO 1'!$D$18*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$18*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="513">
+        <f>'BUDGET CHAITEN 2'!$D$18*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="514">
+        <f>'BUDGET CHAITEN 3'!$D$18*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="513">
+        <f>'BUDGET CHAITEN 2+1'!$D$18*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="514">
+        <f>'BUDGET CHAITEN 2+2'!$D$18*N8</f>
         <v>0</v>
       </c>
       <c r="O15" s="513">
-        <f>'BUDGET CORCOVADO 2'!$D$18*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$18*O8</f>
         <v>0</v>
       </c>
       <c r="P15" s="513">
-        <f>'BUDGET CORCOVADO 2+1'!$D$18*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$18*P8</f>
         <v>0</v>
       </c>
       <c r="Q15" s="513">
-        <f>'BUDGET CORCOVADO 2+2'!$D$18*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$18*Q8</f>
         <v>0</v>
       </c>
       <c r="R15" s="513">
-        <f>'BUDGET CORCOVADO 2+3'!$D$18*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$18*R8</f>
         <v>0</v>
       </c>
       <c r="S15" s="513">
-        <f>'BUDGET CORCOVADO 3'!$D$18*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$18*S8</f>
         <v>0</v>
       </c>
       <c r="T15" s="513">
-        <f>'BUDGET CORCOVADO 3+1'!$D$18*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$18*T8</f>
         <v>0</v>
       </c>
       <c r="U15" s="513">
-        <f>'BUDGET CORCOVADO 3+2'!$D$18*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$18*U8</f>
         <v>0</v>
       </c>
       <c r="V15" s="513">
-        <f>'BUDGET CORCOVADO 4'!$D$18*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W15" s="514">
-        <f>'BUDGET CORCOVADO 4+1'!$D$18*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$18*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W15" s="513">
+        <f>'BUDGET CORCOVADO 4'!$D$18*W8</f>
         <v>0</v>
       </c>
       <c r="X15" s="514">
-        <f>'BUDGET CORCOVADO 5'!$D$18*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$18*X8</f>
         <v>0</v>
       </c>
       <c r="Y15" s="514">
-        <f>'BUDGET NIRE 2+2'!$D$18*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$18*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -54979,72 +54979,72 @@
         <f>'BUDGET NIRE 2+1'!$D$19*H8</f>
         <v>0</v>
       </c>
-      <c r="I16" s="516">
-        <f>'BUDGET CHAITEN 1'!$D$19*I8</f>
+      <c r="I16" s="517">
+        <f>'BUDGET NIRE 2+2'!$D$19*I8</f>
         <v>0</v>
       </c>
       <c r="J16" s="516">
-        <f>'BUDGET CHAITEN 2'!$D$19*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K16" s="517">
-        <f>'BUDGET CHAITEN 3'!$D$19*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="516">
-        <f>'BUDGET CHAITEN 2+1'!$D$19*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="517">
-        <f>'BUDGET CHAITEN 2+2'!$D$19*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="516">
-        <f>'BUDGET CORCOVADO 1'!$D$19*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$19*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="516">
+        <f>'BUDGET CHAITEN 2'!$D$19*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="517">
+        <f>'BUDGET CHAITEN 3'!$D$19*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="516">
+        <f>'BUDGET CHAITEN 2+1'!$D$19*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N16" s="517">
+        <f>'BUDGET CHAITEN 2+2'!$D$19*N8</f>
         <v>0</v>
       </c>
       <c r="O16" s="516">
-        <f>'BUDGET CORCOVADO 2'!$D$19*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$19*O8</f>
         <v>0</v>
       </c>
       <c r="P16" s="516">
-        <f>'BUDGET CORCOVADO 2+1'!$D$19*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$19*P8</f>
         <v>0</v>
       </c>
       <c r="Q16" s="516">
-        <f>'BUDGET CORCOVADO 2+2'!$D$19*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$19*Q8</f>
         <v>0</v>
       </c>
       <c r="R16" s="516">
-        <f>'BUDGET CORCOVADO 2+3'!$D$19*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$19*R8</f>
         <v>0</v>
       </c>
       <c r="S16" s="516">
-        <f>'BUDGET CORCOVADO 3'!$D$19*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$19*S8</f>
         <v>0</v>
       </c>
       <c r="T16" s="516">
-        <f>'BUDGET CORCOVADO 3+1'!$D$19*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$D$19*T8</f>
         <v>0</v>
       </c>
       <c r="U16" s="516">
-        <f>'BUDGET CORCOVADO 3+2'!$D$19*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$D$19*U8</f>
         <v>0</v>
       </c>
       <c r="V16" s="516">
-        <f>'BUDGET CORCOVADO 4'!$D$19*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W16" s="517">
-        <f>'BUDGET CORCOVADO 4+1'!$D$19*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$19*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W16" s="516">
+        <f>'BUDGET CORCOVADO 4'!$D$19*W8</f>
         <v>0</v>
       </c>
       <c r="X16" s="517">
-        <f>'BUDGET CORCOVADO 5'!$D$19*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$19*X8</f>
         <v>0</v>
       </c>
       <c r="Y16" s="517">
-        <f>'BUDGET NIRE 2+2'!$D$19*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$19*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -55076,48 +55076,48 @@
         <f>'BUDGET NIRE 2+1'!$D$20*H8</f>
         <v>0</v>
       </c>
-      <c r="I17" s="519">
-        <f>'BUDGET CHAITEN 1'!$D$20*I8</f>
+      <c r="I17" s="520">
+        <f>'BUDGET NIRE 2+2'!$D$20*I8</f>
         <v>0</v>
       </c>
       <c r="J17" s="519">
-        <f>'BUDGET CHAITEN 2'!$D$20*J8</f>
-        <v>0</v>
-      </c>
-      <c r="K17" s="520">
-        <f>'BUDGET CHAITEN 3'!$D$20*K8</f>
-        <v>0</v>
-      </c>
-      <c r="L17" s="519">
-        <f>'BUDGET CHAITEN 2+1'!$D$20*L8</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="520">
-        <f>'BUDGET CHAITEN 2+2'!$D$20*M8</f>
-        <v>0</v>
-      </c>
-      <c r="N17" s="519">
-        <f>'BUDGET CORCOVADO 1'!$D$20*N8</f>
+        <f>'BUDGET CHAITEN 1'!$D$20*J8</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="519">
+        <f>'BUDGET CHAITEN 2'!$D$20*K8</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="520">
+        <f>'BUDGET CHAITEN 3'!$D$20*L8</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="519">
+        <f>'BUDGET CHAITEN 2+1'!$D$20*M8</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="520">
+        <f>'BUDGET CHAITEN 2+2'!$D$20*N8</f>
         <v>0</v>
       </c>
       <c r="O17" s="519">
-        <f>'BUDGET CORCOVADO 2'!$D$20*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$D$20*O8</f>
         <v>0</v>
       </c>
       <c r="P17" s="519">
-        <f>'BUDGET CORCOVADO 2+1'!$D$20*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$20*P8</f>
         <v>0</v>
       </c>
       <c r="Q17" s="519">
-        <f>'BUDGET CORCOVADO 2+2'!$D$20*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$D$20*Q8</f>
         <v>0</v>
       </c>
       <c r="R17" s="519">
-        <f>'BUDGET CORCOVADO 2+3'!$D$20*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$D$20*R8</f>
         <v>0</v>
       </c>
       <c r="S17" s="519">
-        <f>'BUDGET CORCOVADO 2'!$D$20*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$D$20*S8</f>
         <v>0</v>
       </c>
       <c r="T17" s="519">
@@ -55125,23 +55125,23 @@
         <v>0</v>
       </c>
       <c r="U17" s="519">
-        <f>'BUDGET CORCOVADO 3+2'!$D$20*U8</f>
+        <f>'BUDGET CORCOVADO 2'!$D$20*U8</f>
         <v>0</v>
       </c>
       <c r="V17" s="519">
-        <f>'BUDGET CORCOVADO 2'!$D$20*V8</f>
-        <v>0</v>
-      </c>
-      <c r="W17" s="520">
-        <f>'BUDGET CORCOVADO 4+1'!$D$20*W8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$D$20*V8</f>
+        <v>0</v>
+      </c>
+      <c r="W17" s="519">
+        <f>'BUDGET CORCOVADO 2'!$D$20*W8</f>
         <v>0</v>
       </c>
       <c r="X17" s="520">
-        <f>'BUDGET CORCOVADO 5'!$D$20*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$D$20*X8</f>
         <v>0</v>
       </c>
       <c r="Y17" s="520">
-        <f>'BUDGET NIRE 2+2'!$D$20*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$D$20*Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -55153,12 +55153,12 @@
       <c r="F18" s="522"/>
       <c r="G18" s="522"/>
       <c r="H18" s="523"/>
-      <c r="I18" s="522"/>
+      <c r="I18" s="523"/>
       <c r="J18" s="522"/>
-      <c r="K18" s="523"/>
-      <c r="L18" s="522"/>
-      <c r="M18" s="523"/>
-      <c r="N18" s="522"/>
+      <c r="K18" s="522"/>
+      <c r="L18" s="523"/>
+      <c r="M18" s="522"/>
+      <c r="N18" s="523"/>
       <c r="O18" s="522"/>
       <c r="P18" s="522"/>
       <c r="Q18" s="522"/>
@@ -55167,7 +55167,7 @@
       <c r="T18" s="522"/>
       <c r="U18" s="522"/>
       <c r="V18" s="522"/>
-      <c r="W18" s="523"/>
+      <c r="W18" s="522"/>
       <c r="X18" s="523"/>
       <c r="Y18" s="523"/>
     </row>
@@ -55176,7 +55176,7 @@
         <v>23</v>
       </c>
       <c r="C19" s="135">
-        <f t="shared" ref="C19:X19" si="0">SUM(C10:C17)</f>
+        <f t="shared" ref="C19:Y19" si="0">SUM(C10:C17)</f>
         <v>0</v>
       </c>
       <c r="D19" s="135">
@@ -55199,27 +55199,27 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I19" s="135">
-        <f t="shared" si="0"/>
+      <c r="I19" s="525">
+        <f>SUM(I10:I17)</f>
         <v>0</v>
       </c>
       <c r="J19" s="135">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K19" s="525">
+      <c r="K19" s="135">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L19" s="135">
+      <c r="L19" s="525">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M19" s="525">
+      <c r="M19" s="135">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N19" s="135">
+      <c r="N19" s="525">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -55255,7 +55255,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="W19" s="525">
+      <c r="W19" s="135">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -55264,7 +55264,7 @@
         <v>0</v>
       </c>
       <c r="Y19" s="525">
-        <f>SUM(Y10:Y17)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -55273,7 +55273,7 @@
         <v>24</v>
       </c>
       <c r="C20" s="528">
-        <f t="shared" ref="C20:X20" si="1">C19*0.05</f>
+        <f t="shared" ref="C20:Y20" si="1">C19*0.05</f>
         <v>0</v>
       </c>
       <c r="D20" s="528">
@@ -55296,27 +55296,27 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I20" s="528">
-        <f t="shared" si="1"/>
+      <c r="I20" s="529">
+        <f>I19*0.05</f>
         <v>0</v>
       </c>
       <c r="J20" s="528">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K20" s="529">
+      <c r="K20" s="528">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L20" s="528">
+      <c r="L20" s="529">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="M20" s="529">
+      <c r="M20" s="528">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N20" s="528">
+      <c r="N20" s="529">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -55352,7 +55352,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="W20" s="529">
+      <c r="W20" s="528">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -55361,7 +55361,7 @@
         <v>0</v>
       </c>
       <c r="Y20" s="529">
-        <f>Y19*0.05</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -55370,7 +55370,7 @@
         <v>25</v>
       </c>
       <c r="C21" s="531">
-        <f t="shared" ref="C21:X21" si="2">C19-C20</f>
+        <f t="shared" ref="C21:Y21" si="2">C19-C20</f>
         <v>0</v>
       </c>
       <c r="D21" s="531">
@@ -55393,27 +55393,27 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I21" s="531">
-        <f t="shared" si="2"/>
+      <c r="I21" s="532">
+        <f>I19-I20</f>
         <v>0</v>
       </c>
       <c r="J21" s="531">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K21" s="532">
+      <c r="K21" s="531">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L21" s="531">
+      <c r="L21" s="532">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M21" s="532">
+      <c r="M21" s="531">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="N21" s="531">
+      <c r="N21" s="532">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -55449,7 +55449,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="W21" s="532">
+      <c r="W21" s="531">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -55458,7 +55458,7 @@
         <v>0</v>
       </c>
       <c r="Y21" s="532">
-        <f>Y19-Y20</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -55470,12 +55470,12 @@
       <c r="F22" s="534"/>
       <c r="G22" s="534"/>
       <c r="H22" s="535"/>
-      <c r="I22" s="534"/>
+      <c r="I22" s="535"/>
       <c r="J22" s="534"/>
-      <c r="K22" s="535"/>
-      <c r="L22" s="534"/>
-      <c r="M22" s="535"/>
-      <c r="N22" s="534"/>
+      <c r="K22" s="534"/>
+      <c r="L22" s="535"/>
+      <c r="M22" s="534"/>
+      <c r="N22" s="535"/>
       <c r="O22" s="534"/>
       <c r="P22" s="534"/>
       <c r="Q22" s="534"/>
@@ -55484,7 +55484,7 @@
       <c r="T22" s="534"/>
       <c r="U22" s="534"/>
       <c r="V22" s="534"/>
-      <c r="W22" s="535"/>
+      <c r="W22" s="534"/>
       <c r="X22" s="535"/>
       <c r="Y22" s="535"/>
     </row>
@@ -55501,12 +55501,12 @@
       <c r="F23" s="362"/>
       <c r="G23" s="362"/>
       <c r="H23" s="538"/>
-      <c r="I23" s="362"/>
+      <c r="I23" s="538"/>
       <c r="J23" s="362"/>
       <c r="K23" s="362"/>
       <c r="L23" s="362"/>
-      <c r="M23" s="538"/>
-      <c r="N23" s="362"/>
+      <c r="M23" s="362"/>
+      <c r="N23" s="538"/>
       <c r="O23" s="362"/>
       <c r="P23" s="362"/>
       <c r="Q23" s="362"/>
@@ -55517,7 +55517,7 @@
       <c r="V23" s="362"/>
       <c r="W23" s="362"/>
       <c r="X23" s="362"/>
-      <c r="Y23" s="538"/>
+      <c r="Y23" s="362"/>
     </row>
     <row r="24" spans="2:24" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="B24" s="539" t="s">
@@ -55532,12 +55532,12 @@
       <c r="F24" s="362"/>
       <c r="G24" s="362"/>
       <c r="H24" s="538"/>
-      <c r="I24" s="362"/>
+      <c r="I24" s="538"/>
       <c r="J24" s="362"/>
       <c r="K24" s="362"/>
       <c r="L24" s="362"/>
-      <c r="M24" s="538"/>
-      <c r="N24" s="362"/>
+      <c r="M24" s="362"/>
+      <c r="N24" s="538"/>
       <c r="O24" s="362"/>
       <c r="P24" s="362"/>
       <c r="Q24" s="362"/>
@@ -55548,14 +55548,14 @@
       <c r="V24" s="362"/>
       <c r="W24" s="362"/>
       <c r="X24" s="362"/>
-      <c r="Y24" s="538"/>
+      <c r="Y24" s="362"/>
     </row>
     <row r="25" spans="2:24" s="489" customFormat="1" ht="48" customHeight="1">
       <c r="B25" s="540" t="s">
         <v>28</v>
       </c>
       <c r="C25" s="541">
-        <f t="shared" ref="C25:X25" si="3">C21+(C21*$C$23)</f>
+        <f t="shared" ref="C25:Y25" si="3">C21+(C21*$C$23)</f>
         <v>0</v>
       </c>
       <c r="D25" s="541">
@@ -55578,27 +55578,27 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I25" s="541">
-        <f t="shared" si="3"/>
+      <c r="I25" s="542">
+        <f>I21+(I21*$C$23)</f>
         <v>0</v>
       </c>
       <c r="J25" s="541">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K25" s="542">
+      <c r="K25" s="541">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L25" s="541">
+      <c r="L25" s="542">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M25" s="542">
+      <c r="M25" s="541">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="N25" s="541">
+      <c r="N25" s="542">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -55634,7 +55634,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="W25" s="542">
+      <c r="W25" s="541">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -55643,7 +55643,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="542">
-        <f>Y21+(Y21*$C$23)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -55652,7 +55652,7 @@
         <v>29</v>
       </c>
       <c r="C26" s="104">
-        <f t="shared" ref="C26:X26" si="4">C25+(C25*$C$24)</f>
+        <f t="shared" ref="C26:Y26" si="4">C25+(C25*$C$24)</f>
         <v>0</v>
       </c>
       <c r="D26" s="104">
@@ -55675,27 +55675,27 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I26" s="104">
-        <f t="shared" si="4"/>
+      <c r="I26" s="544">
+        <f>I25+(I25*$C$24)</f>
         <v>0</v>
       </c>
       <c r="J26" s="104">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K26" s="544">
+      <c r="K26" s="104">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L26" s="104">
+      <c r="L26" s="544">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="M26" s="544">
+      <c r="M26" s="104">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N26" s="104">
+      <c r="N26" s="544">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -55731,7 +55731,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="W26" s="544">
+      <c r="W26" s="104">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -55740,7 +55740,7 @@
         <v>0</v>
       </c>
       <c r="Y26" s="544">
-        <f>Y25+(Y25*$C$24)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -55749,7 +55749,7 @@
         <v>30</v>
       </c>
       <c r="C27" s="546">
-        <f t="shared" ref="C27:X27" si="5">C26-C19</f>
+        <f t="shared" ref="C27:Y27" si="5">C26-C19</f>
         <v>0</v>
       </c>
       <c r="D27" s="546">
@@ -55772,27 +55772,27 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I27" s="546">
-        <f t="shared" si="5"/>
+      <c r="I27" s="547">
+        <f>I26-I19</f>
         <v>0</v>
       </c>
       <c r="J27" s="546">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="K27" s="547">
+      <c r="K27" s="546">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L27" s="546">
+      <c r="L27" s="547">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="M27" s="547">
+      <c r="M27" s="546">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N27" s="546">
+      <c r="N27" s="547">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -55828,7 +55828,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="W27" s="547">
+      <c r="W27" s="546">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -55837,7 +55837,7 @@
         <v>0</v>
       </c>
       <c r="Y27" s="547">
-        <f>Y26-Y19</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -55847,7 +55847,7 @@
         <v>31</v>
       </c>
       <c r="C29" s="135">
-        <f t="shared" ref="C29:X29" si="6">C19/C6</f>
+        <f t="shared" ref="C29:Y29" si="6">C19/C6</f>
         <v>0</v>
       </c>
       <c r="D29" s="135">
@@ -55870,27 +55870,27 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I29" s="135">
-        <f t="shared" si="6"/>
+      <c r="I29" s="525">
+        <f>I19/I6</f>
         <v>0</v>
       </c>
       <c r="J29" s="135">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="K29" s="525">
+      <c r="K29" s="135">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L29" s="135">
+      <c r="L29" s="525">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="M29" s="525">
+      <c r="M29" s="135">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="N29" s="135">
+      <c r="N29" s="525">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -55926,7 +55926,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="W29" s="525">
+      <c r="W29" s="135">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -55935,7 +55935,7 @@
         <v>0</v>
       </c>
       <c r="Y29" s="525">
-        <f>Y19/Y6</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -55944,7 +55944,7 @@
         <v>32</v>
       </c>
       <c r="C30" s="104">
-        <f t="shared" ref="C30:X30" si="7">C29+(C29*C28)</f>
+        <f t="shared" ref="C30:Y30" si="7">C29+(C29*C28)</f>
         <v>0</v>
       </c>
       <c r="D30" s="104">
@@ -55967,27 +55967,27 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I30" s="104">
-        <f t="shared" si="7"/>
+      <c r="I30" s="544">
+        <f>I29+(I29*I28)</f>
         <v>0</v>
       </c>
       <c r="J30" s="104">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="K30" s="544">
+      <c r="K30" s="104">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="L30" s="104">
+      <c r="L30" s="544">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="M30" s="544">
+      <c r="M30" s="104">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="N30" s="104">
+      <c r="N30" s="544">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -56023,7 +56023,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="W30" s="544">
+      <c r="W30" s="104">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -56032,7 +56032,7 @@
         <v>0</v>
       </c>
       <c r="Y30" s="544">
-        <f>Y29+(Y29*Y28)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -56041,7 +56041,7 @@
         <v>33</v>
       </c>
       <c r="C31" s="546">
-        <f t="shared" ref="C31:X31" si="8">C30-C24</f>
+        <f t="shared" ref="C31:Y31" si="8">C30-C24</f>
         <v>-0.04</v>
       </c>
       <c r="D31" s="546">
@@ -56064,27 +56064,27 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I31" s="546">
-        <f t="shared" si="8"/>
+      <c r="I31" s="547">
+        <f>I30-I24</f>
         <v>0</v>
       </c>
       <c r="J31" s="546">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="K31" s="547">
+      <c r="K31" s="546">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="L31" s="546">
+      <c r="L31" s="547">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="M31" s="547">
+      <c r="M31" s="546">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="N31" s="546">
+      <c r="N31" s="547">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -56120,7 +56120,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="W31" s="547">
+      <c r="W31" s="546">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -56129,7 +56129,7 @@
         <v>0</v>
       </c>
       <c r="Y31" s="547">
-        <f>Y30-Y24</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -56140,9 +56140,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="2:24" ht="20" customHeight="1">
-      <c r="O35" s="102"/>
-    </row>
+    <row r="35" spans="2:24" ht="20" customHeight="1"/>
     <row r="36" spans="2:24" ht="20" customHeight="1"/>
     <row r="37" spans="2:24" ht="20" customHeight="1"/>
     <row r="38" spans="2:24" ht="20" customHeight="1" thickBot="1"/>
@@ -56174,63 +56172,63 @@
         <f>SUM('BUDGET NIRE 2+1'!G14:G19)</f>
         <v>0</v>
       </c>
-      <c r="I39" s="550">
-        <f t="array" ref="I39:I40">'BUDGET CHAITEN 1'!G20:G21</f>
-        <v>0</v>
-      </c>
       <c r="J39" s="550">
-        <f t="array" ref="J39:J40">'BUDGET CHAITEN 2'!G20:G21</f>
-        <v>0</v>
-      </c>
-      <c r="L39" s="550">
-        <f t="array" ref="L39:L40">'BUDGET CHAITEN 2+1'!G20:G21</f>
-        <v>0</v>
-      </c>
-      <c r="M39" s="551" t="e">
+        <f t="array" ref="J39:J40">'BUDGET CHAITEN 1'!G20:G21</f>
+        <v>0</v>
+      </c>
+      <c r="K39" s="550">
+        <f t="array" ref="K39:K40">'BUDGET CHAITEN 2'!G20:G21</f>
+        <v>0</v>
+      </c>
+      <c r="M39" s="550">
+        <f t="array" ref="M39:M40">'BUDGET CHAITEN 2+1'!G20:G21</f>
+        <v>0</v>
+      </c>
+      <c r="N39" s="551" t="e">
         <f>SUM('BUDGET CHAITEN 2+2'!#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="N39" s="550">
-        <f t="array" ref="N39:N40">'BUDGET CORCOVADO 1'!G20:G21</f>
-        <v>0</v>
-      </c>
       <c r="O39" s="550">
-        <f t="array" ref="O39:O40">'BUDGET CORCOVADO 2'!G20:G21</f>
+        <f t="array" ref="O39:O40">'BUDGET CORCOVADO 1'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="P39" s="550">
-        <f t="array" ref="P39:P40">'BUDGET CORCOVADO 2+1'!G20:G21</f>
+        <f t="array" ref="P39:P40">'BUDGET CORCOVADO 2'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="Q39" s="550">
-        <f t="array" ref="Q39:Q40">'BUDGET CORCOVADO 2+2'!G20:G21</f>
+        <f t="array" ref="Q39:Q40">'BUDGET CORCOVADO 2+1'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="R39" s="550">
-        <f t="array" ref="R39:R40">'BUDGET CORCOVADO 2+3'!G20:G21</f>
+        <f t="array" ref="R39:R40">'BUDGET CORCOVADO 2+2'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="S39" s="550">
-        <f t="array" ref="S39:S40">'BUDGET CORCOVADO 3'!G20:G21</f>
+        <f t="array" ref="S39:S40">'BUDGET CORCOVADO 2+3'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="T39" s="550">
-        <f t="array" ref="T39:T40">'BUDGET CORCOVADO 3+1'!G20:G21</f>
+        <f t="array" ref="T39:T40">'BUDGET CORCOVADO 3'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="U39" s="550">
-        <f t="array" ref="U39:U40">'BUDGET CORCOVADO 3+2'!G20:G21</f>
+        <f t="array" ref="U39:U40">'BUDGET CORCOVADO 3+1'!G20:G21</f>
         <v>0</v>
       </c>
       <c r="V39" s="550">
-        <f t="array" ref="V39:V40">'BUDGET CORCOVADO 4'!G20:G21</f>
-        <v>0</v>
-      </c>
-      <c r="W39" s="551">
+        <f t="array" ref="V39:V40">'BUDGET CORCOVADO 3+2'!G20:G21</f>
+        <v>0</v>
+      </c>
+      <c r="W39" s="550">
+        <f t="array" ref="W39:W40">'BUDGET CORCOVADO 4'!G20:G21</f>
+        <v>0</v>
+      </c>
+      <c r="X39" s="551">
         <f>SUM('BUDGET CORCOVADO 4+1'!G14:G19)</f>
         <v>0</v>
       </c>
-      <c r="X39" s="551">
+      <c r="Y39" s="551">
         <f>SUM('BUDGET CORCOVADO 5'!G14:G19)</f>
         <v>0</v>
       </c>
@@ -56246,19 +56244,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="552"/>
-      <c r="I40" s="7">
-        <v>0</v>
-      </c>
       <c r="J40" s="7">
         <v>0</v>
       </c>
-      <c r="L40" s="7">
-        <v>0</v>
-      </c>
-      <c r="M40" s="552"/>
-      <c r="N40" s="7">
-        <v>0</v>
-      </c>
+      <c r="K40" s="7">
+        <v>0</v>
+      </c>
+      <c r="M40" s="7">
+        <v>0</v>
+      </c>
+      <c r="N40" s="552"/>
       <c r="O40" s="7">
         <v>0</v>
       </c>
@@ -56283,8 +56278,11 @@
       <c r="V40" s="7">
         <v>0</v>
       </c>
-      <c r="W40" s="552"/>
+      <c r="W40" s="7">
+        <v>0</v>
+      </c>
       <c r="X40" s="552"/>
+      <c r="Y40" s="552"/>
     </row>
     <row r="41" spans="2:24" ht="25" customHeight="1">
       <c r="B41" s="553" t="s">
@@ -56314,63 +56312,63 @@
         <f>'BUDGET NIRE 2+1'!G14</f>
         <v>0</v>
       </c>
-      <c r="I41" s="190">
+      <c r="J41" s="190">
         <f>'BUDGET CHAITEN 1'!G14</f>
         <v>0</v>
       </c>
-      <c r="J41" s="190">
+      <c r="K41" s="190">
         <f>'BUDGET CHAITEN 2'!G14</f>
         <v>0</v>
       </c>
-      <c r="L41" s="190">
+      <c r="M41" s="190">
         <f>'BUDGET CHAITEN 2+1'!G14</f>
         <v>0</v>
       </c>
-      <c r="M41" s="554" t="e">
+      <c r="N41" s="554" t="e">
         <f>'BUDGET CHAITEN 2+2'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="N41" s="190">
+      <c r="O41" s="190">
         <f>'BUDGET CORCOVADO 1'!G14</f>
         <v>0</v>
       </c>
-      <c r="O41" s="190">
+      <c r="P41" s="190">
         <f>'BUDGET CORCOVADO 2'!G14</f>
         <v>0</v>
       </c>
-      <c r="P41" s="190">
+      <c r="Q41" s="190">
         <f>'BUDGET CORCOVADO 2+1'!G14</f>
         <v>0</v>
       </c>
-      <c r="Q41" s="190">
+      <c r="R41" s="190">
         <f>'BUDGET CORCOVADO 2+2'!G14</f>
         <v>0</v>
       </c>
-      <c r="R41" s="190">
+      <c r="S41" s="190">
         <f>'BUDGET CORCOVADO 2+3'!G14</f>
         <v>0</v>
       </c>
-      <c r="S41" s="190">
+      <c r="T41" s="190">
         <f>'BUDGET CORCOVADO 3'!G14</f>
         <v>0</v>
       </c>
-      <c r="T41" s="190">
+      <c r="U41" s="190">
         <f>'BUDGET CORCOVADO 3+1'!G14</f>
         <v>0</v>
       </c>
-      <c r="U41" s="190">
+      <c r="V41" s="190">
         <f>'BUDGET CORCOVADO 3+2'!G14</f>
         <v>0</v>
       </c>
-      <c r="V41" s="190">
+      <c r="W41" s="190">
         <f>'BUDGET CORCOVADO 4'!G14</f>
         <v>0</v>
       </c>
-      <c r="W41" s="554">
+      <c r="X41" s="554">
         <f>'BUDGET CORCOVADO 4+1'!G14</f>
         <v>0</v>
       </c>
-      <c r="X41" s="554">
+      <c r="Y41" s="554">
         <f>'BUDGET CORCOVADO 5'!G14</f>
         <v>0</v>
       </c>
@@ -56403,63 +56401,63 @@
         <f>'BUDGET NIRE 2+1'!G15</f>
         <v>0</v>
       </c>
-      <c r="I42" s="190">
+      <c r="J42" s="190">
         <f>'BUDGET CHAITEN 1'!G15</f>
         <v>0</v>
       </c>
-      <c r="J42" s="190">
+      <c r="K42" s="190">
         <f>'BUDGET CHAITEN 2'!G15</f>
         <v>0</v>
       </c>
-      <c r="L42" s="190">
+      <c r="M42" s="190">
         <f>'BUDGET CHAITEN 2+1'!G15</f>
         <v>0</v>
       </c>
-      <c r="M42" s="554" t="e">
+      <c r="N42" s="554" t="e">
         <f>'BUDGET CHAITEN 2+2'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="N42" s="190">
+      <c r="O42" s="190">
         <f>'BUDGET CORCOVADO 1'!G15</f>
         <v>0</v>
       </c>
-      <c r="O42" s="190">
+      <c r="P42" s="190">
         <f>'BUDGET CORCOVADO 2'!G15</f>
         <v>0</v>
       </c>
-      <c r="P42" s="190">
+      <c r="Q42" s="190">
         <f>'BUDGET CORCOVADO 2+1'!G15</f>
         <v>0</v>
       </c>
-      <c r="Q42" s="190">
+      <c r="R42" s="190">
         <f>'BUDGET CORCOVADO 2+2'!G15</f>
         <v>0</v>
       </c>
-      <c r="R42" s="190">
+      <c r="S42" s="190">
         <f>'BUDGET CORCOVADO 2+3'!G15</f>
         <v>0</v>
       </c>
-      <c r="S42" s="190">
+      <c r="T42" s="190">
         <f>'BUDGET CORCOVADO 3'!G15</f>
         <v>0</v>
       </c>
-      <c r="T42" s="190">
+      <c r="U42" s="190">
         <f>'BUDGET CORCOVADO 3+1'!G15</f>
         <v>0</v>
       </c>
-      <c r="U42" s="190">
+      <c r="V42" s="190">
         <f>'BUDGET CORCOVADO 3+2'!G15</f>
         <v>0</v>
       </c>
-      <c r="V42" s="190">
+      <c r="W42" s="190">
         <f>'BUDGET CORCOVADO 4'!G15</f>
         <v>0</v>
       </c>
-      <c r="W42" s="554">
+      <c r="X42" s="554">
         <f>'BUDGET CORCOVADO 4+1'!G15</f>
         <v>0</v>
       </c>
-      <c r="X42" s="554">
+      <c r="Y42" s="554">
         <f>'BUDGET CORCOVADO 5'!G15</f>
         <v>0</v>
       </c>
@@ -56492,63 +56490,63 @@
         <f>'BUDGET NIRE 2+1'!G16</f>
         <v>0</v>
       </c>
-      <c r="I43" s="190">
+      <c r="J43" s="190">
         <f>'BUDGET CHAITEN 1'!G16</f>
         <v>0</v>
       </c>
-      <c r="J43" s="190">
+      <c r="K43" s="190">
         <f>'BUDGET CHAITEN 2'!G16</f>
         <v>0</v>
       </c>
-      <c r="L43" s="190">
+      <c r="M43" s="190">
         <f>'BUDGET CHAITEN 2+1'!G16</f>
         <v>0</v>
       </c>
-      <c r="M43" s="554" t="e">
+      <c r="N43" s="554" t="e">
         <f>'BUDGET CHAITEN 2+2'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="N43" s="190">
+      <c r="O43" s="190">
         <f>'BUDGET CORCOVADO 1'!G16</f>
         <v>0</v>
       </c>
-      <c r="O43" s="190">
+      <c r="P43" s="190">
         <f>'BUDGET CORCOVADO 2'!G16</f>
         <v>0</v>
       </c>
-      <c r="P43" s="190">
+      <c r="Q43" s="190">
         <f>'BUDGET CORCOVADO 2+1'!G16</f>
         <v>0</v>
       </c>
-      <c r="Q43" s="190">
+      <c r="R43" s="190">
         <f>'BUDGET CORCOVADO 2+2'!G16</f>
         <v>0</v>
       </c>
-      <c r="R43" s="190">
+      <c r="S43" s="190">
         <f>'BUDGET CORCOVADO 2+3'!G16</f>
         <v>0</v>
       </c>
-      <c r="S43" s="190">
+      <c r="T43" s="190">
         <f>'BUDGET CORCOVADO 3'!G16</f>
         <v>0</v>
       </c>
-      <c r="T43" s="190">
+      <c r="U43" s="190">
         <f>'BUDGET CORCOVADO 3+1'!G16</f>
         <v>0</v>
       </c>
-      <c r="U43" s="190">
+      <c r="V43" s="190">
         <f>'BUDGET CORCOVADO 3+2'!G16</f>
         <v>0</v>
       </c>
-      <c r="V43" s="190">
+      <c r="W43" s="190">
         <f>'BUDGET CORCOVADO 4'!G16</f>
         <v>0</v>
       </c>
-      <c r="W43" s="554">
+      <c r="X43" s="554">
         <f>'BUDGET CORCOVADO 4+1'!G16</f>
         <v>0</v>
       </c>
-      <c r="X43" s="554">
+      <c r="Y43" s="554">
         <f>'BUDGET CORCOVADO 5'!G16</f>
         <v>0</v>
       </c>
@@ -56581,63 +56579,63 @@
         <f>'BUDGET NIRE 2+1'!G17</f>
         <v>0</v>
       </c>
-      <c r="I44" s="190">
+      <c r="J44" s="190">
         <f>'BUDGET CHAITEN 1'!G17</f>
         <v>0</v>
       </c>
-      <c r="J44" s="190">
+      <c r="K44" s="190">
         <f>'BUDGET CHAITEN 2'!G17</f>
         <v>0</v>
       </c>
-      <c r="L44" s="190">
+      <c r="M44" s="190">
         <f>'BUDGET CHAITEN 2+1'!G17</f>
         <v>0</v>
       </c>
-      <c r="M44" s="554" t="e">
+      <c r="N44" s="554" t="e">
         <f>'BUDGET CHAITEN 2+2'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="N44" s="190">
+      <c r="O44" s="190">
         <f>'BUDGET CORCOVADO 1'!G17</f>
         <v>0</v>
       </c>
-      <c r="O44" s="190">
+      <c r="P44" s="190">
         <f>'BUDGET CORCOVADO 2'!G17</f>
         <v>0</v>
       </c>
-      <c r="P44" s="190">
+      <c r="Q44" s="190">
         <f>'BUDGET CORCOVADO 2+1'!G17</f>
         <v>0</v>
       </c>
-      <c r="Q44" s="190">
+      <c r="R44" s="190">
         <f>'BUDGET CORCOVADO 2+2'!G17</f>
         <v>0</v>
       </c>
-      <c r="R44" s="190">
+      <c r="S44" s="190">
         <f>'BUDGET CORCOVADO 2+3'!G17</f>
         <v>0</v>
       </c>
-      <c r="S44" s="190">
+      <c r="T44" s="190">
         <f>'BUDGET CORCOVADO 3'!G17</f>
         <v>0</v>
       </c>
-      <c r="T44" s="190">
+      <c r="U44" s="190">
         <f>'BUDGET CORCOVADO 3+1'!G17</f>
         <v>0</v>
       </c>
-      <c r="U44" s="190">
+      <c r="V44" s="190">
         <f>'BUDGET CORCOVADO 3+2'!G17</f>
         <v>0</v>
       </c>
-      <c r="V44" s="190">
+      <c r="W44" s="190">
         <f>'BUDGET CORCOVADO 4'!G17</f>
         <v>0</v>
       </c>
-      <c r="W44" s="554">
+      <c r="X44" s="554">
         <f>'BUDGET CORCOVADO 4+1'!G17</f>
         <v>0</v>
       </c>
-      <c r="X44" s="554">
+      <c r="Y44" s="554">
         <f>'BUDGET CORCOVADO 5'!G17</f>
         <v>0</v>
       </c>
@@ -56670,63 +56668,63 @@
         <f>'BUDGET NIRE 2+1'!G18</f>
         <v>0</v>
       </c>
-      <c r="I45" s="190">
+      <c r="J45" s="190">
         <f>'BUDGET CHAITEN 1'!G18</f>
         <v>0</v>
       </c>
-      <c r="J45" s="190">
+      <c r="K45" s="190">
         <f>'BUDGET CHAITEN 2'!G18</f>
         <v>0</v>
       </c>
-      <c r="L45" s="190">
+      <c r="M45" s="190">
         <f>'BUDGET CHAITEN 2+1'!G18</f>
         <v>0</v>
       </c>
-      <c r="M45" s="554" t="e">
+      <c r="N45" s="554" t="e">
         <f>'BUDGET CHAITEN 2+2'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="N45" s="190">
+      <c r="O45" s="190">
         <f>'BUDGET CORCOVADO 1'!G18</f>
         <v>0</v>
       </c>
-      <c r="O45" s="190">
+      <c r="P45" s="190">
         <f>'BUDGET CORCOVADO 2'!G18</f>
         <v>0</v>
       </c>
-      <c r="P45" s="190">
+      <c r="Q45" s="190">
         <f>'BUDGET CORCOVADO 2+1'!G18</f>
         <v>0</v>
       </c>
-      <c r="Q45" s="190">
+      <c r="R45" s="190">
         <f>'BUDGET CORCOVADO 2+2'!G18</f>
         <v>0</v>
       </c>
-      <c r="R45" s="190">
+      <c r="S45" s="190">
         <f>'BUDGET CORCOVADO 2+3'!G18</f>
         <v>0</v>
       </c>
-      <c r="S45" s="190">
+      <c r="T45" s="190">
         <f>'BUDGET CORCOVADO 3'!G18</f>
         <v>0</v>
       </c>
-      <c r="T45" s="190">
+      <c r="U45" s="190">
         <f>'BUDGET CORCOVADO 3+1'!G18</f>
         <v>0</v>
       </c>
-      <c r="U45" s="190">
+      <c r="V45" s="190">
         <f>'BUDGET CORCOVADO 3+2'!G18</f>
         <v>0</v>
       </c>
-      <c r="V45" s="190">
+      <c r="W45" s="190">
         <f>'BUDGET CORCOVADO 4'!G18</f>
         <v>0</v>
       </c>
-      <c r="W45" s="554">
+      <c r="X45" s="554">
         <f>'BUDGET CORCOVADO 4+1'!G18</f>
         <v>0</v>
       </c>
-      <c r="X45" s="554">
+      <c r="Y45" s="554">
         <f>'BUDGET CORCOVADO 5'!G18</f>
         <v>0</v>
       </c>
@@ -56759,63 +56757,63 @@
         <f>'BUDGET NIRE 2+1'!G19</f>
         <v>0</v>
       </c>
-      <c r="I46" s="190">
+      <c r="J46" s="190">
         <f>'BUDGET CHAITEN 1'!G19</f>
         <v>0</v>
       </c>
-      <c r="J46" s="190">
+      <c r="K46" s="190">
         <f>'BUDGET CHAITEN 2'!G19</f>
         <v>0</v>
       </c>
-      <c r="L46" s="190">
+      <c r="M46" s="190">
         <f>'BUDGET CHAITEN 2+1'!G19</f>
         <v>0</v>
       </c>
-      <c r="M46" s="554" t="e">
+      <c r="N46" s="554" t="e">
         <f>'BUDGET CHAITEN 2+2'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="N46" s="190">
+      <c r="O46" s="190">
         <f>'BUDGET CORCOVADO 1'!G19</f>
         <v>0</v>
       </c>
-      <c r="O46" s="190">
+      <c r="P46" s="190">
         <f>'BUDGET CORCOVADO 2'!G19</f>
         <v>0</v>
       </c>
-      <c r="P46" s="190">
+      <c r="Q46" s="190">
         <f>'BUDGET CORCOVADO 2+1'!G19</f>
         <v>0</v>
       </c>
-      <c r="Q46" s="190">
+      <c r="R46" s="190">
         <f>'BUDGET CORCOVADO 2+2'!G19</f>
         <v>0</v>
       </c>
-      <c r="R46" s="190">
+      <c r="S46" s="190">
         <f>'BUDGET CORCOVADO 2+3'!G19</f>
         <v>0</v>
       </c>
-      <c r="S46" s="190">
+      <c r="T46" s="190">
         <f>'BUDGET CORCOVADO 3'!G19</f>
         <v>0</v>
       </c>
-      <c r="T46" s="190">
+      <c r="U46" s="190">
         <f>'BUDGET CORCOVADO 3+1'!G19</f>
         <v>0</v>
       </c>
-      <c r="U46" s="190">
+      <c r="V46" s="190">
         <f>'BUDGET CORCOVADO 3+2'!G19</f>
         <v>0</v>
       </c>
-      <c r="V46" s="190">
+      <c r="W46" s="190">
         <f>'BUDGET CORCOVADO 4'!G19</f>
         <v>0</v>
       </c>
-      <c r="W46" s="554">
+      <c r="X46" s="554">
         <f>'BUDGET CORCOVADO 4+1'!G19</f>
         <v>0</v>
       </c>
-      <c r="X46" s="554">
+      <c r="Y46" s="554">
         <f>'BUDGET CORCOVADO 5'!G19</f>
         <v>0</v>
       </c>
@@ -56836,16 +56834,16 @@
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
       <c r="H55" s="7"/>
-      <c r="I55" s="7"/>
       <c r="J55" s="7"/>
-      <c r="L55" s="7"/>
+      <c r="K55" s="7"/>
       <c r="M55" s="7"/>
+      <c r="N55" s="7"/>
     </row>
     <row r="56" spans="2:13" s="10" customFormat="1" ht="42" customHeight="1">
       <c r="B56" s="9"/>
       <c r="E56" s="9"/>
       <c r="H56" s="9"/>
-      <c r="M56" s="9"/>
+      <c r="N56" s="9"/>
     </row>
     <row r="57" spans="2:13" ht="20" customHeight="1"/>
     <row r="58" spans="2:13" ht="20" customHeight="1"/>
@@ -56866,10 +56864,10 @@
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
       <c r="H68" s="7"/>
-      <c r="I68" s="7"/>
       <c r="J68" s="7"/>
-      <c r="L68" s="7"/>
+      <c r="K68" s="7"/>
       <c r="M68" s="7"/>
+      <c r="N68" s="7"/>
     </row>
     <row r="69" spans="2:13" ht="37" customHeight="1"/>
     <row r="70" spans="2:13" ht="20" customHeight="1"/>
@@ -56886,10 +56884,10 @@
       <c r="F76" s="7"/>
       <c r="G76" s="7"/>
       <c r="H76" s="7"/>
-      <c r="I76" s="7"/>
       <c r="J76" s="7"/>
-      <c r="L76" s="7"/>
+      <c r="K76" s="7"/>
       <c r="M76" s="7"/>
+      <c r="N76" s="7"/>
     </row>
     <row r="77" spans="2:13" s="9" customFormat="1" ht="42" customHeight="1"/>
     <row r="78" spans="2:13" ht="20" customHeight="1"/>
@@ -56904,10 +56902,10 @@
       <c r="F82" s="7"/>
       <c r="G82" s="7"/>
       <c r="H82" s="7"/>
-      <c r="I82" s="7"/>
       <c r="J82" s="7"/>
-      <c r="L82" s="7"/>
+      <c r="K82" s="7"/>
       <c r="M82" s="7"/>
+      <c r="N82" s="7"/>
     </row>
     <row r="83" spans="2:13" ht="38" customHeight="1"/>
     <row r="84" spans="2:13" ht="20" customHeight="1"/>
@@ -56925,10 +56923,10 @@
       <c r="F91" s="7"/>
       <c r="G91" s="7"/>
       <c r="H91" s="7"/>
-      <c r="I91" s="7"/>
       <c r="J91" s="7"/>
-      <c r="L91" s="7"/>
+      <c r="K91" s="7"/>
       <c r="M91" s="7"/>
+      <c r="N91" s="7"/>
     </row>
     <row r="92" spans="2:13" ht="38" customHeight="1"/>
     <row r="93" spans="2:13" ht="23" customHeight="1"/>
@@ -56940,18 +56938,16 @@
       <c r="F95" s="7"/>
       <c r="G95" s="7"/>
       <c r="H95" s="552"/>
-      <c r="I95" s="7"/>
       <c r="J95" s="7"/>
-      <c r="L95" s="7"/>
-      <c r="M95" s="552"/>
+      <c r="K95" s="7"/>
+      <c r="M95" s="7"/>
+      <c r="N95" s="552"/>
     </row>
     <row r="96" spans="2:13" ht="9" customHeight="1"/>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <mergeCells count="3">
+  <mergeCells count="1">
     <mergeCell ref="B5:B8"/>
-    <mergeCell ref="C7:X7"/>
-    <mergeCell ref="M3:X3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -57170,7 +57166,7 @@
       <c r="C11" s="586"/>
       <c r="D11" s="586"/>
       <c r="E11" s="587">
-        <f>('BUDGET RESUMO'!C10*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D10*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F10*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G10*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I10*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J10*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L10*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N10*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O10*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P10*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q10*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R10*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S10*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T10*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U10*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V10*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E10*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H10*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M10*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X10*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W10*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K10*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y10*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C10*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D10*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F10*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G10*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J10*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K10*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M10*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O10*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P10*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q10*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R10*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S10*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T10*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U10*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V10*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W10*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E10*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H10*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N10*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y10*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X10*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L10*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I10*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="H11" s="581"/>
@@ -57189,7 +57185,7 @@
       <c r="C13" s="590"/>
       <c r="D13" s="590"/>
       <c r="E13" s="591">
-        <f>('BUDGET RESUMO'!C11*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D11*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F11*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G11*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I11*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J11*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L11*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N11*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O11*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P11*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q11*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R11*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S11*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T11*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U11*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V11*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E11*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H11*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M11*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X11*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W11*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K11*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y11*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C11*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D11*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F11*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G11*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J11*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K11*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M11*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O11*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P11*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q11*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R11*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S11*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T11*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U11*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V11*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W11*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E11*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H11*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N11*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y11*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X11*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L11*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I11*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="G13" s="592">
@@ -57216,7 +57212,7 @@
       <c r="C15" s="599"/>
       <c r="D15" s="599"/>
       <c r="E15" s="600">
-        <f>('BUDGET RESUMO'!C12*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D12*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F12*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G12*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I12*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J12*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L12*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N12*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O12*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P12*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q12*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R12*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S12*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T12*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U12*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V12*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E12*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H12*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M12*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X12*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W12*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K12*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y12*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C12*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D12*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F12*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G12*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J12*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K12*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M12*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O12*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P12*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q12*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R12*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S12*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T12*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U12*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V12*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W12*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E12*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H12*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N12*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y12*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X12*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L12*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I12*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="H15" s="593">
@@ -57238,7 +57234,7 @@
       <c r="C17" s="606"/>
       <c r="D17" s="606"/>
       <c r="E17" s="607">
-        <f>('BUDGET RESUMO'!C13*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D13*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F13*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G13*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I13*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J13*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L13*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N13*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O13*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P13*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q13*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R13*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S13*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T13*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U13*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V13*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E13*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H13*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M13*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X13*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W13*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K13*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y13*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C13*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D13*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F13*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G13*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J13*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K13*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M13*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O13*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P13*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q13*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R13*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S13*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T13*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U13*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V13*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W13*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E13*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H13*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N13*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y13*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X13*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L13*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I13*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="H17" s="593">
@@ -57260,7 +57256,7 @@
       <c r="C19" s="609"/>
       <c r="D19" s="609"/>
       <c r="E19" s="613">
-        <f>('BUDGET RESUMO'!C14*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D14*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F14*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G14*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I14*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J14*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L14*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N14*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O14*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P14*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q14*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R14*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S14*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T14*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U14*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V14*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E14*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H14*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M14*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X14*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W14*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K14*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y14*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C14*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D14*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F14*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G14*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J14*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K14*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M14*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O14*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P14*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q14*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R14*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S14*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T14*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U14*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V14*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W14*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E14*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H14*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N14*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y14*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X14*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L14*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I14*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="H19" s="593">
@@ -57282,7 +57278,7 @@
       <c r="C21" s="618"/>
       <c r="D21" s="618"/>
       <c r="E21" s="619">
-        <f>('BUDGET RESUMO'!C15*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D15*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F15*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G15*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I15*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J15*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L15*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N15*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O15*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P15*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q15*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R15*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S15*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T15*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U15*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V15*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E15*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H15*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M15*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X15*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W15*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K15*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y15*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C15*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D15*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F15*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G15*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J15*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K15*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M15*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O15*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P15*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q15*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R15*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S15*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T15*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U15*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V15*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W15*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E15*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H15*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N15*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y15*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X15*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L15*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I15*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="H21" s="593">
@@ -57304,7 +57300,7 @@
       <c r="C23" s="624"/>
       <c r="D23" s="624"/>
       <c r="E23" s="625">
-        <f>('BUDGET RESUMO'!C16*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D16*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F16*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G16*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I16*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J16*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L16*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N16*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O16*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P16*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q16*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R16*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S16*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T16*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U16*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V16*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E16*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H16*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M16*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X16*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W16*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K16*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y16*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C16*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D16*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F16*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G16*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J16*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K16*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M16*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O16*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P16*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q16*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R16*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S16*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T16*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U16*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V16*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W16*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E16*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H16*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N16*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y16*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X16*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L16*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I16*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
       <c r="H23" s="593">
@@ -57328,7 +57324,7 @@
       <c r="C25" s="631"/>
       <c r="D25" s="631"/>
       <c r="E25" s="632">
-        <f>('BUDGET RESUMO'!C17*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D17*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F17*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G17*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!I17*'BUDGET RESUMO'!$I$8)+('BUDGET RESUMO'!J17*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!L17*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!N17*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!O17*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P17*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q17*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R17*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S17*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T17*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U17*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V17*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!E17*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H17*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!M17*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!X17*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!W17*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!K17*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!Y17*'BUDGET RESUMO'!$Y$8)</f>
+        <f>('BUDGET RESUMO'!C17*'BUDGET RESUMO'!$C$8)+('BUDGET RESUMO'!D17*'BUDGET RESUMO'!$D$8)+('BUDGET RESUMO'!F17*'BUDGET RESUMO'!$F$8)+('BUDGET RESUMO'!G17*'BUDGET RESUMO'!$G$8)+('BUDGET RESUMO'!J17*'BUDGET RESUMO'!$J$8)+('BUDGET RESUMO'!K17*'BUDGET RESUMO'!$K$8)+('BUDGET RESUMO'!M17*'BUDGET RESUMO'!$M$8)+('BUDGET RESUMO'!O17*'BUDGET RESUMO'!$O$8)+('BUDGET RESUMO'!P17*'BUDGET RESUMO'!$P$8)+('BUDGET RESUMO'!Q17*'BUDGET RESUMO'!$Q$8)+('BUDGET RESUMO'!R17*'BUDGET RESUMO'!$R$8)+('BUDGET RESUMO'!S17*'BUDGET RESUMO'!$S$8)+('BUDGET RESUMO'!T17*'BUDGET RESUMO'!$T$8)+('BUDGET RESUMO'!U17*'BUDGET RESUMO'!$U$8)+('BUDGET RESUMO'!V17*'BUDGET RESUMO'!$V$8)+('BUDGET RESUMO'!W17*'BUDGET RESUMO'!$W$8)+('BUDGET RESUMO'!E17*'BUDGET RESUMO'!$E$8)+('BUDGET RESUMO'!H17*'BUDGET RESUMO'!$H$8)+('BUDGET RESUMO'!N17*'BUDGET RESUMO'!$N$8)+('BUDGET RESUMO'!Y17*'BUDGET RESUMO'!$Y$8)+('BUDGET RESUMO'!X17*'BUDGET RESUMO'!$X$8)+('BUDGET RESUMO'!L17*'BUDGET RESUMO'!$L$8)+('BUDGET RESUMO'!I17*'BUDGET RESUMO'!$I$8)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige formato de data das celulas C2/C3 na aba CALENDAR
C2 (check-in) e C3 (check-out) estavam com formatos de numero
diferentes entre si (nenhum dos dois era formato de data), fazendo
os valores aparecerem como numeros grandes em vez de datas legiveis
e com aparencia inconsistente uma da outra. Ambas agora usam o mesmo
formato DD/MM/YYYY. O calculo de noites (J2 = C3-C2) ja estava
matematicamente correto (datas sao numeros de serie internamente),
o problema era so de exibicao.
</commit_message>
<xml_diff>
--- a/assets/templates/planilha_orcamentos_python.xlsx
+++ b/assets/templates/planilha_orcamentos_python.xlsx
@@ -690,7 +690,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="[$USD]\ #,##0.00"/>
@@ -703,6 +703,7 @@
     <numFmt numFmtId="173" formatCode="_-[$CLP]\ * #,##0_-;\-[$CLP]\ * #,##0_-;_-[$CLP]\ * &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="[$CLP]\ #,##0.00;\-[$CLP]\ #,##0.00"/>
     <numFmt numFmtId="175" formatCode="[$-409]h:mm\ AM/PM;@"/>
+    <numFmt numFmtId="176" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -1910,7 +1911,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="740">
+  <cellXfs count="742">
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4095,6 +4096,14 @@
     <xf numFmtId="0" fontId="15" fillId="35" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="8" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
@@ -4844,7 +4853,7 @@
         <v>36</v>
       </c>
       <c r="B2" s="696"/>
-      <c r="C2" s="29"/>
+      <c r="C2" s="740"/>
       <c r="D2" s="366"/>
       <c r="E2" s="366"/>
       <c r="F2" s="367"/>
@@ -4871,7 +4880,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="696"/>
-      <c r="C3" s="30"/>
+      <c r="C3" s="741"/>
       <c r="D3" s="304">
         <v>46305</v>
       </c>

</xml_diff>

<commit_message>
Restaura fórmulas vivas de preço de cabana no template, com bugs corrigidos
C24-C27 de todas as 23 abas BUDGET voltam a ser fórmula ligada ao
MAPU_PLANNER (como o ANOMESDIA_nomecliente.xlsx tentava fazer), mas
corrigindo os 2 bugs que esse arquivo tinha: inclui março na Alta
temporada e usa desconto de 5% (não 10%) para 7+ noites. Cache do link
externo atualizado com preços/taxas atuais.

Isso é redundante com o cálculo em Python (load_precos/populate_excel
sempre sobrescreve com o valor correto na hora de gerar) — mas garante
que quem abrir o template direto no Excel também veja um valor coerente
com o Planner, não um número de teste antigo parado na célula.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/planilha_orcamentos_python.xlsx
+++ b/assets/templates/planilha_orcamentos_python.xlsx
@@ -4929,6 +4929,48 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0">
+        <row r="6">
+          <cell r="B6">
+            <v>315000</v>
+          </cell>
+          <cell r="C6">
+            <v>280000</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="B7">
+            <v>340000</v>
+          </cell>
+          <cell r="C7">
+            <v>300000</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="B8">
+            <v>352000</v>
+          </cell>
+          <cell r="C8">
+            <v>320000</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="B9">
+            <v>432000</v>
+          </cell>
+          <cell r="C9">
+            <v>400000</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="B12">
+            <v>50000</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="B32">
+            <v>0.19</v>
+          </cell>
+        </row>
         <row r="16">
           <cell r="B16">
             <v>24000</v>
@@ -4951,12 +4993,12 @@
         </row>
         <row r="33">
           <cell r="B33">
-            <v>0.04</v>
+            <v>0.05</v>
           </cell>
         </row>
         <row r="34">
           <cell r="B34">
-            <v>0.15</v>
+            <v>0.2</v>
           </cell>
         </row>
       </sheetData>
@@ -6562,7 +6604,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>249200</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -6588,11 +6630,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>249200</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -6616,7 +6659,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>224280</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -6642,11 +6685,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>224280</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -9342,7 +9386,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>288190.9</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -9368,11 +9412,11 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>288190.9</f>
+        <f>C24</f>
         <v/>
       </c>
       <c r="D25" s="913">
-        <f>$B$6*50000</f>
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
         <v/>
       </c>
       <c r="E25" s="914">
@@ -9397,7 +9441,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>259371.81</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -9423,11 +9467,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>259371.81</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -12134,7 +12179,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>288190.9</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -12160,11 +12205,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>288190.9</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -12188,7 +12234,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>259371.81</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -12214,11 +12260,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>259371.81</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -14915,7 +14962,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>288190.9</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -14941,11 +14988,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>288190.9</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -14969,7 +15017,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>259371.81</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -14995,11 +15043,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>259371.81</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -17696,7 +17745,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>288190.9</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -17722,11 +17771,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>288190.9</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -17750,7 +17800,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>259371.81</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -17776,11 +17826,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>259371.81</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -20487,7 +20538,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>288190.9</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -20513,11 +20564,11 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>288190.9</f>
+        <f>C24</f>
         <v/>
       </c>
       <c r="D25" s="913">
-        <f>$B$6*50000</f>
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
         <v/>
       </c>
       <c r="E25" s="914">
@@ -20542,7 +20593,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>259371.81</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -20568,11 +20619,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>259371.81</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -23279,7 +23331,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>288190.9</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -23305,11 +23357,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>288190.9</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -23333,7 +23386,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>259371.81</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -23359,11 +23412,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>259371.81</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -26068,7 +26122,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -26094,11 +26148,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -26122,7 +26177,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -26148,11 +26203,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -28848,7 +28904,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -28874,11 +28930,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -28902,7 +28959,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -28928,11 +28985,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -31628,7 +31686,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -31654,11 +31712,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -31682,7 +31741,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -31708,11 +31767,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -36077,7 +36137,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -36103,11 +36163,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -36131,7 +36192,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -36157,11 +36218,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -38868,7 +38930,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -38894,11 +38956,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -38922,7 +38985,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -38948,11 +39011,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -41659,7 +41723,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -41685,11 +41749,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -41713,7 +41778,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -41739,11 +41804,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -44440,7 +44506,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -44466,11 +44532,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -44494,7 +44561,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -44520,11 +44587,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -47232,7 +47300,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -47258,11 +47326,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -47286,7 +47355,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -47312,11 +47381,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -50022,7 +50092,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -50048,11 +50118,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -50076,7 +50147,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -50102,11 +50173,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -52802,7 +52874,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -52828,11 +52900,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -52856,7 +52929,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -52882,11 +52955,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -55582,7 +55656,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>398381.8</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -55608,11 +55682,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>398381.8</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -55636,7 +55711,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>358543.62</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -55662,11 +55737,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>358543.62</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -62364,7 +62440,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>249200</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -62390,11 +62466,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>249200</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -62418,7 +62495,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>224280</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -62444,11 +62521,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>224280</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -65139,7 +65217,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>249200</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -65165,11 +65243,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>249200</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -65193,7 +65272,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>224280</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -65219,11 +65298,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>224280</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -67913,7 +67993,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>249200</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -67939,11 +68019,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>249200</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -67967,7 +68048,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>224280</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -67993,11 +68074,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>224280</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -70693,7 +70775,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>249200</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -70719,11 +70801,12 @@
         <v>0</v>
       </c>
       <c r="C25" s="912">
-        <f>249200</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -70747,7 +70830,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>224280</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -70773,11 +70856,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>224280</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>
@@ -73474,7 +73558,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>249200</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -73500,11 +73584,12 @@
         <v>1</v>
       </c>
       <c r="C25" s="912">
-        <f>249200</f>
-        <v/>
-      </c>
-      <c r="D25" s="913" t="n">
-        <v>50000</v>
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E25" s="914">
         <f>(C25+D25)*$B$9*B25</f>
@@ -73528,7 +73613,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="912">
-        <f>224280</f>
+        <f>C24*0.95</f>
         <v/>
       </c>
       <c r="D26" s="913" t="n"/>
@@ -73554,11 +73639,12 @@
         <v>0</v>
       </c>
       <c r="C27" s="912">
-        <f>224280</f>
-        <v/>
-      </c>
-      <c r="D27" s="913" t="n">
-        <v>50000</v>
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="913">
+        <f>'[1]⚙️ INPUTS'!$B$12</f>
+        <v/>
       </c>
       <c r="E27" s="914">
         <f>(C27+D27)*$B$9*B27</f>

</xml_diff>

<commit_message>
Corrige bug de IVA embutido indevidamente no preço da cabana
load_precos()/_extract_precos_from_workbook() estava aplicando ×(1+IVA)
no preço da cabana lido do Planner (INPUTS!B6:C9, que já é líquido).
Isso fazia todo cliente pagar como se fosse chileno, mesmo turistas
isentos — o IVA "informativo" no PDF nunca era somado de verdade
(chilean_client sempre False), mas o valor já vinha inflado 19% na
tarifa da cabana.

Correção: preço da cabana fica líquido; IVA só é aplicado (e só quando
chilean_client=True) como linha separada em calculate(), igual já
estava desenhado — o problema era só a dupla contagem na origem.
precos.json e os 4 templates (planilha_orcamentos_python.xlsx ×2,
ANOMESDIA_nomecliente.xlsx ×2) atualizados junto.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/planilha_orcamentos_python.xlsx
+++ b/assets/templates/planilha_orcamentos_python.xlsx
@@ -6604,7 +6604,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -9386,7 +9386,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -12179,7 +12179,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -14962,7 +14962,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -17745,7 +17745,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -20538,7 +20538,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -23331,7 +23331,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$8,'[1]⚙️ INPUTS'!$C$8)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -26122,7 +26122,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -28904,7 +28904,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -31686,7 +31686,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -36137,7 +36137,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -38930,7 +38930,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -41723,7 +41723,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -44506,7 +44506,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -47300,7 +47300,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -50092,7 +50092,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -52874,7 +52874,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -55656,7 +55656,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$9,'[1]⚙️ INPUTS'!$C$9)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -62440,7 +62440,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -65217,7 +65217,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -67993,7 +67993,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$6,'[1]⚙️ INPUTS'!$C$6)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -70775,7 +70775,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>
@@ -73558,7 +73558,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="912">
-        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)*(1+'[1]⚙️ INPUTS'!$B$32)</f>
+        <f>IF(OR(MONTH($B$7)=1,MONTH($B$7)=2,MONTH($B$7)=3,MONTH($B$7)=12),'[1]⚙️ INPUTS'!$B$7,'[1]⚙️ INPUTS'!$C$7)</f>
         <v/>
       </c>
       <c r="D24" s="913" t="n"/>

</xml_diff>

<commit_message>
Atualiza template fallback (assets/templates) com fixes da aba RESULTADO/BUDGET RESUMO
Fica sincronizado com o template principal (2027/template/) - cadeia de CC sem gross-up, linhas 19-27 corrigidas, taxas linkadas ao Planner.
</commit_message>
<xml_diff>
--- a/assets/templates/planilha_orcamentos_python.xlsx
+++ b/assets/templates/planilha_orcamentos_python.xlsx
@@ -1283,7 +1283,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1063">
+  <cellXfs count="1064">
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4440,6 +4440,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="171" fontId="8" fillId="30" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6207,8 +6210,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -8989,8 +8993,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -11782,8 +11787,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -14565,8 +14571,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -17348,8 +17355,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -20141,8 +20149,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -22934,8 +22943,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -25725,8 +25735,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -28507,8 +28518,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -31289,8 +31301,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -35740,8 +35753,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -38533,8 +38547,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -41326,8 +41341,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -44109,8 +44125,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -46903,8 +46920,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -49695,8 +49713,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -52477,8 +52496,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -55259,8 +55279,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -58446,95 +58467,95 @@
         </is>
       </c>
       <c r="C10" s="814">
-        <f>'BUDGET COIGUE 1'!D13*C8</f>
+        <f>'BUDGET COIGUE 1'!B13*C8</f>
         <v/>
       </c>
       <c r="D10" s="814">
-        <f>'BUDGET COIGUE 2'!$D$13*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$13*D8</f>
         <v/>
       </c>
       <c r="E10" s="814">
-        <f>'BUDGET COIGUE 2+1'!$D$13*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$13*E8</f>
         <v/>
       </c>
       <c r="F10" s="814">
-        <f>'BUDGET NIRE 1'!$D$13*F8</f>
+        <f>'BUDGET NIRE 1'!$B$13*F8</f>
         <v/>
       </c>
       <c r="G10" s="814">
-        <f>'BUDGET NIRE 2'!$D$13*G8</f>
+        <f>'BUDGET NIRE 2'!$B$13*G8</f>
         <v/>
       </c>
       <c r="H10" s="815">
-        <f>'BUDGET NIRE 2+1'!$D$13*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$13*H8</f>
         <v/>
       </c>
       <c r="I10" s="815">
-        <f>'BUDGET NIRE 2+2'!$D$13*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$13*I8</f>
         <v/>
       </c>
       <c r="J10" s="814">
-        <f>'BUDGET CHAITEN 1'!$D$13*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$13*J8</f>
         <v/>
       </c>
       <c r="K10" s="814">
-        <f>'BUDGET CHAITEN 2'!$D$13*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$13*K8</f>
         <v/>
       </c>
       <c r="L10" s="815">
-        <f>'BUDGET CHAITEN 3'!$D$13*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$13*L8</f>
         <v/>
       </c>
       <c r="M10" s="814">
-        <f>'BUDGET CHAITEN 2+1'!$D$13*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$13*M8</f>
         <v/>
       </c>
       <c r="N10" s="815">
-        <f>'BUDGET CHAITEN 2+2'!$D$13*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$13*N8</f>
         <v/>
       </c>
       <c r="O10" s="814">
-        <f>'BUDGET CORCOVADO 1'!$D$13*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$13*O8</f>
         <v/>
       </c>
       <c r="P10" s="814">
-        <f>'BUDGET CORCOVADO 2'!$D$13*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$13*P8</f>
         <v/>
       </c>
       <c r="Q10" s="814">
-        <f>'BUDGET CORCOVADO 2+1'!$D$13*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$13*Q8</f>
         <v/>
       </c>
       <c r="R10" s="814">
-        <f>'BUDGET CORCOVADO 2+2'!$D$13*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$13*R8</f>
         <v/>
       </c>
       <c r="S10" s="814">
-        <f>'BUDGET CORCOVADO 2+3'!$D$13*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$13*S8</f>
         <v/>
       </c>
       <c r="T10" s="814">
-        <f>'BUDGET CORCOVADO 3'!$D$13*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$13*T8</f>
         <v/>
       </c>
       <c r="U10" s="814">
-        <f>'BUDGET CORCOVADO 3+1'!$D$13*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$13*U8</f>
         <v/>
       </c>
       <c r="V10" s="814">
-        <f>'BUDGET CORCOVADO 3+2'!$D$13*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$13*V8</f>
         <v/>
       </c>
       <c r="W10" s="814">
-        <f>'BUDGET CORCOVADO 4'!$D$13*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$13*W8</f>
         <v/>
       </c>
       <c r="X10" s="815">
-        <f>'BUDGET CORCOVADO 4+1'!$D$13*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$13*X8</f>
         <v/>
       </c>
       <c r="Y10" s="815">
-        <f>'BUDGET CORCOVADO 5'!$D$13*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$13*Y8</f>
         <v/>
       </c>
     </row>
@@ -58545,95 +58566,95 @@
         </is>
       </c>
       <c r="C11" s="816">
-        <f>'BUDGET COIGUE 1'!$D$14*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$14*C8</f>
         <v/>
       </c>
       <c r="D11" s="816">
-        <f>'BUDGET COIGUE 2'!$D$14*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$14*D8</f>
         <v/>
       </c>
       <c r="E11" s="816">
-        <f>'BUDGET COIGUE 2+1'!$D$14*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$14*E8</f>
         <v/>
       </c>
       <c r="F11" s="816">
-        <f>'BUDGET NIRE 1'!$D$14*F8</f>
+        <f>'BUDGET NIRE 1'!$B$14*F8</f>
         <v/>
       </c>
       <c r="G11" s="816">
-        <f>'BUDGET NIRE 2'!$D$14*G8</f>
+        <f>'BUDGET NIRE 2'!$B$14*G8</f>
         <v/>
       </c>
       <c r="H11" s="817">
-        <f>'BUDGET NIRE 2+1'!$D$14*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$14*H8</f>
         <v/>
       </c>
       <c r="I11" s="817">
-        <f>'BUDGET NIRE 2+2'!$D$14*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$14*I8</f>
         <v/>
       </c>
       <c r="J11" s="816">
-        <f>'BUDGET CHAITEN 1'!$D$14*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$14*J8</f>
         <v/>
       </c>
       <c r="K11" s="816">
-        <f>'BUDGET CHAITEN 2'!$D$14*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$14*K8</f>
         <v/>
       </c>
       <c r="L11" s="817">
-        <f>'BUDGET CHAITEN 3'!$D$14*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$14*L8</f>
         <v/>
       </c>
       <c r="M11" s="816">
-        <f>'BUDGET CHAITEN 2+1'!$D$14*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$14*M8</f>
         <v/>
       </c>
       <c r="N11" s="817">
-        <f>'BUDGET CHAITEN 2+2'!$D$14*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$14*N8</f>
         <v/>
       </c>
       <c r="O11" s="816">
-        <f>'BUDGET CORCOVADO 1'!$D$14*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$14*O8</f>
         <v/>
       </c>
       <c r="P11" s="816">
-        <f>'BUDGET CORCOVADO 2'!$D$14*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$14*P8</f>
         <v/>
       </c>
       <c r="Q11" s="816">
-        <f>'BUDGET CORCOVADO 2+1'!$D$14*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$14*Q8</f>
         <v/>
       </c>
       <c r="R11" s="816">
-        <f>'BUDGET CORCOVADO 2+2'!$D$14*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$14*R8</f>
         <v/>
       </c>
       <c r="S11" s="816">
-        <f>'BUDGET CORCOVADO 2+3'!$D$14*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$14*S8</f>
         <v/>
       </c>
       <c r="T11" s="816">
-        <f>'BUDGET CORCOVADO 3'!$D$14*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$14*T8</f>
         <v/>
       </c>
       <c r="U11" s="816">
-        <f>'BUDGET CORCOVADO 3+1'!$D$14*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$14*U8</f>
         <v/>
       </c>
       <c r="V11" s="816">
-        <f>'BUDGET CORCOVADO 3+2'!$D$14*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$14*V8</f>
         <v/>
       </c>
       <c r="W11" s="816">
-        <f>'BUDGET CORCOVADO 4'!$D$14*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$14*W8</f>
         <v/>
       </c>
       <c r="X11" s="817">
-        <f>'BUDGET CORCOVADO 4+1'!$D$14*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$14*X8</f>
         <v/>
       </c>
       <c r="Y11" s="817">
-        <f>'BUDGET CORCOVADO 5'!$D$14*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$14*Y8</f>
         <v/>
       </c>
     </row>
@@ -58644,95 +58665,95 @@
         </is>
       </c>
       <c r="C12" s="818">
-        <f>'BUDGET COIGUE 1'!$D$15*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$15*C8</f>
         <v/>
       </c>
       <c r="D12" s="818">
-        <f>'BUDGET COIGUE 2'!$D$15*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$15*D8</f>
         <v/>
       </c>
       <c r="E12" s="818">
-        <f>'BUDGET COIGUE 2+1'!$D$15*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$15*E8</f>
         <v/>
       </c>
       <c r="F12" s="818">
-        <f>'BUDGET NIRE 1'!$D$15*F8</f>
+        <f>'BUDGET NIRE 1'!$B$15*F8</f>
         <v/>
       </c>
       <c r="G12" s="818">
-        <f>'BUDGET NIRE 2'!$D$15*G8</f>
+        <f>'BUDGET NIRE 2'!$B$15*G8</f>
         <v/>
       </c>
       <c r="H12" s="819">
-        <f>'BUDGET NIRE 2+1'!$D$15*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$15*H8</f>
         <v/>
       </c>
       <c r="I12" s="819">
-        <f>'BUDGET NIRE 2+2'!$D$15*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$15*I8</f>
         <v/>
       </c>
       <c r="J12" s="818">
-        <f>'BUDGET CHAITEN 1'!$D$15*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$15*J8</f>
         <v/>
       </c>
       <c r="K12" s="818">
-        <f>'BUDGET CHAITEN 2'!$D$15*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$15*K8</f>
         <v/>
       </c>
       <c r="L12" s="819">
-        <f>'BUDGET CHAITEN 3'!$D$15*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$15*L8</f>
         <v/>
       </c>
       <c r="M12" s="818">
-        <f>'BUDGET CHAITEN 2+1'!$D$15*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$15*M8</f>
         <v/>
       </c>
       <c r="N12" s="819">
-        <f>'BUDGET CHAITEN 2+2'!$D$15*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$15*N8</f>
         <v/>
       </c>
       <c r="O12" s="818">
-        <f>'BUDGET CORCOVADO 1'!$D$15*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$15*O8</f>
         <v/>
       </c>
       <c r="P12" s="818">
-        <f>'BUDGET CORCOVADO 2'!$D$15*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$15*P8</f>
         <v/>
       </c>
       <c r="Q12" s="818">
-        <f>'BUDGET CORCOVADO 2+1'!$D$15*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$15*Q8</f>
         <v/>
       </c>
       <c r="R12" s="818">
-        <f>'BUDGET CORCOVADO 2+2'!$D$15*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$15*R8</f>
         <v/>
       </c>
       <c r="S12" s="818">
-        <f>'BUDGET CORCOVADO 2+3'!$D$15*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$15*S8</f>
         <v/>
       </c>
       <c r="T12" s="818">
-        <f>'BUDGET CORCOVADO 3'!$D$15*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$15*T8</f>
         <v/>
       </c>
       <c r="U12" s="818">
-        <f>'BUDGET CORCOVADO 3+1'!$D$15*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$15*U8</f>
         <v/>
       </c>
       <c r="V12" s="818">
-        <f>'BUDGET CORCOVADO 3+2'!$D$15*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$15*V8</f>
         <v/>
       </c>
       <c r="W12" s="818">
-        <f>'BUDGET CORCOVADO 4'!$D$15*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$15*W8</f>
         <v/>
       </c>
       <c r="X12" s="819">
-        <f>'BUDGET CORCOVADO 4+1'!$D$15*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$15*X8</f>
         <v/>
       </c>
       <c r="Y12" s="819">
-        <f>'BUDGET CORCOVADO 5'!$D$15*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$15*Y8</f>
         <v/>
       </c>
     </row>
@@ -58743,95 +58764,95 @@
         </is>
       </c>
       <c r="C13" s="820">
-        <f>'BUDGET COIGUE 1'!$D$16*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$16*C8</f>
         <v/>
       </c>
       <c r="D13" s="820">
-        <f>'BUDGET COIGUE 2'!$D$16*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$16*D8</f>
         <v/>
       </c>
       <c r="E13" s="820">
-        <f>'BUDGET COIGUE 2+1'!$D$16*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$16*E8</f>
         <v/>
       </c>
       <c r="F13" s="820">
-        <f>'BUDGET NIRE 1'!$D$16*F8</f>
+        <f>'BUDGET NIRE 1'!$B$16*F8</f>
         <v/>
       </c>
       <c r="G13" s="820">
-        <f>'BUDGET NIRE 2'!$D$16*G8</f>
+        <f>'BUDGET NIRE 2'!$B$16*G8</f>
         <v/>
       </c>
       <c r="H13" s="821">
-        <f>'BUDGET NIRE 2+1'!$D$16*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$16*H8</f>
         <v/>
       </c>
       <c r="I13" s="821">
-        <f>'BUDGET NIRE 2+2'!$D$16*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$16*I8</f>
         <v/>
       </c>
       <c r="J13" s="820">
-        <f>'BUDGET CHAITEN 1'!$D$16*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$16*J8</f>
         <v/>
       </c>
       <c r="K13" s="820">
-        <f>'BUDGET CHAITEN 2'!$D$16*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$16*K8</f>
         <v/>
       </c>
       <c r="L13" s="821">
-        <f>'BUDGET CHAITEN 3'!$D$16*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$16*L8</f>
         <v/>
       </c>
       <c r="M13" s="820">
-        <f>'BUDGET CHAITEN 2+1'!$D$16*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$16*M8</f>
         <v/>
       </c>
       <c r="N13" s="821">
-        <f>'BUDGET CHAITEN 2+2'!$D$16*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$16*N8</f>
         <v/>
       </c>
       <c r="O13" s="820">
-        <f>'BUDGET CORCOVADO 1'!$D$16*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$16*O8</f>
         <v/>
       </c>
       <c r="P13" s="820">
-        <f>'BUDGET CORCOVADO 2'!$D$16*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$16*P8</f>
         <v/>
       </c>
       <c r="Q13" s="820">
-        <f>'BUDGET CORCOVADO 2+1'!$D$16*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$16*Q8</f>
         <v/>
       </c>
       <c r="R13" s="820">
-        <f>'BUDGET CORCOVADO 2+2'!$D$16*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$16*R8</f>
         <v/>
       </c>
       <c r="S13" s="820">
-        <f>'BUDGET CORCOVADO 2+3'!$D$16*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$16*S8</f>
         <v/>
       </c>
       <c r="T13" s="820">
-        <f>'BUDGET CORCOVADO 3'!$D$16*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$16*T8</f>
         <v/>
       </c>
       <c r="U13" s="820">
-        <f>'BUDGET CORCOVADO 3+1'!$D$16*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$16*U8</f>
         <v/>
       </c>
       <c r="V13" s="820">
-        <f>'BUDGET CORCOVADO 3+2'!$D$16*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$16*V8</f>
         <v/>
       </c>
       <c r="W13" s="820">
-        <f>'BUDGET CORCOVADO 4'!$D$16*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$16*W8</f>
         <v/>
       </c>
       <c r="X13" s="821">
-        <f>'BUDGET CORCOVADO 4+1'!$D$16*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$16*X8</f>
         <v/>
       </c>
       <c r="Y13" s="821">
-        <f>'BUDGET CORCOVADO 5'!$D$16*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$16*Y8</f>
         <v/>
       </c>
     </row>
@@ -58842,95 +58863,95 @@
         </is>
       </c>
       <c r="C14" s="822">
-        <f>'BUDGET COIGUE 1'!$D$17*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$17*C8</f>
         <v/>
       </c>
       <c r="D14" s="822">
-        <f>'BUDGET COIGUE 2'!$D$17*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$17*D8</f>
         <v/>
       </c>
       <c r="E14" s="822">
-        <f>'BUDGET COIGUE 2+1'!$D$17*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$17*E8</f>
         <v/>
       </c>
       <c r="F14" s="822">
-        <f>'BUDGET NIRE 1'!$D$17*F8</f>
+        <f>'BUDGET NIRE 1'!$B$17*F8</f>
         <v/>
       </c>
       <c r="G14" s="822">
-        <f>'BUDGET NIRE 2'!$D$17*G8</f>
+        <f>'BUDGET NIRE 2'!$B$17*G8</f>
         <v/>
       </c>
       <c r="H14" s="823">
-        <f>'BUDGET NIRE 2+1'!$D$17*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$17*H8</f>
         <v/>
       </c>
       <c r="I14" s="823">
-        <f>'BUDGET NIRE 2+2'!$D$17*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$17*I8</f>
         <v/>
       </c>
       <c r="J14" s="822">
-        <f>'BUDGET CHAITEN 1'!$D$17*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$17*J8</f>
         <v/>
       </c>
       <c r="K14" s="822">
-        <f>'BUDGET CHAITEN 2'!$D$17*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$17*K8</f>
         <v/>
       </c>
       <c r="L14" s="823">
-        <f>'BUDGET CHAITEN 3'!$D$17*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$17*L8</f>
         <v/>
       </c>
       <c r="M14" s="822">
-        <f>'BUDGET CHAITEN 2+1'!$D$17*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$17*M8</f>
         <v/>
       </c>
       <c r="N14" s="823">
-        <f>'BUDGET CHAITEN 2+2'!$D$17*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$17*N8</f>
         <v/>
       </c>
       <c r="O14" s="822">
-        <f>'BUDGET CORCOVADO 1'!$D$17*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$17*O8</f>
         <v/>
       </c>
       <c r="P14" s="822">
-        <f>'BUDGET CORCOVADO 2'!$D$17*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$17*P8</f>
         <v/>
       </c>
       <c r="Q14" s="822">
-        <f>'BUDGET CORCOVADO 2+1'!$D$17*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$17*Q8</f>
         <v/>
       </c>
       <c r="R14" s="822">
-        <f>'BUDGET CORCOVADO 2+2'!$D$17*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$17*R8</f>
         <v/>
       </c>
       <c r="S14" s="822">
-        <f>'BUDGET CORCOVADO 2+3'!$D$17*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$17*S8</f>
         <v/>
       </c>
       <c r="T14" s="822">
-        <f>'BUDGET CORCOVADO 3'!$D$17*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$17*T8</f>
         <v/>
       </c>
       <c r="U14" s="822">
-        <f>'BUDGET CORCOVADO 3+1'!$D$17*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$17*U8</f>
         <v/>
       </c>
       <c r="V14" s="822">
-        <f>'BUDGET CORCOVADO 3+2'!$D$17*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$17*V8</f>
         <v/>
       </c>
       <c r="W14" s="822">
-        <f>'BUDGET CORCOVADO 4'!$D$17*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$17*W8</f>
         <v/>
       </c>
       <c r="X14" s="823">
-        <f>'BUDGET CORCOVADO 4+1'!$D$17*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$17*X8</f>
         <v/>
       </c>
       <c r="Y14" s="823">
-        <f>'BUDGET CORCOVADO 5'!$D$17*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$17*Y8</f>
         <v/>
       </c>
     </row>
@@ -58941,95 +58962,95 @@
         </is>
       </c>
       <c r="C15" s="824">
-        <f>'BUDGET COIGUE 1'!$D$18*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$18*C8</f>
         <v/>
       </c>
       <c r="D15" s="824">
-        <f>'BUDGET COIGUE 2'!$D$18*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$18*D8</f>
         <v/>
       </c>
       <c r="E15" s="824">
-        <f>'BUDGET COIGUE 2+1'!$D$18*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$18*E8</f>
         <v/>
       </c>
       <c r="F15" s="824">
-        <f>'BUDGET NIRE 1'!$D$18*F8</f>
+        <f>'BUDGET NIRE 1'!$B$18*F8</f>
         <v/>
       </c>
       <c r="G15" s="824">
-        <f>'BUDGET NIRE 2'!$D$18*G8</f>
+        <f>'BUDGET NIRE 2'!$B$18*G8</f>
         <v/>
       </c>
       <c r="H15" s="825">
-        <f>'BUDGET NIRE 2+1'!$D$18*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$18*H8</f>
         <v/>
       </c>
       <c r="I15" s="825">
-        <f>'BUDGET NIRE 2+2'!$D$18*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$18*I8</f>
         <v/>
       </c>
       <c r="J15" s="824">
-        <f>'BUDGET CHAITEN 1'!$D$18*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$18*J8</f>
         <v/>
       </c>
       <c r="K15" s="824">
-        <f>'BUDGET CHAITEN 2'!$D$18*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$18*K8</f>
         <v/>
       </c>
       <c r="L15" s="825">
-        <f>'BUDGET CHAITEN 3'!$D$18*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$18*L8</f>
         <v/>
       </c>
       <c r="M15" s="824">
-        <f>'BUDGET CHAITEN 2+1'!$D$18*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$18*M8</f>
         <v/>
       </c>
       <c r="N15" s="825">
-        <f>'BUDGET CHAITEN 2+2'!$D$18*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$18*N8</f>
         <v/>
       </c>
       <c r="O15" s="824">
-        <f>'BUDGET CORCOVADO 1'!$D$18*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$18*O8</f>
         <v/>
       </c>
       <c r="P15" s="824">
-        <f>'BUDGET CORCOVADO 2'!$D$18*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$18*P8</f>
         <v/>
       </c>
       <c r="Q15" s="824">
-        <f>'BUDGET CORCOVADO 2+1'!$D$18*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$18*Q8</f>
         <v/>
       </c>
       <c r="R15" s="824">
-        <f>'BUDGET CORCOVADO 2+2'!$D$18*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$18*R8</f>
         <v/>
       </c>
       <c r="S15" s="824">
-        <f>'BUDGET CORCOVADO 2+3'!$D$18*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$18*S8</f>
         <v/>
       </c>
       <c r="T15" s="824">
-        <f>'BUDGET CORCOVADO 3'!$D$18*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$18*T8</f>
         <v/>
       </c>
       <c r="U15" s="824">
-        <f>'BUDGET CORCOVADO 3+1'!$D$18*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$18*U8</f>
         <v/>
       </c>
       <c r="V15" s="824">
-        <f>'BUDGET CORCOVADO 3+2'!$D$18*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$18*V8</f>
         <v/>
       </c>
       <c r="W15" s="824">
-        <f>'BUDGET CORCOVADO 4'!$D$18*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$18*W8</f>
         <v/>
       </c>
       <c r="X15" s="825">
-        <f>'BUDGET CORCOVADO 4+1'!$D$18*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$18*X8</f>
         <v/>
       </c>
       <c r="Y15" s="825">
-        <f>'BUDGET CORCOVADO 5'!$D$18*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$18*Y8</f>
         <v/>
       </c>
     </row>
@@ -59040,95 +59061,95 @@
         </is>
       </c>
       <c r="C16" s="826">
-        <f>'BUDGET COIGUE 1'!$D$19*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$19*C8</f>
         <v/>
       </c>
       <c r="D16" s="826">
-        <f>'BUDGET COIGUE 2'!$D$19*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$19*D8</f>
         <v/>
       </c>
       <c r="E16" s="826">
-        <f>'BUDGET COIGUE 2+1'!$D$19*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$19*E8</f>
         <v/>
       </c>
       <c r="F16" s="826">
-        <f>'BUDGET NIRE 1'!$D$19*F8</f>
+        <f>'BUDGET NIRE 1'!$B$19*F8</f>
         <v/>
       </c>
       <c r="G16" s="826">
-        <f>'BUDGET NIRE 2'!$D$19*G8</f>
+        <f>'BUDGET NIRE 2'!$B$19*G8</f>
         <v/>
       </c>
       <c r="H16" s="827">
-        <f>'BUDGET NIRE 2+1'!$D$19*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$19*H8</f>
         <v/>
       </c>
       <c r="I16" s="827">
-        <f>'BUDGET NIRE 2+2'!$D$19*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$19*I8</f>
         <v/>
       </c>
       <c r="J16" s="826">
-        <f>'BUDGET CHAITEN 1'!$D$19*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$19*J8</f>
         <v/>
       </c>
       <c r="K16" s="826">
-        <f>'BUDGET CHAITEN 2'!$D$19*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$19*K8</f>
         <v/>
       </c>
       <c r="L16" s="827">
-        <f>'BUDGET CHAITEN 3'!$D$19*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$19*L8</f>
         <v/>
       </c>
       <c r="M16" s="826">
-        <f>'BUDGET CHAITEN 2+1'!$D$19*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$19*M8</f>
         <v/>
       </c>
       <c r="N16" s="827">
-        <f>'BUDGET CHAITEN 2+2'!$D$19*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$19*N8</f>
         <v/>
       </c>
       <c r="O16" s="826">
-        <f>'BUDGET CORCOVADO 1'!$D$19*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$19*O8</f>
         <v/>
       </c>
       <c r="P16" s="826">
-        <f>'BUDGET CORCOVADO 2'!$D$19*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$19*P8</f>
         <v/>
       </c>
       <c r="Q16" s="826">
-        <f>'BUDGET CORCOVADO 2+1'!$D$19*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$19*Q8</f>
         <v/>
       </c>
       <c r="R16" s="826">
-        <f>'BUDGET CORCOVADO 2+2'!$D$19*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$19*R8</f>
         <v/>
       </c>
       <c r="S16" s="826">
-        <f>'BUDGET CORCOVADO 2+3'!$D$19*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$19*S8</f>
         <v/>
       </c>
       <c r="T16" s="826">
-        <f>'BUDGET CORCOVADO 3'!$D$19*T8</f>
+        <f>'BUDGET CORCOVADO 3'!$B$19*T8</f>
         <v/>
       </c>
       <c r="U16" s="826">
-        <f>'BUDGET CORCOVADO 3+1'!$D$19*U8</f>
+        <f>'BUDGET CORCOVADO 3+1'!$B$19*U8</f>
         <v/>
       </c>
       <c r="V16" s="826">
-        <f>'BUDGET CORCOVADO 3+2'!$D$19*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$19*V8</f>
         <v/>
       </c>
       <c r="W16" s="826">
-        <f>'BUDGET CORCOVADO 4'!$D$19*W8</f>
+        <f>'BUDGET CORCOVADO 4'!$B$19*W8</f>
         <v/>
       </c>
       <c r="X16" s="827">
-        <f>'BUDGET CORCOVADO 4+1'!$D$19*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$19*X8</f>
         <v/>
       </c>
       <c r="Y16" s="827">
-        <f>'BUDGET CORCOVADO 5'!$D$19*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$19*Y8</f>
         <v/>
       </c>
     </row>
@@ -59139,95 +59160,95 @@
         </is>
       </c>
       <c r="C17" s="828">
-        <f>'BUDGET COIGUE 1'!$D$20*C8</f>
+        <f>'BUDGET COIGUE 1'!$B$20*C8</f>
         <v/>
       </c>
       <c r="D17" s="828">
-        <f>'BUDGET COIGUE 2'!$D$20*D8</f>
+        <f>'BUDGET COIGUE 2'!$B$20*D8</f>
         <v/>
       </c>
       <c r="E17" s="828">
-        <f>'BUDGET COIGUE 2+1'!$D$20*E8</f>
+        <f>'BUDGET COIGUE 2+1'!$B$20*E8</f>
         <v/>
       </c>
       <c r="F17" s="828">
-        <f>'BUDGET NIRE 1'!$D$20*F8</f>
+        <f>'BUDGET NIRE 1'!$B$20*F8</f>
         <v/>
       </c>
       <c r="G17" s="828">
-        <f>'BUDGET NIRE 2'!$D$20*G8</f>
+        <f>'BUDGET NIRE 2'!$B$20*G8</f>
         <v/>
       </c>
       <c r="H17" s="829">
-        <f>'BUDGET NIRE 2+1'!$D$20*H8</f>
+        <f>'BUDGET NIRE 2+1'!$B$20*H8</f>
         <v/>
       </c>
       <c r="I17" s="829">
-        <f>'BUDGET NIRE 2+2'!$D$20*I8</f>
+        <f>'BUDGET NIRE 2+2'!$B$20*I8</f>
         <v/>
       </c>
       <c r="J17" s="828">
-        <f>'BUDGET CHAITEN 1'!$D$20*J8</f>
+        <f>'BUDGET CHAITEN 1'!$B$20*J8</f>
         <v/>
       </c>
       <c r="K17" s="828">
-        <f>'BUDGET CHAITEN 2'!$D$20*K8</f>
+        <f>'BUDGET CHAITEN 2'!$B$20*K8</f>
         <v/>
       </c>
       <c r="L17" s="829">
-        <f>'BUDGET CHAITEN 3'!$D$20*L8</f>
+        <f>'BUDGET CHAITEN 3'!$B$20*L8</f>
         <v/>
       </c>
       <c r="M17" s="828">
-        <f>'BUDGET CHAITEN 2+1'!$D$20*M8</f>
+        <f>'BUDGET CHAITEN 2+1'!$B$20*M8</f>
         <v/>
       </c>
       <c r="N17" s="829">
-        <f>'BUDGET CHAITEN 2+2'!$D$20*N8</f>
+        <f>'BUDGET CHAITEN 2+2'!$B$20*N8</f>
         <v/>
       </c>
       <c r="O17" s="828">
-        <f>'BUDGET CORCOVADO 1'!$D$20*O8</f>
+        <f>'BUDGET CORCOVADO 1'!$B$20*O8</f>
         <v/>
       </c>
       <c r="P17" s="828">
-        <f>'BUDGET CORCOVADO 2'!$D$20*P8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$20*P8</f>
         <v/>
       </c>
       <c r="Q17" s="828">
-        <f>'BUDGET CORCOVADO 2+1'!$D$20*Q8</f>
+        <f>'BUDGET CORCOVADO 2+1'!$B$20*Q8</f>
         <v/>
       </c>
       <c r="R17" s="828">
-        <f>'BUDGET CORCOVADO 2+2'!$D$20*R8</f>
+        <f>'BUDGET CORCOVADO 2+2'!$B$20*R8</f>
         <v/>
       </c>
       <c r="S17" s="828">
-        <f>'BUDGET CORCOVADO 2+3'!$D$20*S8</f>
+        <f>'BUDGET CORCOVADO 2+3'!$B$20*S8</f>
         <v/>
       </c>
       <c r="T17" s="828">
-        <f>'BUDGET CORCOVADO 2'!$D$20*T8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$20*T8</f>
         <v/>
       </c>
       <c r="U17" s="828">
-        <f>'BUDGET CORCOVADO 2'!$D$20*U8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$20*U8</f>
         <v/>
       </c>
       <c r="V17" s="828">
-        <f>'BUDGET CORCOVADO 3+2'!$D$20*V8</f>
+        <f>'BUDGET CORCOVADO 3+2'!$B$20*V8</f>
         <v/>
       </c>
       <c r="W17" s="828">
-        <f>'BUDGET CORCOVADO 2'!$D$20*W8</f>
+        <f>'BUDGET CORCOVADO 2'!$B$20*W8</f>
         <v/>
       </c>
       <c r="X17" s="829">
-        <f>'BUDGET CORCOVADO 4+1'!$D$20*X8</f>
+        <f>'BUDGET CORCOVADO 4+1'!$B$20*X8</f>
         <v/>
       </c>
       <c r="Y17" s="829">
-        <f>'BUDGET CORCOVADO 5'!$D$20*Y8</f>
+        <f>'BUDGET CORCOVADO 5'!$B$20*Y8</f>
         <v/>
       </c>
     </row>
@@ -59260,7 +59281,7 @@
     <row r="19" ht="40" customFormat="1" customHeight="1" s="526" thickBot="1">
       <c r="B19" s="524" t="inlineStr">
         <is>
-          <t>SUBTOTAL SEM AGÊNCIA [CC]</t>
+          <t>SUBTOTAL SEM CC</t>
         </is>
       </c>
       <c r="C19" s="832">
@@ -59359,198 +59380,198 @@
     <row r="20" ht="29" customFormat="1" customHeight="1" s="526" thickBot="1">
       <c r="B20" s="527" t="inlineStr">
         <is>
-          <t>desconto 5%</t>
+          <t>Taxa CC</t>
         </is>
       </c>
       <c r="C20" s="834">
-        <f>C19*0.05</f>
+        <f>C19*$C$24</f>
         <v/>
       </c>
       <c r="D20" s="834">
-        <f>D19*0.05</f>
+        <f>D19*$C$24</f>
         <v/>
       </c>
       <c r="E20" s="835">
-        <f>E19*0.05</f>
+        <f>E19*$C$24</f>
         <v/>
       </c>
       <c r="F20" s="834">
-        <f>F19*0.05</f>
+        <f>F19*$C$24</f>
         <v/>
       </c>
       <c r="G20" s="834">
-        <f>G19*0.05</f>
+        <f>G19*$C$24</f>
         <v/>
       </c>
       <c r="H20" s="835">
-        <f>H19*0.05</f>
+        <f>H19*$C$24</f>
         <v/>
       </c>
       <c r="I20" s="835">
-        <f>I19*0.05</f>
+        <f>I19*$C$24</f>
         <v/>
       </c>
       <c r="J20" s="834">
-        <f>J19*0.05</f>
+        <f>J19*$C$24</f>
         <v/>
       </c>
       <c r="K20" s="834">
-        <f>K19*0.05</f>
+        <f>K19*$C$24</f>
         <v/>
       </c>
       <c r="L20" s="835">
-        <f>L19*0.05</f>
+        <f>L19*$C$24</f>
         <v/>
       </c>
       <c r="M20" s="834">
-        <f>M19*0.05</f>
+        <f>M19*$C$24</f>
         <v/>
       </c>
       <c r="N20" s="835">
-        <f>N19*0.05</f>
+        <f>N19*$C$24</f>
         <v/>
       </c>
       <c r="O20" s="834">
-        <f>O19*0.05</f>
+        <f>O19*$C$24</f>
         <v/>
       </c>
       <c r="P20" s="834">
-        <f>P19*0.05</f>
+        <f>P19*$C$24</f>
         <v/>
       </c>
       <c r="Q20" s="834">
-        <f>Q19*0.05</f>
+        <f>Q19*$C$24</f>
         <v/>
       </c>
       <c r="R20" s="834">
-        <f>R19*0.05</f>
+        <f>R19*$C$24</f>
         <v/>
       </c>
       <c r="S20" s="834">
-        <f>S19*0.05</f>
+        <f>S19*$C$24</f>
         <v/>
       </c>
       <c r="T20" s="834">
-        <f>T19*0.05</f>
+        <f>T19*$C$24</f>
         <v/>
       </c>
       <c r="U20" s="834">
-        <f>U19*0.05</f>
+        <f>U19*$C$24</f>
         <v/>
       </c>
       <c r="V20" s="834">
-        <f>V19*0.05</f>
+        <f>V19*$C$24</f>
         <v/>
       </c>
       <c r="W20" s="834">
-        <f>W19*0.05</f>
+        <f>W19*$C$24</f>
         <v/>
       </c>
       <c r="X20" s="835">
-        <f>X19*0.05</f>
+        <f>X19*$C$24</f>
         <v/>
       </c>
       <c r="Y20" s="835">
-        <f>Y19*0.05</f>
+        <f>Y19*$C$24</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="40" customFormat="1" customHeight="1" s="526" thickBot="1">
       <c r="B21" s="530" t="inlineStr">
         <is>
-          <t>SUBTOTAL  [no cash]</t>
+          <t>SUBTOTAL COM CC</t>
         </is>
       </c>
       <c r="C21" s="836">
-        <f>C19-C20</f>
+        <f>C19+C20</f>
         <v/>
       </c>
       <c r="D21" s="836">
-        <f>D19-D20</f>
+        <f>D19+D20</f>
         <v/>
       </c>
       <c r="E21" s="837">
-        <f>E19-E20</f>
+        <f>E19+E20</f>
         <v/>
       </c>
       <c r="F21" s="836">
-        <f>F19-F20</f>
+        <f>F19+F20</f>
         <v/>
       </c>
       <c r="G21" s="836">
-        <f>G19-G20</f>
+        <f>G19+G20</f>
         <v/>
       </c>
       <c r="H21" s="837">
-        <f>H19-H20</f>
+        <f>H19+H20</f>
         <v/>
       </c>
       <c r="I21" s="837">
-        <f>I19-I20</f>
+        <f>I19+I20</f>
         <v/>
       </c>
       <c r="J21" s="836">
-        <f>J19-J20</f>
+        <f>J19+J20</f>
         <v/>
       </c>
       <c r="K21" s="836">
-        <f>K19-K20</f>
+        <f>K19+K20</f>
         <v/>
       </c>
       <c r="L21" s="837">
-        <f>L19-L20</f>
+        <f>L19+L20</f>
         <v/>
       </c>
       <c r="M21" s="836">
-        <f>M19-M20</f>
+        <f>M19+M20</f>
         <v/>
       </c>
       <c r="N21" s="837">
-        <f>N19-N20</f>
+        <f>N19+N20</f>
         <v/>
       </c>
       <c r="O21" s="836">
-        <f>O19-O20</f>
+        <f>O19+O20</f>
         <v/>
       </c>
       <c r="P21" s="836">
-        <f>P19-P20</f>
+        <f>P19+P20</f>
         <v/>
       </c>
       <c r="Q21" s="836">
-        <f>Q19-Q20</f>
+        <f>Q19+Q20</f>
         <v/>
       </c>
       <c r="R21" s="836">
-        <f>R19-R20</f>
+        <f>R19+R20</f>
         <v/>
       </c>
       <c r="S21" s="836">
-        <f>S19-S20</f>
+        <f>S19+S20</f>
         <v/>
       </c>
       <c r="T21" s="836">
-        <f>T19-T20</f>
+        <f>T19+T20</f>
         <v/>
       </c>
       <c r="U21" s="836">
-        <f>U19-U20</f>
+        <f>U19+U20</f>
         <v/>
       </c>
       <c r="V21" s="836">
-        <f>V19-V20</f>
+        <f>V19+V20</f>
         <v/>
       </c>
       <c r="W21" s="836">
-        <f>W19-W20</f>
+        <f>W19+W20</f>
         <v/>
       </c>
       <c r="X21" s="837">
-        <f>X19-X20</f>
+        <f>X19+X20</f>
         <v/>
       </c>
       <c r="Y21" s="837">
-        <f>Y19-Y20</f>
+        <f>Y19+Y20</f>
         <v/>
       </c>
     </row>
@@ -59586,7 +59607,7 @@
           <t>taxa agência</t>
         </is>
       </c>
-      <c r="C23" s="840">
+      <c r="C23" s="1063">
         <f>'[1]⚙️ INPUTS'!$B$34</f>
         <v/>
       </c>
@@ -59619,7 +59640,7 @@
           <t>taxa SUMUP</t>
         </is>
       </c>
-      <c r="C24" s="840">
+      <c r="C24" s="1063">
         <f>'[1]⚙️ INPUTS'!$B$33</f>
         <v/>
       </c>
@@ -59649,99 +59670,99 @@
     <row r="25" ht="48" customFormat="1" customHeight="1" s="489">
       <c r="B25" s="540" t="inlineStr">
         <is>
-          <t>SUBTOTAL COM TAXA DE AG [pago em cash]</t>
+          <t>SUBTOTAL COM TAXA AG E PAGO CASH</t>
         </is>
       </c>
       <c r="C25" s="841">
-        <f>C21+(C21*$C$23)</f>
+        <f>C19+(C19*$C$23)</f>
         <v/>
       </c>
       <c r="D25" s="841">
-        <f>D21+(D21*$C$23)</f>
+        <f>D19+(D19*$C$23)</f>
         <v/>
       </c>
       <c r="E25" s="842">
-        <f>E21+(E21*$C$23)</f>
+        <f>E19+(E19*$C$23)</f>
         <v/>
       </c>
       <c r="F25" s="841">
-        <f>F21+(F21*$C$23)</f>
+        <f>F19+(F19*$C$23)</f>
         <v/>
       </c>
       <c r="G25" s="841">
-        <f>G21+(G21*$C$23)</f>
+        <f>G19+(G19*$C$23)</f>
         <v/>
       </c>
       <c r="H25" s="842">
-        <f>H21+(H21*$C$23)</f>
+        <f>H19+(H19*$C$23)</f>
         <v/>
       </c>
       <c r="I25" s="842">
-        <f>I21+(I21*$C$23)</f>
+        <f>I19+(I19*$C$23)</f>
         <v/>
       </c>
       <c r="J25" s="841">
-        <f>J21+(J21*$C$23)</f>
+        <f>J19+(J19*$C$23)</f>
         <v/>
       </c>
       <c r="K25" s="841">
-        <f>K21+(K21*$C$23)</f>
+        <f>K19+(K19*$C$23)</f>
         <v/>
       </c>
       <c r="L25" s="842">
-        <f>L21+(L21*$C$23)</f>
+        <f>L19+(L19*$C$23)</f>
         <v/>
       </c>
       <c r="M25" s="841">
-        <f>M21+(M21*$C$23)</f>
+        <f>M19+(M19*$C$23)</f>
         <v/>
       </c>
       <c r="N25" s="842">
-        <f>N21+(N21*$C$23)</f>
+        <f>N19+(N19*$C$23)</f>
         <v/>
       </c>
       <c r="O25" s="841">
-        <f>O21+(O21*$C$23)</f>
+        <f>O19+(O19*$C$23)</f>
         <v/>
       </c>
       <c r="P25" s="841">
-        <f>P21+(P21*$C$23)</f>
+        <f>P19+(P19*$C$23)</f>
         <v/>
       </c>
       <c r="Q25" s="841">
-        <f>Q21+(Q21*$C$23)</f>
+        <f>Q19+(Q19*$C$23)</f>
         <v/>
       </c>
       <c r="R25" s="841">
-        <f>R21+(R21*$C$23)</f>
+        <f>R19+(R19*$C$23)</f>
         <v/>
       </c>
       <c r="S25" s="841">
-        <f>S21+(S21*$C$23)</f>
+        <f>S19+(S19*$C$23)</f>
         <v/>
       </c>
       <c r="T25" s="841">
-        <f>T21+(T21*$C$23)</f>
+        <f>T19+(T19*$C$23)</f>
         <v/>
       </c>
       <c r="U25" s="841">
-        <f>U21+(U21*$C$23)</f>
+        <f>U19+(U19*$C$23)</f>
         <v/>
       </c>
       <c r="V25" s="841">
-        <f>V21+(V21*$C$23)</f>
+        <f>V19+(V19*$C$23)</f>
         <v/>
       </c>
       <c r="W25" s="841">
-        <f>W21+(W21*$C$23)</f>
+        <f>W19+(W19*$C$23)</f>
         <v/>
       </c>
       <c r="X25" s="842">
-        <f>X21+(X21*$C$23)</f>
+        <f>X19+(X19*$C$23)</f>
         <v/>
       </c>
       <c r="Y25" s="842">
-        <f>Y21+(Y21*$C$23)</f>
+        <f>Y19+(Y19*$C$23)</f>
         <v/>
       </c>
     </row>
@@ -59851,95 +59872,95 @@
         </is>
       </c>
       <c r="C27" s="845">
-        <f>C26-C19</f>
+        <f>C25-C19</f>
         <v/>
       </c>
       <c r="D27" s="845">
-        <f>D26-D19</f>
+        <f>D25-D19</f>
         <v/>
       </c>
       <c r="E27" s="846">
-        <f>E26-E19</f>
+        <f>E25-E19</f>
         <v/>
       </c>
       <c r="F27" s="845">
-        <f>F26-F19</f>
+        <f>F25-F19</f>
         <v/>
       </c>
       <c r="G27" s="845">
-        <f>G26-G19</f>
+        <f>G25-G19</f>
         <v/>
       </c>
       <c r="H27" s="846">
-        <f>H26-H19</f>
+        <f>H25-H19</f>
         <v/>
       </c>
       <c r="I27" s="846">
-        <f>I26-I19</f>
+        <f>I25-I19</f>
         <v/>
       </c>
       <c r="J27" s="845">
-        <f>J26-J19</f>
+        <f>J25-J19</f>
         <v/>
       </c>
       <c r="K27" s="845">
-        <f>K26-K19</f>
+        <f>K25-K19</f>
         <v/>
       </c>
       <c r="L27" s="846">
-        <f>L26-L19</f>
+        <f>L25-L19</f>
         <v/>
       </c>
       <c r="M27" s="845">
-        <f>M26-M19</f>
+        <f>M25-M19</f>
         <v/>
       </c>
       <c r="N27" s="846">
-        <f>N26-N19</f>
+        <f>N25-N19</f>
         <v/>
       </c>
       <c r="O27" s="845">
-        <f>O26-O19</f>
+        <f>O25-O19</f>
         <v/>
       </c>
       <c r="P27" s="845">
-        <f>P26-P19</f>
+        <f>P25-P19</f>
         <v/>
       </c>
       <c r="Q27" s="845">
-        <f>Q26-Q19</f>
+        <f>Q25-Q19</f>
         <v/>
       </c>
       <c r="R27" s="845">
-        <f>R26-R19</f>
+        <f>R25-R19</f>
         <v/>
       </c>
       <c r="S27" s="845">
-        <f>S26-S19</f>
+        <f>S25-S19</f>
         <v/>
       </c>
       <c r="T27" s="845">
-        <f>T26-T19</f>
+        <f>T25-T19</f>
         <v/>
       </c>
       <c r="U27" s="845">
-        <f>U26-U19</f>
+        <f>U25-U19</f>
         <v/>
       </c>
       <c r="V27" s="845">
-        <f>V26-V19</f>
+        <f>V25-V19</f>
         <v/>
       </c>
       <c r="W27" s="845">
-        <f>W26-W19</f>
+        <f>W25-W19</f>
         <v/>
       </c>
       <c r="X27" s="846">
-        <f>X26-X19</f>
+        <f>X25-X19</f>
         <v/>
       </c>
       <c r="Y27" s="846">
-        <f>Y26-Y19</f>
+        <f>Y25-Y19</f>
         <v/>
       </c>
     </row>
@@ -61509,7 +61530,7 @@
       <c r="C27" s="673" t="n"/>
       <c r="D27" s="696" t="n"/>
       <c r="E27" s="878">
-        <f>E26-(E26*0.05)</f>
+        <f>E26</f>
         <v/>
       </c>
     </row>
@@ -61522,7 +61543,7 @@
       <c r="C28" s="673" t="n"/>
       <c r="D28" s="696" t="n"/>
       <c r="E28" s="878">
-        <f>E27*(1+'BUDGET RESUMO'!$C$23)</f>
+        <f>E27*(1+'BUDGET RESUMO'!$C$24)</f>
         <v/>
       </c>
     </row>
@@ -61546,7 +61567,7 @@
       <c r="C31" s="673" t="n"/>
       <c r="D31" s="696" t="n"/>
       <c r="E31" s="861">
-        <f>E28*(1+'BUDGET RESUMO'!$C$24)</f>
+        <f>E27*(1+'BUDGET RESUMO'!$C$23)*(1+'BUDGET RESUMO'!$C$24)</f>
         <v/>
       </c>
       <c r="F31" s="634">
@@ -62043,8 +62064,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -64820,8 +64842,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -67596,8 +67619,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -70378,8 +70402,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>
@@ -73161,8 +73186,9 @@
       <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="32" customFormat="1" customHeight="1" s="659">
-      <c r="C12" s="58" t="n">
-        <v>0.05</v>
+      <c r="C12" s="58">
+        <f>'[1]⚙️ INPUTS'!$B$33</f>
+        <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="665" t="n"/>

</xml_diff>